<commit_message>
Add first version of 3D model
</commit_message>
<xml_diff>
--- a/setup.xlsx
+++ b/setup.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cmarinriver\Projects\ConfinedLab\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2F86C74-0976-402F-9CFD-ED91783869A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75F3F5C0-3490-43C3-8877-8A4444AB859E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15796" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="555" uniqueCount="330">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="589" uniqueCount="339">
   <si>
     <t>nlay</t>
   </si>
@@ -1012,9 +1012,6 @@
     <t>14k - 11k BP</t>
   </si>
   <si>
-    <t>11kBP - present - 39kAP</t>
-  </si>
-  <si>
     <t>Transient recharge step change experiment</t>
   </si>
   <si>
@@ -1034,13 +1031,43 @@
   </si>
   <si>
     <t>One thousand years</t>
+  </si>
+  <si>
+    <t>UncAq</t>
+  </si>
+  <si>
+    <t>Aqt 1</t>
+  </si>
+  <si>
+    <t>Caq 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aqt 2 </t>
+  </si>
+  <si>
+    <t>Caq 2</t>
+  </si>
+  <si>
+    <t>Caq 1 outcrop</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HEAD </t>
+  </si>
+  <si>
+    <t>WELL_07</t>
+  </si>
+  <si>
+    <t>WELL_08</t>
+  </si>
+  <si>
+    <t>WELL_09</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1057,13 +1084,6 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <b/>
@@ -1154,11 +1174,11 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="11" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1504,19 +1524,19 @@
         <v>5</v>
       </c>
       <c r="B2">
-        <v>1</v>
+        <v>4500</v>
       </c>
       <c r="C2">
-        <v>600</v>
+        <v>450</v>
       </c>
       <c r="D2">
-        <v>1</v>
+        <v>450000</v>
       </c>
       <c r="E2">
-        <v>600000</v>
+        <v>450000</v>
       </c>
       <c r="F2">
-        <v>1</v>
+        <v>1000</v>
       </c>
       <c r="G2">
         <v>1000</v>
@@ -2959,7 +2979,7 @@
         <v>36000</v>
       </c>
       <c r="K18" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="R18" t="s">
         <v>123</v>
@@ -3081,20 +3101,23 @@
       <c r="I20">
         <v>36000</v>
       </c>
-      <c r="K20" t="s">
-        <v>24</v>
-      </c>
-      <c r="L20" t="s">
-        <v>25</v>
-      </c>
-      <c r="M20" t="s">
-        <v>26</v>
-      </c>
-      <c r="N20" t="s">
-        <v>27</v>
-      </c>
-      <c r="O20" t="s">
-        <v>28</v>
+      <c r="K20" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="L20" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="M20" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="N20" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="O20" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="P20" s="6" t="s">
+        <v>36</v>
       </c>
       <c r="U20">
         <v>1968</v>
@@ -3150,20 +3173,23 @@
       <c r="I21">
         <v>36000</v>
       </c>
-      <c r="K21">
+      <c r="K21" s="6">
         <v>0</v>
       </c>
-      <c r="L21">
-        <v>0</v>
-      </c>
-      <c r="M21">
-        <v>1</v>
-      </c>
-      <c r="N21">
-        <v>1</v>
-      </c>
-      <c r="O21" t="s">
-        <v>29</v>
+      <c r="L21" s="1">
+        <v>3.0000000000000003E-4</v>
+      </c>
+      <c r="M21" s="1">
+        <v>3.0000000000000001E-6</v>
+      </c>
+      <c r="N21" s="1">
+        <v>2.9999999999999997E-4</v>
+      </c>
+      <c r="O21" s="1">
+        <v>3.0000000000000001E-6</v>
+      </c>
+      <c r="P21" s="1">
+        <v>2.9999999999999997E-4</v>
       </c>
       <c r="U21">
         <v>1969</v>
@@ -3219,20 +3245,23 @@
       <c r="I22">
         <v>36000</v>
       </c>
-      <c r="K22">
-        <v>1</v>
-      </c>
-      <c r="L22">
-        <v>2520000</v>
-      </c>
-      <c r="M22">
-        <v>10</v>
-      </c>
-      <c r="N22">
-        <v>1</v>
-      </c>
-      <c r="O22" t="s">
-        <v>320</v>
+      <c r="K22" s="6">
+        <v>3600000</v>
+      </c>
+      <c r="L22" s="1">
+        <v>1.5E-5</v>
+      </c>
+      <c r="M22" s="1">
+        <v>1.4999999999999999E-7</v>
+      </c>
+      <c r="N22" s="1">
+        <v>1.4999999999999999E-5</v>
+      </c>
+      <c r="O22" s="1">
+        <v>1.4999999999999999E-7</v>
+      </c>
+      <c r="P22" s="1">
+        <v>1.4999999999999999E-5</v>
       </c>
       <c r="U22">
         <v>1970</v>
@@ -3288,20 +3317,23 @@
       <c r="I23">
         <v>36000</v>
       </c>
-      <c r="K23">
-        <v>2</v>
-      </c>
-      <c r="L23">
-        <v>1080000</v>
-      </c>
-      <c r="M23">
-        <v>20</v>
-      </c>
-      <c r="N23">
-        <v>1</v>
-      </c>
-      <c r="O23" t="s">
-        <v>321</v>
+      <c r="K23" s="6">
+        <v>400000000</v>
+      </c>
+      <c r="L23" s="1">
+        <v>1.4999999999999999E-5</v>
+      </c>
+      <c r="M23" s="1">
+        <v>1.4999999999999999E-7</v>
+      </c>
+      <c r="N23" s="1">
+        <v>1.4999999999999999E-5</v>
+      </c>
+      <c r="O23" s="1">
+        <v>1.4999999999999999E-7</v>
+      </c>
+      <c r="P23" s="1">
+        <v>1.4999999999999999E-5</v>
       </c>
       <c r="U23">
         <v>1971</v>
@@ -3357,21 +3389,6 @@
       <c r="I24">
         <v>36000</v>
       </c>
-      <c r="K24">
-        <v>3</v>
-      </c>
-      <c r="L24">
-        <v>18000000</v>
-      </c>
-      <c r="M24">
-        <v>1000</v>
-      </c>
-      <c r="N24">
-        <v>1</v>
-      </c>
-      <c r="O24" t="s">
-        <v>322</v>
-      </c>
       <c r="U24">
         <v>1972</v>
       </c>
@@ -3426,6 +3443,21 @@
       <c r="I25">
         <v>36000</v>
       </c>
+      <c r="K25" t="s">
+        <v>24</v>
+      </c>
+      <c r="L25" t="s">
+        <v>25</v>
+      </c>
+      <c r="M25" t="s">
+        <v>26</v>
+      </c>
+      <c r="N25" t="s">
+        <v>27</v>
+      </c>
+      <c r="O25" t="s">
+        <v>28</v>
+      </c>
       <c r="U25">
         <v>1973</v>
       </c>
@@ -3480,23 +3512,20 @@
       <c r="I26">
         <v>36000</v>
       </c>
-      <c r="K26" t="s">
-        <v>31</v>
-      </c>
-      <c r="L26" t="s">
-        <v>32</v>
-      </c>
-      <c r="M26" t="s">
-        <v>33</v>
-      </c>
-      <c r="N26" t="s">
-        <v>34</v>
+      <c r="K26">
+        <v>0</v>
+      </c>
+      <c r="L26">
+        <v>0</v>
+      </c>
+      <c r="M26">
+        <v>1</v>
+      </c>
+      <c r="N26">
+        <v>1</v>
       </c>
       <c r="O26" t="s">
-        <v>35</v>
-      </c>
-      <c r="P26" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="U26">
         <v>1974</v>
@@ -3553,22 +3582,19 @@
         <v>36000</v>
       </c>
       <c r="K27">
-        <v>0</v>
-      </c>
-      <c r="L27" s="1">
-        <v>1.1999999999999999E-3</v>
-      </c>
-      <c r="M27" s="1">
-        <v>1.9999999999999999E-6</v>
-      </c>
-      <c r="N27" s="1">
-        <v>1.1999999999999999E-3</v>
-      </c>
-      <c r="O27" s="1">
-        <v>1.9999999999999999E-6</v>
-      </c>
-      <c r="P27" s="1">
-        <v>1.1999999999999999E-3</v>
+        <v>1</v>
+      </c>
+      <c r="L27">
+        <v>2520000</v>
+      </c>
+      <c r="M27">
+        <v>100</v>
+      </c>
+      <c r="N27">
+        <v>1</v>
+      </c>
+      <c r="O27" t="s">
+        <v>320</v>
       </c>
       <c r="U27">
         <v>1975</v>
@@ -3625,22 +3651,19 @@
         <v>36000</v>
       </c>
       <c r="K28">
-        <v>2520000</v>
-      </c>
-      <c r="L28" s="1">
-        <v>1.1999999999999999E-3</v>
-      </c>
-      <c r="M28" s="1">
-        <v>1.9999999999999999E-6</v>
-      </c>
-      <c r="N28" s="1">
-        <v>1.1999999999999999E-3</v>
-      </c>
-      <c r="O28" s="1">
-        <v>1.9999999999999999E-6</v>
-      </c>
-      <c r="P28" s="1">
-        <v>1.1999999999999999E-3</v>
+        <v>2</v>
+      </c>
+      <c r="L28">
+        <v>1080000</v>
+      </c>
+      <c r="M28">
+        <v>200</v>
+      </c>
+      <c r="N28">
+        <v>1</v>
+      </c>
+      <c r="O28" t="s">
+        <v>321</v>
       </c>
       <c r="U28">
         <v>1976</v>
@@ -3697,22 +3720,19 @@
         <v>36000</v>
       </c>
       <c r="K29">
-        <v>3600000</v>
-      </c>
-      <c r="L29" s="1">
-        <v>2.9999999999999997E-4</v>
-      </c>
-      <c r="M29" s="1">
-        <v>4.9999999999999998E-7</v>
-      </c>
-      <c r="N29" s="1">
-        <v>2.9999999999999997E-4</v>
-      </c>
-      <c r="O29" s="1">
-        <v>4.9999999999999998E-7</v>
-      </c>
-      <c r="P29" s="1">
-        <v>2.9999999999999997E-4</v>
+        <v>3</v>
+      </c>
+      <c r="L29">
+        <v>180000</v>
+      </c>
+      <c r="M29">
+        <v>500</v>
+      </c>
+      <c r="N29">
+        <v>1</v>
+      </c>
+      <c r="O29" t="s">
+        <v>323</v>
       </c>
       <c r="U29">
         <v>1977</v>
@@ -3769,22 +3789,19 @@
         <v>36000</v>
       </c>
       <c r="K30">
-        <v>30000000</v>
-      </c>
-      <c r="L30" s="6">
-        <v>2.9999999999999997E-4</v>
-      </c>
-      <c r="M30" s="6">
-        <v>4.9999999999999998E-7</v>
-      </c>
-      <c r="N30" s="6">
-        <v>2.9999999999999997E-4</v>
-      </c>
-      <c r="O30" s="6">
-        <v>4.9999999999999998E-7</v>
-      </c>
-      <c r="P30" s="6">
-        <v>2.9999999999999997E-4</v>
+        <v>4</v>
+      </c>
+      <c r="L30">
+        <v>17820000</v>
+      </c>
+      <c r="M30">
+        <v>495</v>
+      </c>
+      <c r="N30">
+        <v>1</v>
+      </c>
+      <c r="O30" t="s">
+        <v>324</v>
       </c>
       <c r="U30">
         <v>1978</v>
@@ -3840,6 +3857,21 @@
       <c r="I31">
         <v>36000</v>
       </c>
+      <c r="K31">
+        <v>5</v>
+      </c>
+      <c r="L31">
+        <v>360000000</v>
+      </c>
+      <c r="M31">
+        <v>100</v>
+      </c>
+      <c r="N31">
+        <v>1</v>
+      </c>
+      <c r="O31" t="s">
+        <v>328</v>
+      </c>
       <c r="U31">
         <v>1979</v>
       </c>
@@ -3894,12 +3926,6 @@
       <c r="I32">
         <v>36000</v>
       </c>
-      <c r="K32" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="L32" s="6">
-        <v>2.9999999999999997E-4</v>
-      </c>
       <c r="U32">
         <v>1980</v>
       </c>
@@ -3954,12 +3980,6 @@
       <c r="I33">
         <v>36000</v>
       </c>
-      <c r="K33" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="L33" s="6">
-        <v>4.9999999999999998E-7</v>
-      </c>
       <c r="U33">
         <v>1981</v>
       </c>
@@ -4014,12 +4034,6 @@
       <c r="I34">
         <v>36000</v>
       </c>
-      <c r="K34" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="L34" s="6">
-        <v>2.9999999999999997E-4</v>
-      </c>
       <c r="U34">
         <v>1982</v>
       </c>
@@ -4074,12 +4088,6 @@
       <c r="I35">
         <v>36000</v>
       </c>
-      <c r="K35" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="L35" s="6">
-        <v>4.9999999999999998E-7</v>
-      </c>
       <c r="U35">
         <v>1983</v>
       </c>
@@ -4133,12 +4141,6 @@
       </c>
       <c r="I36">
         <v>36000</v>
-      </c>
-      <c r="K36" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="L36" s="6">
-        <v>2.9999999999999997E-4</v>
       </c>
       <c r="U36">
         <v>1984</v>
@@ -16662,7 +16664,7 @@
         <v>13</v>
       </c>
       <c r="H1" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.45">
@@ -16684,8 +16686,8 @@
       <c r="F2">
         <v>300</v>
       </c>
-      <c r="G2">
-        <v>300</v>
+      <c r="G2" s="8">
+        <v>225</v>
       </c>
       <c r="H2">
         <v>5</v>
@@ -16710,8 +16712,8 @@
       <c r="F3">
         <v>150</v>
       </c>
-      <c r="G3">
-        <v>250</v>
+      <c r="G3" s="8">
+        <v>187.5</v>
       </c>
       <c r="H3">
         <v>5</v>
@@ -16736,8 +16738,8 @@
       <c r="F4">
         <v>200</v>
       </c>
-      <c r="G4">
-        <v>150</v>
+      <c r="G4" s="8">
+        <v>112.5</v>
       </c>
       <c r="H4">
         <v>5</v>
@@ -16762,8 +16764,8 @@
       <c r="F5">
         <v>150</v>
       </c>
-      <c r="G5">
-        <v>100</v>
+      <c r="G5" s="8">
+        <v>75</v>
       </c>
       <c r="H5">
         <v>5</v>
@@ -16788,7 +16790,7 @@
       <c r="F6">
         <v>200</v>
       </c>
-      <c r="G6">
+      <c r="G6" s="8">
         <v>0</v>
       </c>
       <c r="H6">
@@ -16850,7 +16852,7 @@
         <v>2520000</v>
       </c>
       <c r="C3">
-        <v>10</v>
+        <v>100</v>
       </c>
       <c r="D3">
         <v>1</v>
@@ -16867,7 +16869,7 @@
         <v>1080000</v>
       </c>
       <c r="C4">
-        <v>20</v>
+        <v>200</v>
       </c>
       <c r="D4">
         <v>1</v>
@@ -16890,7 +16892,7 @@
         <v>1</v>
       </c>
       <c r="E5" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.45">
@@ -16907,24 +16909,7 @@
         <v>1</v>
       </c>
       <c r="E6" t="s">
-        <v>325</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A7">
-        <v>5</v>
-      </c>
-      <c r="B7">
-        <v>360000000</v>
-      </c>
-      <c r="C7">
-        <v>100</v>
-      </c>
-      <c r="D7">
-        <v>1</v>
-      </c>
-      <c r="E7" t="s">
-        <v>329</v>
+        <v>324</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.45">
@@ -18008,114 +17993,119 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:G363"/>
+  <dimension ref="A1:L363"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A1" s="7" t="s">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="A1" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="B1" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="C1" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="D1" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="E1" s="7" t="s">
+      <c r="E1" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="F1" s="7" t="s">
+      <c r="F1" s="6" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A2" s="7">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="A2" s="6">
         <v>0</v>
       </c>
       <c r="B2" s="1">
-        <v>3.0000000000000003E-4</v>
+        <v>5.5555555555555556E-4</v>
       </c>
       <c r="C2" s="1">
-        <v>3.0000000000000001E-6</v>
+        <v>5.5555555555555558E-5</v>
       </c>
       <c r="D2" s="1">
-        <v>2.9999999999999997E-4</v>
+        <v>5.5555555555555556E-4</v>
       </c>
       <c r="E2" s="1">
-        <v>3.0000000000000001E-6</v>
+        <v>5.5555555555555558E-5</v>
       </c>
       <c r="F2" s="1">
-        <v>2.9999999999999997E-4</v>
+        <v>5.5555555555555556E-4</v>
       </c>
       <c r="G2" s="3"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A3" s="7">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="A3" s="6">
         <v>3600000</v>
       </c>
       <c r="B3" s="1">
-        <v>1.5E-5</v>
+        <v>5.5555555555555558E-5</v>
       </c>
       <c r="C3" s="1">
-        <v>1.4999999999999999E-7</v>
+        <v>5.5555555555555558E-6</v>
       </c>
       <c r="D3" s="1">
-        <v>1.4999999999999999E-5</v>
+        <v>5.5555555555555558E-5</v>
       </c>
       <c r="E3" s="1">
-        <v>1.4999999999999999E-7</v>
+        <v>5.5555555555555558E-6</v>
       </c>
       <c r="F3" s="1">
-        <v>1.4999999999999999E-5</v>
+        <v>5.5555555555555558E-5</v>
       </c>
       <c r="G3" s="3"/>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A4" s="7">
+      <c r="H3" s="1"/>
+      <c r="I3" s="1"/>
+      <c r="J3" s="1"/>
+      <c r="K3" s="1"/>
+      <c r="L3" s="1"/>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="A4" s="6">
         <v>400000000</v>
       </c>
       <c r="B4" s="1">
-        <v>1.4999999999999999E-5</v>
+        <v>5.5555555555555558E-5</v>
       </c>
       <c r="C4" s="1">
-        <v>1.4999999999999999E-7</v>
+        <v>5.5555555555555558E-6</v>
       </c>
       <c r="D4" s="1">
-        <v>1.4999999999999999E-5</v>
+        <v>5.5555555555555558E-5</v>
       </c>
       <c r="E4" s="1">
-        <v>1.4999999999999999E-7</v>
+        <v>5.5555555555555558E-6</v>
       </c>
       <c r="F4" s="1">
-        <v>1.4999999999999999E-5</v>
+        <v>5.5555555555555558E-5</v>
       </c>
       <c r="G4" s="3"/>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.45">
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
       <c r="D5" s="1"/>
       <c r="E5" s="1"/>
       <c r="F5" s="1"/>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.45">
       <c r="B6" s="1"/>
       <c r="C6" s="1"/>
       <c r="D6" s="1"/>
       <c r="E6" s="1"/>
       <c r="F6" s="1"/>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.45">
       <c r="B7" s="1"/>
       <c r="C7" s="3"/>
       <c r="D7" s="3"/>
       <c r="E7" s="1"/>
       <c r="F7" s="1"/>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.45">
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
       <c r="D8" s="1"/>
@@ -18123,7 +18113,7 @@
       <c r="F8" s="1"/>
       <c r="G8" s="1"/>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.45">
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
       <c r="D9" s="1"/>
@@ -18131,7 +18121,7 @@
       <c r="F9" s="1"/>
       <c r="G9" s="1"/>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.45">
       <c r="B10" s="1"/>
       <c r="C10" s="1"/>
       <c r="D10" s="1"/>
@@ -18139,7 +18129,7 @@
       <c r="F10" s="1"/>
       <c r="G10" s="1"/>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.45">
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
       <c r="D11" s="1"/>
@@ -18147,7 +18137,7 @@
       <c r="F11" s="1"/>
       <c r="G11" s="1"/>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.45">
       <c r="B12" s="1"/>
       <c r="C12" s="1"/>
       <c r="D12" s="1"/>
@@ -18155,7 +18145,7 @@
       <c r="F12" s="1"/>
       <c r="G12" s="1"/>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.45">
       <c r="B13" s="1"/>
       <c r="C13" s="1"/>
       <c r="D13" s="1"/>
@@ -18163,7 +18153,7 @@
       <c r="F13" s="1"/>
       <c r="G13" s="1"/>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.45">
       <c r="B14" s="1"/>
       <c r="C14" s="1"/>
       <c r="D14" s="1"/>
@@ -18171,7 +18161,7 @@
       <c r="F14" s="1"/>
       <c r="G14" s="1"/>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.45">
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
       <c r="D15" s="1"/>
@@ -18179,7 +18169,7 @@
       <c r="F15" s="1"/>
       <c r="G15" s="1"/>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.45">
       <c r="B16" s="1"/>
       <c r="C16" s="1"/>
       <c r="D16" s="1"/>
@@ -21376,7 +21366,7 @@
         <v>32</v>
       </c>
       <c r="B22" s="1">
-        <v>1.4999999999999999E-5</v>
+        <v>5.5555555555555558E-5</v>
       </c>
       <c r="C22">
         <v>3.1154231364886891E-4</v>
@@ -21402,7 +21392,7 @@
         <v>33</v>
       </c>
       <c r="B23" s="1">
-        <v>1.4999999999999999E-7</v>
+        <v>5.5555555555555558E-6</v>
       </c>
       <c r="C23">
         <v>3.1154231364886891E-5</v>
@@ -21428,7 +21418,7 @@
         <v>34</v>
       </c>
       <c r="B24" s="1">
-        <v>1.4999999999999999E-5</v>
+        <v>5.5555555555555558E-5</v>
       </c>
       <c r="C24">
         <v>3.1154231364886891E-4</v>
@@ -21454,7 +21444,7 @@
         <v>35</v>
       </c>
       <c r="B25" s="1">
-        <v>1.4999999999999999E-7</v>
+        <v>5.5555555555555558E-6</v>
       </c>
       <c r="C25">
         <v>3.1154231364886891E-5</v>
@@ -21480,7 +21470,7 @@
         <v>36</v>
       </c>
       <c r="B26" s="1">
-        <v>1.4999999999999999E-5</v>
+        <v>5.5555555555555558E-5</v>
       </c>
       <c r="C26">
         <v>3.1154231364886891E-4</v>
@@ -21632,8 +21622,8 @@
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A32" s="8" t="s">
-        <v>327</v>
+      <c r="A32" s="7" t="s">
+        <v>326</v>
       </c>
       <c r="B32" s="1">
         <v>0</v>
@@ -21654,18 +21644,18 @@
         <v>0</v>
       </c>
       <c r="H32" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="5" type="noConversion"/>
+  <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="37" bestFit="1" customWidth="1"/>
@@ -21689,37 +21679,105 @@
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A2">
-        <v>3</v>
+      <c r="A2" t="s">
+        <v>329</v>
       </c>
       <c r="B2" t="s">
         <v>83</v>
       </c>
       <c r="C2">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D2">
-        <v>0</v>
+        <v>225</v>
       </c>
       <c r="E2">
-        <v>597</v>
+        <v>300</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A3">
-        <v>4</v>
+      <c r="A3" t="s">
+        <v>330</v>
       </c>
       <c r="B3" t="s">
         <v>83</v>
       </c>
       <c r="C3">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D3">
-        <v>0</v>
+        <v>225</v>
       </c>
       <c r="E3">
-        <v>596</v>
+        <v>300</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A4" t="s">
+        <v>331</v>
+      </c>
+      <c r="B4" t="s">
+        <v>83</v>
+      </c>
+      <c r="C4">
+        <v>12</v>
+      </c>
+      <c r="D4">
+        <v>225</v>
+      </c>
+      <c r="E4">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A5" t="s">
+        <v>332</v>
+      </c>
+      <c r="B5" t="s">
+        <v>83</v>
+      </c>
+      <c r="C5">
+        <v>17</v>
+      </c>
+      <c r="D5">
+        <v>225</v>
+      </c>
+      <c r="E5">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A6" t="s">
+        <v>333</v>
+      </c>
+      <c r="B6" t="s">
+        <v>83</v>
+      </c>
+      <c r="C6">
+        <v>22</v>
+      </c>
+      <c r="D6">
+        <v>225</v>
+      </c>
+      <c r="E6">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A7" t="s">
+        <v>334</v>
+      </c>
+      <c r="B7" t="s">
+        <v>335</v>
+      </c>
+      <c r="C7">
+        <v>12</v>
+      </c>
+      <c r="D7">
+        <v>225</v>
+      </c>
+      <c r="E7">
+        <v>112</v>
       </c>
     </row>
   </sheetData>
@@ -21729,7 +21787,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.06640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="9.73046875" bestFit="1" customWidth="1"/>
@@ -21766,10 +21824,10 @@
         <v>12</v>
       </c>
       <c r="D2">
-        <v>0</v>
+        <v>224</v>
       </c>
       <c r="E2">
-        <v>400</v>
+        <v>299</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -21779,17 +21837,17 @@
       <c r="A3" t="s">
         <v>86</v>
       </c>
-      <c r="B3" s="7">
+      <c r="B3" s="6">
         <v>3600000</v>
       </c>
       <c r="C3">
         <v>12</v>
       </c>
       <c r="D3">
-        <v>0</v>
+        <v>224</v>
       </c>
       <c r="E3">
-        <v>400</v>
+        <v>299</v>
       </c>
       <c r="F3">
         <v>0</v>
@@ -21806,10 +21864,10 @@
         <v>12</v>
       </c>
       <c r="D4">
-        <v>0</v>
+        <v>224</v>
       </c>
       <c r="E4">
-        <v>400</v>
+        <v>299</v>
       </c>
       <c r="F4">
         <v>0</v>
@@ -21826,10 +21884,10 @@
         <v>12</v>
       </c>
       <c r="D5">
-        <v>0</v>
+        <v>224</v>
       </c>
       <c r="E5">
-        <v>399</v>
+        <v>300</v>
       </c>
       <c r="F5">
         <v>0</v>
@@ -21839,17 +21897,17 @@
       <c r="A6" t="s">
         <v>87</v>
       </c>
-      <c r="B6" s="7">
+      <c r="B6" s="6">
         <v>3600000</v>
       </c>
       <c r="C6">
         <v>12</v>
       </c>
       <c r="D6">
-        <v>0</v>
+        <v>224</v>
       </c>
       <c r="E6">
-        <v>399</v>
+        <v>300</v>
       </c>
       <c r="F6">
         <v>0</v>
@@ -21866,10 +21924,10 @@
         <v>12</v>
       </c>
       <c r="D7">
-        <v>0</v>
+        <v>224</v>
       </c>
       <c r="E7">
-        <v>399</v>
+        <v>300</v>
       </c>
       <c r="F7">
         <v>0</v>
@@ -21886,10 +21944,10 @@
         <v>12</v>
       </c>
       <c r="D8">
-        <v>0</v>
+        <v>224</v>
       </c>
       <c r="E8">
-        <v>401</v>
+        <v>301</v>
       </c>
       <c r="F8">
         <v>0</v>
@@ -21899,17 +21957,17 @@
       <c r="A9" t="s">
         <v>88</v>
       </c>
-      <c r="B9" s="7">
+      <c r="B9" s="6">
         <v>3600000</v>
       </c>
       <c r="C9">
         <v>12</v>
       </c>
       <c r="D9">
-        <v>0</v>
+        <v>224</v>
       </c>
       <c r="E9">
-        <v>401</v>
+        <v>301</v>
       </c>
       <c r="F9">
         <v>0</v>
@@ -21926,10 +21984,10 @@
         <v>12</v>
       </c>
       <c r="D10">
-        <v>0</v>
+        <v>224</v>
       </c>
       <c r="E10">
-        <v>401</v>
+        <v>301</v>
       </c>
       <c r="F10">
         <v>0</v>
@@ -21946,10 +22004,10 @@
         <v>12</v>
       </c>
       <c r="D11">
-        <v>0</v>
+        <v>225</v>
       </c>
       <c r="E11">
-        <v>402</v>
+        <v>299</v>
       </c>
       <c r="F11">
         <v>0</v>
@@ -21959,17 +22017,17 @@
       <c r="A12" t="s">
         <v>89</v>
       </c>
-      <c r="B12" s="7">
+      <c r="B12" s="6">
         <v>3600000</v>
       </c>
       <c r="C12">
         <v>12</v>
       </c>
       <c r="D12">
-        <v>0</v>
+        <v>225</v>
       </c>
       <c r="E12">
-        <v>402</v>
+        <v>299</v>
       </c>
       <c r="F12">
         <v>0</v>
@@ -21986,10 +22044,10 @@
         <v>12</v>
       </c>
       <c r="D13">
-        <v>0</v>
+        <v>225</v>
       </c>
       <c r="E13">
-        <v>402</v>
+        <v>299</v>
       </c>
       <c r="F13">
         <v>0</v>
@@ -22006,10 +22064,10 @@
         <v>12</v>
       </c>
       <c r="D14">
-        <v>0</v>
+        <v>225</v>
       </c>
       <c r="E14">
-        <v>398</v>
+        <v>300</v>
       </c>
       <c r="F14">
         <v>0</v>
@@ -22019,17 +22077,17 @@
       <c r="A15" t="s">
         <v>90</v>
       </c>
-      <c r="B15" s="7">
+      <c r="B15" s="6">
         <v>3600000</v>
       </c>
       <c r="C15">
         <v>12</v>
       </c>
       <c r="D15">
-        <v>0</v>
+        <v>225</v>
       </c>
       <c r="E15">
-        <v>398</v>
+        <v>300</v>
       </c>
       <c r="F15">
         <v>0</v>
@@ -22046,12 +22104,252 @@
         <v>12</v>
       </c>
       <c r="D16">
+        <v>225</v>
+      </c>
+      <c r="E16">
+        <v>300</v>
+      </c>
+      <c r="F16">
         <v>0</v>
       </c>
-      <c r="E16">
-        <v>398</v>
-      </c>
-      <c r="F16">
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A17" t="s">
+        <v>123</v>
+      </c>
+      <c r="B17">
+        <v>0</v>
+      </c>
+      <c r="C17">
+        <v>12</v>
+      </c>
+      <c r="D17">
+        <v>225</v>
+      </c>
+      <c r="E17">
+        <v>301</v>
+      </c>
+      <c r="F17">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A18" t="s">
+        <v>123</v>
+      </c>
+      <c r="B18" s="6">
+        <v>3600000</v>
+      </c>
+      <c r="C18">
+        <v>12</v>
+      </c>
+      <c r="D18">
+        <v>225</v>
+      </c>
+      <c r="E18">
+        <v>301</v>
+      </c>
+      <c r="F18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A19" t="s">
+        <v>123</v>
+      </c>
+      <c r="B19">
+        <v>400000000</v>
+      </c>
+      <c r="C19">
+        <v>12</v>
+      </c>
+      <c r="D19">
+        <v>225</v>
+      </c>
+      <c r="E19">
+        <v>301</v>
+      </c>
+      <c r="F19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A20" t="s">
+        <v>336</v>
+      </c>
+      <c r="B20">
+        <v>0</v>
+      </c>
+      <c r="C20">
+        <v>12</v>
+      </c>
+      <c r="D20">
+        <v>226</v>
+      </c>
+      <c r="E20">
+        <v>299</v>
+      </c>
+      <c r="F20">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A21" t="s">
+        <v>336</v>
+      </c>
+      <c r="B21" s="6">
+        <v>3600000</v>
+      </c>
+      <c r="C21">
+        <v>12</v>
+      </c>
+      <c r="D21">
+        <v>226</v>
+      </c>
+      <c r="E21">
+        <v>299</v>
+      </c>
+      <c r="F21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A22" t="s">
+        <v>336</v>
+      </c>
+      <c r="B22">
+        <v>400000000</v>
+      </c>
+      <c r="C22">
+        <v>12</v>
+      </c>
+      <c r="D22">
+        <v>226</v>
+      </c>
+      <c r="E22">
+        <v>299</v>
+      </c>
+      <c r="F22">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A23" t="s">
+        <v>337</v>
+      </c>
+      <c r="B23">
+        <v>0</v>
+      </c>
+      <c r="C23">
+        <v>12</v>
+      </c>
+      <c r="D23">
+        <v>226</v>
+      </c>
+      <c r="E23">
+        <v>300</v>
+      </c>
+      <c r="F23">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A24" t="s">
+        <v>337</v>
+      </c>
+      <c r="B24" s="6">
+        <v>3600000</v>
+      </c>
+      <c r="C24">
+        <v>12</v>
+      </c>
+      <c r="D24">
+        <v>226</v>
+      </c>
+      <c r="E24">
+        <v>300</v>
+      </c>
+      <c r="F24">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A25" t="s">
+        <v>337</v>
+      </c>
+      <c r="B25">
+        <v>400000000</v>
+      </c>
+      <c r="C25">
+        <v>12</v>
+      </c>
+      <c r="D25">
+        <v>226</v>
+      </c>
+      <c r="E25">
+        <v>300</v>
+      </c>
+      <c r="F25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A26" t="s">
+        <v>338</v>
+      </c>
+      <c r="B26">
+        <v>0</v>
+      </c>
+      <c r="C26">
+        <v>12</v>
+      </c>
+      <c r="D26">
+        <v>226</v>
+      </c>
+      <c r="E26">
+        <v>301</v>
+      </c>
+      <c r="F26">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A27" t="s">
+        <v>338</v>
+      </c>
+      <c r="B27" s="6">
+        <v>3600000</v>
+      </c>
+      <c r="C27">
+        <v>12</v>
+      </c>
+      <c r="D27">
+        <v>226</v>
+      </c>
+      <c r="E27">
+        <v>301</v>
+      </c>
+      <c r="F27">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A28" t="s">
+        <v>338</v>
+      </c>
+      <c r="B28">
+        <v>400000000</v>
+      </c>
+      <c r="C28">
+        <v>12</v>
+      </c>
+      <c r="D28">
+        <v>226</v>
+      </c>
+      <c r="E28">
+        <v>301</v>
+      </c>
+      <c r="F28">
         <v>0</v>
       </c>
     </row>
@@ -22062,7 +22360,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:J10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.45">
@@ -22262,14 +22560,147 @@
         <v>-30</v>
       </c>
     </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="A7" t="s">
+        <v>123</v>
+      </c>
+      <c r="B7">
+        <v>0</v>
+      </c>
+      <c r="C7">
+        <f t="shared" ref="C7:C10" si="0">D7/2</f>
+        <v>-1</v>
+      </c>
+      <c r="D7">
+        <v>-2</v>
+      </c>
+      <c r="E7">
+        <v>-4</v>
+      </c>
+      <c r="F7">
+        <v>-6</v>
+      </c>
+      <c r="G7">
+        <v>-8</v>
+      </c>
+      <c r="H7">
+        <v>-10</v>
+      </c>
+      <c r="I7">
+        <v>-20</v>
+      </c>
+      <c r="J7">
+        <v>-30</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="A8" t="s">
+        <v>336</v>
+      </c>
+      <c r="B8">
+        <v>0</v>
+      </c>
+      <c r="C8">
+        <f t="shared" si="0"/>
+        <v>-1</v>
+      </c>
+      <c r="D8">
+        <v>-2</v>
+      </c>
+      <c r="E8">
+        <v>-4</v>
+      </c>
+      <c r="F8">
+        <v>-6</v>
+      </c>
+      <c r="G8">
+        <v>-8</v>
+      </c>
+      <c r="H8">
+        <v>-10</v>
+      </c>
+      <c r="I8">
+        <v>-20</v>
+      </c>
+      <c r="J8">
+        <v>-30</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="A9" t="s">
+        <v>337</v>
+      </c>
+      <c r="B9">
+        <v>0</v>
+      </c>
+      <c r="C9">
+        <f t="shared" si="0"/>
+        <v>-1</v>
+      </c>
+      <c r="D9">
+        <v>-2</v>
+      </c>
+      <c r="E9">
+        <v>-4</v>
+      </c>
+      <c r="F9">
+        <v>-6</v>
+      </c>
+      <c r="G9">
+        <v>-8</v>
+      </c>
+      <c r="H9">
+        <v>-10</v>
+      </c>
+      <c r="I9">
+        <v>-20</v>
+      </c>
+      <c r="J9">
+        <v>-30</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="A10" t="s">
+        <v>338</v>
+      </c>
+      <c r="B10">
+        <v>0</v>
+      </c>
+      <c r="C10">
+        <f t="shared" si="0"/>
+        <v>-1</v>
+      </c>
+      <c r="D10">
+        <v>-2</v>
+      </c>
+      <c r="E10">
+        <v>-4</v>
+      </c>
+      <c r="F10">
+        <v>-6</v>
+      </c>
+      <c r="G10">
+        <v>-8</v>
+      </c>
+      <c r="H10">
+        <v>-10</v>
+      </c>
+      <c r="I10">
+        <v>-20</v>
+      </c>
+      <c r="J10">
+        <v>-30</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="A1:K16"/>
+  <dimension ref="A1:K28"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.45">
@@ -22346,8 +22777,8 @@
       <c r="A3" t="s">
         <v>86</v>
       </c>
-      <c r="B3">
-        <v>7578000</v>
+      <c r="B3" s="6">
+        <v>3600000</v>
       </c>
       <c r="C3">
         <v>0</v>
@@ -22382,7 +22813,7 @@
         <v>86</v>
       </c>
       <c r="B4">
-        <v>30000000</v>
+        <v>400000000</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -22451,8 +22882,8 @@
       <c r="A6" t="s">
         <v>87</v>
       </c>
-      <c r="B6">
-        <v>7578000</v>
+      <c r="B6" s="6">
+        <v>3600000</v>
       </c>
       <c r="C6">
         <v>0</v>
@@ -22487,7 +22918,7 @@
         <v>87</v>
       </c>
       <c r="B7">
-        <v>30000000</v>
+        <v>400000000</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -22556,8 +22987,8 @@
       <c r="A9" t="s">
         <v>88</v>
       </c>
-      <c r="B9">
-        <v>7578000</v>
+      <c r="B9" s="6">
+        <v>3600000</v>
       </c>
       <c r="C9">
         <v>0</v>
@@ -22592,7 +23023,7 @@
         <v>88</v>
       </c>
       <c r="B10">
-        <v>30000000</v>
+        <v>400000000</v>
       </c>
       <c r="C10">
         <v>0</v>
@@ -22661,8 +23092,8 @@
       <c r="A12" t="s">
         <v>89</v>
       </c>
-      <c r="B12">
-        <v>7578000</v>
+      <c r="B12" s="6">
+        <v>3600000</v>
       </c>
       <c r="C12">
         <v>0</v>
@@ -22697,7 +23128,7 @@
         <v>89</v>
       </c>
       <c r="B13">
-        <v>30000000</v>
+        <v>400000000</v>
       </c>
       <c r="C13">
         <v>0</v>
@@ -22766,8 +23197,8 @@
       <c r="A15" t="s">
         <v>90</v>
       </c>
-      <c r="B15">
-        <v>7578000</v>
+      <c r="B15" s="6">
+        <v>3600000</v>
       </c>
       <c r="C15">
         <v>0</v>
@@ -22802,7 +23233,7 @@
         <v>90</v>
       </c>
       <c r="B16">
-        <v>30000000</v>
+        <v>400000000</v>
       </c>
       <c r="C16">
         <v>0</v>
@@ -22829,6 +23260,426 @@
         <v>-20</v>
       </c>
       <c r="K16">
+        <v>-30</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A17" t="s">
+        <v>123</v>
+      </c>
+      <c r="B17">
+        <v>0</v>
+      </c>
+      <c r="C17">
+        <v>0</v>
+      </c>
+      <c r="D17">
+        <v>0</v>
+      </c>
+      <c r="E17">
+        <v>0</v>
+      </c>
+      <c r="F17">
+        <v>0</v>
+      </c>
+      <c r="G17">
+        <v>0</v>
+      </c>
+      <c r="H17">
+        <v>0</v>
+      </c>
+      <c r="I17">
+        <v>0</v>
+      </c>
+      <c r="J17">
+        <v>0</v>
+      </c>
+      <c r="K17">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A18" t="s">
+        <v>123</v>
+      </c>
+      <c r="B18" s="6">
+        <v>3600000</v>
+      </c>
+      <c r="C18">
+        <v>0</v>
+      </c>
+      <c r="D18">
+        <v>-1</v>
+      </c>
+      <c r="E18">
+        <v>-2</v>
+      </c>
+      <c r="F18">
+        <v>-4</v>
+      </c>
+      <c r="G18">
+        <v>-6</v>
+      </c>
+      <c r="H18">
+        <v>-8</v>
+      </c>
+      <c r="I18">
+        <v>-10</v>
+      </c>
+      <c r="J18">
+        <v>-20</v>
+      </c>
+      <c r="K18">
+        <v>-30</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A19" t="s">
+        <v>123</v>
+      </c>
+      <c r="B19">
+        <v>400000000</v>
+      </c>
+      <c r="C19">
+        <v>0</v>
+      </c>
+      <c r="D19">
+        <v>-1</v>
+      </c>
+      <c r="E19">
+        <v>-2</v>
+      </c>
+      <c r="F19">
+        <v>-4</v>
+      </c>
+      <c r="G19">
+        <v>-6</v>
+      </c>
+      <c r="H19">
+        <v>-8</v>
+      </c>
+      <c r="I19">
+        <v>-10</v>
+      </c>
+      <c r="J19">
+        <v>-20</v>
+      </c>
+      <c r="K19">
+        <v>-30</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A20" t="s">
+        <v>336</v>
+      </c>
+      <c r="B20">
+        <v>0</v>
+      </c>
+      <c r="C20">
+        <v>0</v>
+      </c>
+      <c r="D20">
+        <v>0</v>
+      </c>
+      <c r="E20">
+        <v>0</v>
+      </c>
+      <c r="F20">
+        <v>0</v>
+      </c>
+      <c r="G20">
+        <v>0</v>
+      </c>
+      <c r="H20">
+        <v>0</v>
+      </c>
+      <c r="I20">
+        <v>0</v>
+      </c>
+      <c r="J20">
+        <v>0</v>
+      </c>
+      <c r="K20">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A21" t="s">
+        <v>336</v>
+      </c>
+      <c r="B21" s="6">
+        <v>3600000</v>
+      </c>
+      <c r="C21">
+        <v>0</v>
+      </c>
+      <c r="D21">
+        <v>-1</v>
+      </c>
+      <c r="E21">
+        <v>-2</v>
+      </c>
+      <c r="F21">
+        <v>-4</v>
+      </c>
+      <c r="G21">
+        <v>-6</v>
+      </c>
+      <c r="H21">
+        <v>-8</v>
+      </c>
+      <c r="I21">
+        <v>-10</v>
+      </c>
+      <c r="J21">
+        <v>-20</v>
+      </c>
+      <c r="K21">
+        <v>-30</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A22" t="s">
+        <v>336</v>
+      </c>
+      <c r="B22">
+        <v>400000000</v>
+      </c>
+      <c r="C22">
+        <v>0</v>
+      </c>
+      <c r="D22">
+        <v>-1</v>
+      </c>
+      <c r="E22">
+        <v>-2</v>
+      </c>
+      <c r="F22">
+        <v>-4</v>
+      </c>
+      <c r="G22">
+        <v>-6</v>
+      </c>
+      <c r="H22">
+        <v>-8</v>
+      </c>
+      <c r="I22">
+        <v>-10</v>
+      </c>
+      <c r="J22">
+        <v>-20</v>
+      </c>
+      <c r="K22">
+        <v>-30</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A23" t="s">
+        <v>337</v>
+      </c>
+      <c r="B23">
+        <v>0</v>
+      </c>
+      <c r="C23">
+        <v>0</v>
+      </c>
+      <c r="D23">
+        <v>0</v>
+      </c>
+      <c r="E23">
+        <v>0</v>
+      </c>
+      <c r="F23">
+        <v>0</v>
+      </c>
+      <c r="G23">
+        <v>0</v>
+      </c>
+      <c r="H23">
+        <v>0</v>
+      </c>
+      <c r="I23">
+        <v>0</v>
+      </c>
+      <c r="J23">
+        <v>0</v>
+      </c>
+      <c r="K23">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A24" t="s">
+        <v>337</v>
+      </c>
+      <c r="B24" s="6">
+        <v>3600000</v>
+      </c>
+      <c r="C24">
+        <v>0</v>
+      </c>
+      <c r="D24">
+        <v>-1</v>
+      </c>
+      <c r="E24">
+        <v>-2</v>
+      </c>
+      <c r="F24">
+        <v>-4</v>
+      </c>
+      <c r="G24">
+        <v>-6</v>
+      </c>
+      <c r="H24">
+        <v>-8</v>
+      </c>
+      <c r="I24">
+        <v>-10</v>
+      </c>
+      <c r="J24">
+        <v>-20</v>
+      </c>
+      <c r="K24">
+        <v>-30</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A25" t="s">
+        <v>337</v>
+      </c>
+      <c r="B25">
+        <v>400000000</v>
+      </c>
+      <c r="C25">
+        <v>0</v>
+      </c>
+      <c r="D25">
+        <v>-1</v>
+      </c>
+      <c r="E25">
+        <v>-2</v>
+      </c>
+      <c r="F25">
+        <v>-4</v>
+      </c>
+      <c r="G25">
+        <v>-6</v>
+      </c>
+      <c r="H25">
+        <v>-8</v>
+      </c>
+      <c r="I25">
+        <v>-10</v>
+      </c>
+      <c r="J25">
+        <v>-20</v>
+      </c>
+      <c r="K25">
+        <v>-30</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A26" t="s">
+        <v>338</v>
+      </c>
+      <c r="B26">
+        <v>0</v>
+      </c>
+      <c r="C26">
+        <v>0</v>
+      </c>
+      <c r="D26">
+        <v>0</v>
+      </c>
+      <c r="E26">
+        <v>0</v>
+      </c>
+      <c r="F26">
+        <v>0</v>
+      </c>
+      <c r="G26">
+        <v>0</v>
+      </c>
+      <c r="H26">
+        <v>0</v>
+      </c>
+      <c r="I26">
+        <v>0</v>
+      </c>
+      <c r="J26">
+        <v>0</v>
+      </c>
+      <c r="K26">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A27" t="s">
+        <v>338</v>
+      </c>
+      <c r="B27" s="6">
+        <v>3600000</v>
+      </c>
+      <c r="C27">
+        <v>0</v>
+      </c>
+      <c r="D27">
+        <v>-1</v>
+      </c>
+      <c r="E27">
+        <v>-2</v>
+      </c>
+      <c r="F27">
+        <v>-4</v>
+      </c>
+      <c r="G27">
+        <v>-6</v>
+      </c>
+      <c r="H27">
+        <v>-8</v>
+      </c>
+      <c r="I27">
+        <v>-10</v>
+      </c>
+      <c r="J27">
+        <v>-20</v>
+      </c>
+      <c r="K27">
+        <v>-30</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A28" t="s">
+        <v>338</v>
+      </c>
+      <c r="B28">
+        <v>400000000</v>
+      </c>
+      <c r="C28">
+        <v>0</v>
+      </c>
+      <c r="D28">
+        <v>-1</v>
+      </c>
+      <c r="E28">
+        <v>-2</v>
+      </c>
+      <c r="F28">
+        <v>-4</v>
+      </c>
+      <c r="G28">
+        <v>-6</v>
+      </c>
+      <c r="H28">
+        <v>-8</v>
+      </c>
+      <c r="I28">
+        <v>-10</v>
+      </c>
+      <c r="J28">
+        <v>-20</v>
+      </c>
+      <c r="K28">
         <v>-30</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix plotting functions in modtransient6 and starts adding a new iterate_pumping_rate_transient function to modpump
</commit_message>
<xml_diff>
--- a/setup.xlsx
+++ b/setup.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="X:\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cmarinriver\Projects\ConfinedLab\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01A7D49A-AAD6-45E3-A045-8B734DDF89A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDDBCA2E-14E4-4EED-84CD-DEACA90F24F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11620" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11620" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="grid" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="591" uniqueCount="341">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="564" uniqueCount="339">
   <si>
     <t>nlay</t>
   </si>
@@ -1054,19 +1054,13 @@
     <t xml:space="preserve">HEAD </t>
   </si>
   <si>
-    <t>WELL_07</t>
-  </si>
-  <si>
-    <t>WELL_08</t>
-  </si>
-  <si>
-    <t>WELL_09</t>
-  </si>
-  <si>
     <t>transition_cells</t>
   </si>
   <si>
     <t>epsilon</t>
+  </si>
+  <si>
+    <t>Caq 2 outcrop</t>
   </si>
 </sst>
 </file>
@@ -1530,22 +1524,22 @@
         <v>5</v>
       </c>
       <c r="B2">
-        <v>100</v>
+        <v>1</v>
       </c>
       <c r="C2">
-        <v>100</v>
+        <v>450</v>
       </c>
       <c r="D2">
-        <v>450000</v>
+        <v>1</v>
       </c>
       <c r="E2">
         <v>450000</v>
       </c>
       <c r="F2">
-        <v>4500</v>
+        <v>1</v>
       </c>
       <c r="G2">
-        <v>4500</v>
+        <v>1000</v>
       </c>
     </row>
   </sheetData>
@@ -16642,7 +16636,7 @@
     <col min="4" max="4" width="11.54296875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="11.81640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="14.08984375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.1796875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.90625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="8.36328125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="8.453125" customWidth="1"/>
   </cols>
@@ -16673,10 +16667,10 @@
         <v>325</v>
       </c>
       <c r="I1" t="s">
-        <v>339</v>
+        <v>336</v>
       </c>
       <c r="J1" t="s">
-        <v>340</v>
+        <v>337</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.35">
@@ -16690,7 +16684,7 @@
         <v>100</v>
       </c>
       <c r="D2">
-        <v>-50</v>
+        <v>0</v>
       </c>
       <c r="E2">
         <v>100</v>
@@ -16699,13 +16693,13 @@
         <v>300</v>
       </c>
       <c r="G2" s="8">
-        <v>50</v>
+        <v>225</v>
       </c>
       <c r="H2">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I2">
-        <v>11</v>
+        <v>52</v>
       </c>
       <c r="J2">
         <v>0</v>
@@ -16725,19 +16719,19 @@
         <v>100</v>
       </c>
       <c r="E3">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="F3">
         <v>150</v>
       </c>
       <c r="G3" s="8">
-        <v>42</v>
+        <v>190</v>
       </c>
       <c r="H3">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I3">
-        <v>11</v>
+        <v>52</v>
       </c>
       <c r="J3">
         <v>0</v>
@@ -16754,22 +16748,22 @@
         <v>200</v>
       </c>
       <c r="D4">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="E4">
-        <v>300</v>
+        <v>225</v>
       </c>
       <c r="F4">
         <v>200</v>
       </c>
       <c r="G4" s="8">
-        <v>25</v>
+        <v>112</v>
       </c>
       <c r="H4">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I4">
-        <v>11</v>
+        <v>52</v>
       </c>
       <c r="J4">
         <v>0</v>
@@ -16786,22 +16780,22 @@
         <v>250</v>
       </c>
       <c r="D5">
+        <v>225</v>
+      </c>
+      <c r="E5">
         <v>300</v>
-      </c>
-      <c r="E5">
-        <v>400</v>
       </c>
       <c r="F5">
         <v>150</v>
       </c>
       <c r="G5" s="8">
-        <v>17</v>
+        <v>76</v>
       </c>
       <c r="H5">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I5">
-        <v>11</v>
+        <v>52</v>
       </c>
       <c r="J5">
         <v>0</v>
@@ -16818,10 +16812,10 @@
         <v>350</v>
       </c>
       <c r="D6">
-        <v>400</v>
+        <v>300</v>
       </c>
       <c r="E6">
-        <v>450</v>
+        <v>350</v>
       </c>
       <c r="F6">
         <v>200</v>
@@ -16830,10 +16824,10 @@
         <v>0</v>
       </c>
       <c r="H6">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I6">
-        <v>11</v>
+        <v>52</v>
       </c>
       <c r="J6">
         <v>0</v>
@@ -16846,7 +16840,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:E365"/>
+  <dimension ref="A1:E364"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="5" max="5" width="40.90625" bestFit="1" customWidth="1"/>
@@ -16891,7 +16885,7 @@
         <v>1</v>
       </c>
       <c r="B3">
-        <v>2520000</v>
+        <v>3600000</v>
       </c>
       <c r="C3">
         <v>100</v>
@@ -16908,16 +16902,16 @@
         <v>2</v>
       </c>
       <c r="B4">
-        <v>1080000</v>
+        <v>180000</v>
       </c>
       <c r="C4">
-        <v>200</v>
+        <v>500</v>
       </c>
       <c r="D4">
         <v>1</v>
       </c>
       <c r="E4" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
@@ -16925,34 +16919,20 @@
         <v>3</v>
       </c>
       <c r="B5">
-        <v>180000</v>
+        <v>17820000</v>
       </c>
       <c r="C5">
-        <v>500</v>
+        <v>495</v>
       </c>
       <c r="D5">
         <v>1</v>
       </c>
       <c r="E5" t="s">
-        <v>323</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A6">
-        <v>4</v>
-      </c>
-      <c r="B6">
-        <v>17820000</v>
-      </c>
-      <c r="C6">
-        <v>495</v>
-      </c>
-      <c r="D6">
-        <v>1</v>
-      </c>
-      <c r="E6" t="s">
         <v>324</v>
       </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A7" s="3"/>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" s="3"/>
@@ -18024,9 +18004,6 @@
     </row>
     <row r="364" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A364" s="3"/>
-    </row>
-    <row r="365" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A365" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -18063,21 +18040,21 @@
         <v>0</v>
       </c>
       <c r="B2" s="1">
-        <v>5.5555555555555558E-5</v>
+        <v>5.9999999999999995E-4</v>
       </c>
       <c r="C2" s="1">
-        <v>5.5555555555555558E-6</v>
+        <v>6.0000000000000002E-5</v>
       </c>
       <c r="D2" s="1">
-        <v>5.5555555555555558E-5</v>
+        <v>5.9999999999999995E-4</v>
       </c>
       <c r="E2" s="1">
-        <v>5.5555555555555558E-6</v>
+        <v>6.0000000000000002E-5</v>
       </c>
       <c r="F2" s="1">
-        <v>5.5555555555555558E-5</v>
-      </c>
-      <c r="G2" s="3"/>
+        <v>5.9999999999999995E-4</v>
+      </c>
+      <c r="G2" s="1"/>
       <c r="H2" s="1"/>
       <c r="I2" s="1"/>
       <c r="J2" s="1"/>
@@ -18089,21 +18066,21 @@
         <v>3600000</v>
       </c>
       <c r="B3" s="1">
-        <v>5.5555555555555558E-5</v>
+        <v>9.9999999999999995E-7</v>
       </c>
       <c r="C3" s="1">
-        <v>5.5555555555555558E-6</v>
+        <v>9.9999999999999995E-8</v>
       </c>
       <c r="D3" s="1">
-        <v>5.5555555555555558E-5</v>
+        <v>9.9999999999999995E-7</v>
       </c>
       <c r="E3" s="1">
-        <v>5.5555555555555558E-6</v>
+        <v>9.9999999999999995E-8</v>
       </c>
       <c r="F3" s="1">
-        <v>5.5555555555555558E-5</v>
-      </c>
-      <c r="G3" s="3"/>
+        <v>9.9999999999999995E-7</v>
+      </c>
+      <c r="G3" s="1"/>
       <c r="H3" s="1"/>
       <c r="I3" s="1"/>
       <c r="J3" s="1"/>
@@ -18115,21 +18092,21 @@
         <v>400000000</v>
       </c>
       <c r="B4" s="1">
-        <v>5.5555555555555558E-5</v>
+        <v>9.9999999999999995E-7</v>
       </c>
       <c r="C4" s="1">
-        <v>5.5555555555555558E-6</v>
+        <v>9.9999999999999995E-8</v>
       </c>
       <c r="D4" s="1">
-        <v>5.5555555555555558E-5</v>
+        <v>9.9999999999999995E-7</v>
       </c>
       <c r="E4" s="1">
-        <v>5.5555555555555558E-6</v>
+        <v>9.9999999999999995E-8</v>
       </c>
       <c r="F4" s="1">
-        <v>5.5555555555555558E-5</v>
-      </c>
-      <c r="G4" s="3"/>
+        <v>9.9999999999999995E-7</v>
+      </c>
+      <c r="G4" s="1"/>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.35">
       <c r="B5" s="1"/>
@@ -18137,6 +18114,7 @@
       <c r="D5" s="1"/>
       <c r="E5" s="1"/>
       <c r="F5" s="1"/>
+      <c r="G5" s="1"/>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.35">
       <c r="B6" s="1"/>
@@ -20893,7 +20871,7 @@
         <v>44</v>
       </c>
       <c r="B2">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="C2">
         <v>225</v>
@@ -20919,7 +20897,7 @@
         <v>48</v>
       </c>
       <c r="B3" s="1">
-        <v>9.9999999999999995E-7</v>
+        <v>0.1</v>
       </c>
       <c r="C3">
         <v>9.0000000000000002E-6</v>
@@ -20945,7 +20923,7 @@
         <v>50</v>
       </c>
       <c r="B4">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="C4">
         <v>22.5</v>
@@ -20971,7 +20949,7 @@
         <v>52</v>
       </c>
       <c r="B5" s="1">
-        <v>9.9999999999999995E-7</v>
+        <v>0.1</v>
       </c>
       <c r="C5">
         <v>9.0000000000000002E-6</v>
@@ -20997,7 +20975,7 @@
         <v>54</v>
       </c>
       <c r="B6">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="C6">
         <v>22.5</v>
@@ -21049,7 +21027,7 @@
         <v>57</v>
       </c>
       <c r="B8" s="1">
-        <v>9.9999999999999995E-8</v>
+        <v>0.01</v>
       </c>
       <c r="C8">
         <v>9.0000000000000017E-7</v>
@@ -21101,7 +21079,7 @@
         <v>59</v>
       </c>
       <c r="B10" s="1">
-        <v>9.9999999999999995E-8</v>
+        <v>0.01</v>
       </c>
       <c r="C10">
         <v>9.0000000000000017E-7</v>
@@ -21413,7 +21391,7 @@
         <v>32</v>
       </c>
       <c r="B22" s="1">
-        <v>5.5555555555555558E-5</v>
+        <v>9.9999999999999995E-7</v>
       </c>
       <c r="C22">
         <v>3.1154231364886891E-4</v>
@@ -21439,7 +21417,7 @@
         <v>33</v>
       </c>
       <c r="B23" s="1">
-        <v>5.5555555555555558E-6</v>
+        <v>9.9999999999999995E-8</v>
       </c>
       <c r="C23">
         <v>3.1154231364886891E-5</v>
@@ -21465,7 +21443,7 @@
         <v>34</v>
       </c>
       <c r="B24" s="1">
-        <v>5.5555555555555558E-5</v>
+        <v>9.9999999999999995E-7</v>
       </c>
       <c r="C24">
         <v>3.1154231364886891E-4</v>
@@ -21491,7 +21469,7 @@
         <v>35</v>
       </c>
       <c r="B25" s="1">
-        <v>5.5555555555555558E-6</v>
+        <v>9.9999999999999995E-8</v>
       </c>
       <c r="C25">
         <v>3.1154231364886891E-5</v>
@@ -21517,7 +21495,7 @@
         <v>36</v>
       </c>
       <c r="B26" s="1">
-        <v>5.5555555555555558E-5</v>
+        <v>9.9999999999999995E-7</v>
       </c>
       <c r="C26">
         <v>3.1154231364886891E-4</v>
@@ -21673,7 +21651,7 @@
         <v>326</v>
       </c>
       <c r="B32" s="1">
-        <v>-50000</v>
+        <v>0</v>
       </c>
       <c r="C32">
         <v>3.1154231364886891E-4</v>
@@ -21702,7 +21680,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="37" bestFit="1" customWidth="1"/>
@@ -21736,10 +21714,10 @@
         <v>1</v>
       </c>
       <c r="D2">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="E2">
-        <v>67</v>
+        <v>300</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
@@ -21750,13 +21728,13 @@
         <v>83</v>
       </c>
       <c r="C3">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D3">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="E3">
-        <v>67</v>
+        <v>300</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
@@ -21767,13 +21745,13 @@
         <v>83</v>
       </c>
       <c r="C4">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="D4">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="E4">
-        <v>67</v>
+        <v>300</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
@@ -21784,13 +21762,13 @@
         <v>83</v>
       </c>
       <c r="C5">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D5">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="E5">
-        <v>67</v>
+        <v>300</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
@@ -21801,13 +21779,13 @@
         <v>83</v>
       </c>
       <c r="C6">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="D6">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="E6">
-        <v>67</v>
+        <v>300</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
@@ -21818,13 +21796,30 @@
         <v>335</v>
       </c>
       <c r="C7">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="D7">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="E7">
-        <v>25</v>
+        <v>125</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>338</v>
+      </c>
+      <c r="B8" t="s">
+        <v>335</v>
+      </c>
+      <c r="C8">
+        <v>22</v>
+      </c>
+      <c r="D8">
+        <v>0</v>
+      </c>
+      <c r="E8">
+        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -21834,7 +21829,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:F27"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.08984375" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="9.7265625" bestFit="1" customWidth="1"/>
@@ -21868,13 +21863,13 @@
         <v>0</v>
       </c>
       <c r="C2">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="D2">
-        <v>49</v>
+        <v>0</v>
       </c>
       <c r="E2">
-        <v>66</v>
+        <v>299</v>
       </c>
       <c r="F2">
         <v>0</v>
@@ -21888,16 +21883,16 @@
         <v>3600000</v>
       </c>
       <c r="C3">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="D3">
-        <v>49</v>
+        <v>0</v>
       </c>
       <c r="E3">
-        <v>66</v>
+        <v>299</v>
       </c>
       <c r="F3">
-        <v>-50000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
@@ -21908,16 +21903,16 @@
         <v>400000000</v>
       </c>
       <c r="C4">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="D4">
-        <v>49</v>
+        <v>0</v>
       </c>
       <c r="E4">
-        <v>66</v>
+        <v>299</v>
       </c>
       <c r="F4">
-        <v>-50000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.35">
@@ -21928,13 +21923,13 @@
         <v>0</v>
       </c>
       <c r="C5">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="D5">
-        <v>49</v>
+        <v>0</v>
       </c>
       <c r="E5">
-        <v>67</v>
+        <v>300</v>
       </c>
       <c r="F5">
         <v>0</v>
@@ -21948,16 +21943,16 @@
         <v>3600000</v>
       </c>
       <c r="C6">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="D6">
-        <v>49</v>
+        <v>0</v>
       </c>
       <c r="E6">
-        <v>67</v>
+        <v>300</v>
       </c>
       <c r="F6">
-        <v>-50000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.35">
@@ -21968,16 +21963,16 @@
         <v>400000000</v>
       </c>
       <c r="C7">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="D7">
-        <v>49</v>
+        <v>0</v>
       </c>
       <c r="E7">
-        <v>67</v>
+        <v>300</v>
       </c>
       <c r="F7">
-        <v>-50000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.35">
@@ -21988,13 +21983,13 @@
         <v>0</v>
       </c>
       <c r="C8">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="D8">
-        <v>49</v>
+        <v>0</v>
       </c>
       <c r="E8">
-        <v>68</v>
+        <v>301</v>
       </c>
       <c r="F8">
         <v>0</v>
@@ -22008,16 +22003,16 @@
         <v>3600000</v>
       </c>
       <c r="C9">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="D9">
-        <v>49</v>
+        <v>0</v>
       </c>
       <c r="E9">
-        <v>68</v>
+        <v>301</v>
       </c>
       <c r="F9">
-        <v>-50000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.35">
@@ -22028,16 +22023,16 @@
         <v>400000000</v>
       </c>
       <c r="C10">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="D10">
-        <v>49</v>
+        <v>0</v>
       </c>
       <c r="E10">
-        <v>68</v>
+        <v>301</v>
       </c>
       <c r="F10">
-        <v>-50000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.35">
@@ -22048,13 +22043,13 @@
         <v>0</v>
       </c>
       <c r="C11">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="D11">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="E11">
-        <v>66</v>
+        <v>298</v>
       </c>
       <c r="F11">
         <v>0</v>
@@ -22068,16 +22063,16 @@
         <v>3600000</v>
       </c>
       <c r="C12">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="D12">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="E12">
-        <v>66</v>
+        <v>298</v>
       </c>
       <c r="F12">
-        <v>-50000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.35">
@@ -22088,16 +22083,16 @@
         <v>400000000</v>
       </c>
       <c r="C13">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="D13">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="E13">
-        <v>66</v>
+        <v>298</v>
       </c>
       <c r="F13">
-        <v>-50000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.35">
@@ -22108,13 +22103,13 @@
         <v>0</v>
       </c>
       <c r="C14">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="D14">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="E14">
-        <v>67</v>
+        <v>302</v>
       </c>
       <c r="F14">
         <v>0</v>
@@ -22128,16 +22123,16 @@
         <v>3600000</v>
       </c>
       <c r="C15">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="D15">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="E15">
-        <v>67</v>
+        <v>302</v>
       </c>
       <c r="F15">
-        <v>-50000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.35">
@@ -22148,257 +22143,29 @@
         <v>400000000</v>
       </c>
       <c r="C16">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="D16">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="E16">
-        <v>67</v>
+        <v>302</v>
       </c>
       <c r="F16">
-        <v>-50000</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A17" t="s">
-        <v>123</v>
-      </c>
-      <c r="B17">
         <v>0</v>
       </c>
-      <c r="C17">
-        <v>7</v>
-      </c>
-      <c r="D17">
-        <v>50</v>
-      </c>
-      <c r="E17">
-        <v>68</v>
-      </c>
-      <c r="F17">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A18" t="s">
-        <v>123</v>
-      </c>
-      <c r="B18" s="6">
-        <v>3600000</v>
-      </c>
-      <c r="C18">
-        <v>7</v>
-      </c>
-      <c r="D18">
-        <v>50</v>
-      </c>
-      <c r="E18">
-        <v>68</v>
-      </c>
-      <c r="F18">
-        <v>-50000</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A19" t="s">
-        <v>123</v>
-      </c>
-      <c r="B19">
-        <v>400000000</v>
-      </c>
-      <c r="C19">
-        <v>7</v>
-      </c>
-      <c r="D19">
-        <v>50</v>
-      </c>
-      <c r="E19">
-        <v>68</v>
-      </c>
-      <c r="F19">
-        <v>-50000</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A20" t="s">
-        <v>336</v>
-      </c>
-      <c r="B20">
-        <v>0</v>
-      </c>
-      <c r="C20">
-        <v>7</v>
-      </c>
-      <c r="D20">
-        <v>51</v>
-      </c>
-      <c r="E20">
-        <v>66</v>
-      </c>
-      <c r="F20">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A21" t="s">
-        <v>336</v>
-      </c>
-      <c r="B21" s="6">
-        <v>3600000</v>
-      </c>
-      <c r="C21">
-        <v>7</v>
-      </c>
-      <c r="D21">
-        <v>51</v>
-      </c>
-      <c r="E21">
-        <v>66</v>
-      </c>
-      <c r="F21">
-        <v>-50000</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A22" t="s">
-        <v>336</v>
-      </c>
-      <c r="B22">
-        <v>400000000</v>
-      </c>
-      <c r="C22">
-        <v>7</v>
-      </c>
-      <c r="D22">
-        <v>51</v>
-      </c>
-      <c r="E22">
-        <v>66</v>
-      </c>
-      <c r="F22">
-        <v>-50000</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A23" t="s">
-        <v>337</v>
-      </c>
-      <c r="B23">
-        <v>0</v>
-      </c>
-      <c r="C23">
-        <v>7</v>
-      </c>
-      <c r="D23">
-        <v>51</v>
-      </c>
-      <c r="E23">
-        <v>67</v>
-      </c>
-      <c r="F23">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A24" t="s">
-        <v>337</v>
-      </c>
-      <c r="B24" s="6">
-        <v>3600000</v>
-      </c>
-      <c r="C24">
-        <v>7</v>
-      </c>
-      <c r="D24">
-        <v>51</v>
-      </c>
-      <c r="E24">
-        <v>67</v>
-      </c>
-      <c r="F24">
-        <v>-50000</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A25" t="s">
-        <v>337</v>
-      </c>
-      <c r="B25">
-        <v>400000000</v>
-      </c>
-      <c r="C25">
-        <v>7</v>
-      </c>
-      <c r="D25">
-        <v>51</v>
-      </c>
-      <c r="E25">
-        <v>67</v>
-      </c>
-      <c r="F25">
-        <v>-50000</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A26" t="s">
-        <v>338</v>
-      </c>
-      <c r="B26">
-        <v>0</v>
-      </c>
-      <c r="C26">
-        <v>7</v>
-      </c>
-      <c r="D26">
-        <v>51</v>
-      </c>
-      <c r="E26">
-        <v>68</v>
-      </c>
-      <c r="F26">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A27" t="s">
-        <v>338</v>
-      </c>
-      <c r="B27" s="6">
-        <v>3600000</v>
-      </c>
-      <c r="C27">
-        <v>7</v>
-      </c>
-      <c r="D27">
-        <v>51</v>
-      </c>
-      <c r="E27">
-        <v>68</v>
-      </c>
-      <c r="F27">
-        <v>-50000</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A28" t="s">
-        <v>338</v>
-      </c>
-      <c r="B28">
-        <v>400000000</v>
-      </c>
-      <c r="C28">
-        <v>7</v>
-      </c>
-      <c r="D28">
-        <v>51</v>
-      </c>
-      <c r="E28">
-        <v>68</v>
-      </c>
-      <c r="F28">
-        <v>-50000</v>
-      </c>
+    </row>
+    <row r="18" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B18" s="6"/>
+    </row>
+    <row r="21" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B21" s="6"/>
+    </row>
+    <row r="24" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B24" s="6"/>
+    </row>
+    <row r="27" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B27" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -22407,7 +22174,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
-  <dimension ref="A1:J10"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.35">
@@ -22604,138 +22371,6 @@
         <v>-20</v>
       </c>
       <c r="J6">
-        <v>-30</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
-        <v>123</v>
-      </c>
-      <c r="B7">
-        <v>0</v>
-      </c>
-      <c r="C7">
-        <f t="shared" ref="C7:C10" si="0">D7/2</f>
-        <v>-1</v>
-      </c>
-      <c r="D7">
-        <v>-2</v>
-      </c>
-      <c r="E7">
-        <v>-4</v>
-      </c>
-      <c r="F7">
-        <v>-6</v>
-      </c>
-      <c r="G7">
-        <v>-8</v>
-      </c>
-      <c r="H7">
-        <v>-10</v>
-      </c>
-      <c r="I7">
-        <v>-20</v>
-      </c>
-      <c r="J7">
-        <v>-30</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
-        <v>336</v>
-      </c>
-      <c r="B8">
-        <v>0</v>
-      </c>
-      <c r="C8">
-        <f t="shared" si="0"/>
-        <v>-1</v>
-      </c>
-      <c r="D8">
-        <v>-2</v>
-      </c>
-      <c r="E8">
-        <v>-4</v>
-      </c>
-      <c r="F8">
-        <v>-6</v>
-      </c>
-      <c r="G8">
-        <v>-8</v>
-      </c>
-      <c r="H8">
-        <v>-10</v>
-      </c>
-      <c r="I8">
-        <v>-20</v>
-      </c>
-      <c r="J8">
-        <v>-30</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
-        <v>337</v>
-      </c>
-      <c r="B9">
-        <v>0</v>
-      </c>
-      <c r="C9">
-        <f t="shared" si="0"/>
-        <v>-1</v>
-      </c>
-      <c r="D9">
-        <v>-2</v>
-      </c>
-      <c r="E9">
-        <v>-4</v>
-      </c>
-      <c r="F9">
-        <v>-6</v>
-      </c>
-      <c r="G9">
-        <v>-8</v>
-      </c>
-      <c r="H9">
-        <v>-10</v>
-      </c>
-      <c r="I9">
-        <v>-20</v>
-      </c>
-      <c r="J9">
-        <v>-30</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A10" t="s">
-        <v>338</v>
-      </c>
-      <c r="B10">
-        <v>0</v>
-      </c>
-      <c r="C10">
-        <f t="shared" si="0"/>
-        <v>-1</v>
-      </c>
-      <c r="D10">
-        <v>-2</v>
-      </c>
-      <c r="E10">
-        <v>-4</v>
-      </c>
-      <c r="F10">
-        <v>-6</v>
-      </c>
-      <c r="G10">
-        <v>-8</v>
-      </c>
-      <c r="H10">
-        <v>-10</v>
-      </c>
-      <c r="I10">
-        <v>-20</v>
-      </c>
-      <c r="J10">
         <v>-30</v>
       </c>
     </row>
@@ -22747,7 +22382,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="A1:K28"/>
+  <dimension ref="A1:K27"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.35">
@@ -23310,425 +22945,17 @@
         <v>-30</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A17" t="s">
-        <v>123</v>
-      </c>
-      <c r="B17">
-        <v>0</v>
-      </c>
-      <c r="C17">
-        <v>0</v>
-      </c>
-      <c r="D17">
-        <v>0</v>
-      </c>
-      <c r="E17">
-        <v>0</v>
-      </c>
-      <c r="F17">
-        <v>0</v>
-      </c>
-      <c r="G17">
-        <v>0</v>
-      </c>
-      <c r="H17">
-        <v>0</v>
-      </c>
-      <c r="I17">
-        <v>0</v>
-      </c>
-      <c r="J17">
-        <v>0</v>
-      </c>
-      <c r="K17">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A18" t="s">
-        <v>123</v>
-      </c>
-      <c r="B18" s="6">
-        <v>3600000</v>
-      </c>
-      <c r="C18">
-        <v>0</v>
-      </c>
-      <c r="D18">
-        <v>-1</v>
-      </c>
-      <c r="E18">
-        <v>-2</v>
-      </c>
-      <c r="F18">
-        <v>-4</v>
-      </c>
-      <c r="G18">
-        <v>-6</v>
-      </c>
-      <c r="H18">
-        <v>-8</v>
-      </c>
-      <c r="I18">
-        <v>-10</v>
-      </c>
-      <c r="J18">
-        <v>-20</v>
-      </c>
-      <c r="K18">
-        <v>-30</v>
-      </c>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A19" t="s">
-        <v>123</v>
-      </c>
-      <c r="B19">
-        <v>400000000</v>
-      </c>
-      <c r="C19">
-        <v>0</v>
-      </c>
-      <c r="D19">
-        <v>-1</v>
-      </c>
-      <c r="E19">
-        <v>-2</v>
-      </c>
-      <c r="F19">
-        <v>-4</v>
-      </c>
-      <c r="G19">
-        <v>-6</v>
-      </c>
-      <c r="H19">
-        <v>-8</v>
-      </c>
-      <c r="I19">
-        <v>-10</v>
-      </c>
-      <c r="J19">
-        <v>-20</v>
-      </c>
-      <c r="K19">
-        <v>-30</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A20" t="s">
-        <v>336</v>
-      </c>
-      <c r="B20">
-        <v>0</v>
-      </c>
-      <c r="C20">
-        <v>0</v>
-      </c>
-      <c r="D20">
-        <v>0</v>
-      </c>
-      <c r="E20">
-        <v>0</v>
-      </c>
-      <c r="F20">
-        <v>0</v>
-      </c>
-      <c r="G20">
-        <v>0</v>
-      </c>
-      <c r="H20">
-        <v>0</v>
-      </c>
-      <c r="I20">
-        <v>0</v>
-      </c>
-      <c r="J20">
-        <v>0</v>
-      </c>
-      <c r="K20">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A21" t="s">
-        <v>336</v>
-      </c>
-      <c r="B21" s="6">
-        <v>3600000</v>
-      </c>
-      <c r="C21">
-        <v>0</v>
-      </c>
-      <c r="D21">
-        <v>-1</v>
-      </c>
-      <c r="E21">
-        <v>-2</v>
-      </c>
-      <c r="F21">
-        <v>-4</v>
-      </c>
-      <c r="G21">
-        <v>-6</v>
-      </c>
-      <c r="H21">
-        <v>-8</v>
-      </c>
-      <c r="I21">
-        <v>-10</v>
-      </c>
-      <c r="J21">
-        <v>-20</v>
-      </c>
-      <c r="K21">
-        <v>-30</v>
-      </c>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A22" t="s">
-        <v>336</v>
-      </c>
-      <c r="B22">
-        <v>400000000</v>
-      </c>
-      <c r="C22">
-        <v>0</v>
-      </c>
-      <c r="D22">
-        <v>-1</v>
-      </c>
-      <c r="E22">
-        <v>-2</v>
-      </c>
-      <c r="F22">
-        <v>-4</v>
-      </c>
-      <c r="G22">
-        <v>-6</v>
-      </c>
-      <c r="H22">
-        <v>-8</v>
-      </c>
-      <c r="I22">
-        <v>-10</v>
-      </c>
-      <c r="J22">
-        <v>-20</v>
-      </c>
-      <c r="K22">
-        <v>-30</v>
-      </c>
-    </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A23" t="s">
-        <v>337</v>
-      </c>
-      <c r="B23">
-        <v>0</v>
-      </c>
-      <c r="C23">
-        <v>0</v>
-      </c>
-      <c r="D23">
-        <v>0</v>
-      </c>
-      <c r="E23">
-        <v>0</v>
-      </c>
-      <c r="F23">
-        <v>0</v>
-      </c>
-      <c r="G23">
-        <v>0</v>
-      </c>
-      <c r="H23">
-        <v>0</v>
-      </c>
-      <c r="I23">
-        <v>0</v>
-      </c>
-      <c r="J23">
-        <v>0</v>
-      </c>
-      <c r="K23">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A24" t="s">
-        <v>337</v>
-      </c>
-      <c r="B24" s="6">
-        <v>3600000</v>
-      </c>
-      <c r="C24">
-        <v>0</v>
-      </c>
-      <c r="D24">
-        <v>-1</v>
-      </c>
-      <c r="E24">
-        <v>-2</v>
-      </c>
-      <c r="F24">
-        <v>-4</v>
-      </c>
-      <c r="G24">
-        <v>-6</v>
-      </c>
-      <c r="H24">
-        <v>-8</v>
-      </c>
-      <c r="I24">
-        <v>-10</v>
-      </c>
-      <c r="J24">
-        <v>-20</v>
-      </c>
-      <c r="K24">
-        <v>-30</v>
-      </c>
-    </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A25" t="s">
-        <v>337</v>
-      </c>
-      <c r="B25">
-        <v>400000000</v>
-      </c>
-      <c r="C25">
-        <v>0</v>
-      </c>
-      <c r="D25">
-        <v>-1</v>
-      </c>
-      <c r="E25">
-        <v>-2</v>
-      </c>
-      <c r="F25">
-        <v>-4</v>
-      </c>
-      <c r="G25">
-        <v>-6</v>
-      </c>
-      <c r="H25">
-        <v>-8</v>
-      </c>
-      <c r="I25">
-        <v>-10</v>
-      </c>
-      <c r="J25">
-        <v>-20</v>
-      </c>
-      <c r="K25">
-        <v>-30</v>
-      </c>
-    </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A26" t="s">
-        <v>338</v>
-      </c>
-      <c r="B26">
-        <v>0</v>
-      </c>
-      <c r="C26">
-        <v>0</v>
-      </c>
-      <c r="D26">
-        <v>0</v>
-      </c>
-      <c r="E26">
-        <v>0</v>
-      </c>
-      <c r="F26">
-        <v>0</v>
-      </c>
-      <c r="G26">
-        <v>0</v>
-      </c>
-      <c r="H26">
-        <v>0</v>
-      </c>
-      <c r="I26">
-        <v>0</v>
-      </c>
-      <c r="J26">
-        <v>0</v>
-      </c>
-      <c r="K26">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A27" t="s">
-        <v>338</v>
-      </c>
-      <c r="B27" s="6">
-        <v>3600000</v>
-      </c>
-      <c r="C27">
-        <v>0</v>
-      </c>
-      <c r="D27">
-        <v>-1</v>
-      </c>
-      <c r="E27">
-        <v>-2</v>
-      </c>
-      <c r="F27">
-        <v>-4</v>
-      </c>
-      <c r="G27">
-        <v>-6</v>
-      </c>
-      <c r="H27">
-        <v>-8</v>
-      </c>
-      <c r="I27">
-        <v>-10</v>
-      </c>
-      <c r="J27">
-        <v>-20</v>
-      </c>
-      <c r="K27">
-        <v>-30</v>
-      </c>
-    </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A28" t="s">
-        <v>338</v>
-      </c>
-      <c r="B28">
-        <v>400000000</v>
-      </c>
-      <c r="C28">
-        <v>0</v>
-      </c>
-      <c r="D28">
-        <v>-1</v>
-      </c>
-      <c r="E28">
-        <v>-2</v>
-      </c>
-      <c r="F28">
-        <v>-4</v>
-      </c>
-      <c r="G28">
-        <v>-6</v>
-      </c>
-      <c r="H28">
-        <v>-8</v>
-      </c>
-      <c r="I28">
-        <v>-10</v>
-      </c>
-      <c r="J28">
-        <v>-20</v>
-      </c>
-      <c r="K28">
-        <v>-30</v>
-      </c>
+    <row r="18" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B18" s="6"/>
+    </row>
+    <row r="21" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B21" s="6"/>
+    </row>
+    <row r="24" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B24" s="6"/>
+    </row>
+    <row r="27" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B27" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Add right files to assets for 2D and 3D cases: 2D uses zone budgets, 3D uses csv files with different packages
</commit_message>
<xml_diff>
--- a/setup.xlsx
+++ b/setup.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cmarinriver\Projects\ConfinedLab\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8003329C-1995-40ED-BA0D-098451C1DA7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{018E0D94-7410-4978-BC62-6014EF51136D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7200" yWindow="4178" windowWidth="21600" windowHeight="11422" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2205" yWindow="2205" windowWidth="21600" windowHeight="11475" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="grid" sheetId="1" r:id="rId1"/>
@@ -23074,7 +23074,7 @@
         <v>71</v>
       </c>
       <c r="B17" s="1">
-        <v>1E-4</v>
+        <v>1.0000000000000001E-5</v>
       </c>
       <c r="C17">
         <v>9.0000000000000002E-6</v>
@@ -23100,7 +23100,7 @@
         <v>72</v>
       </c>
       <c r="B18" s="1">
-        <v>1E-4</v>
+        <v>1.0000000000000001E-5</v>
       </c>
       <c r="C18">
         <v>9.0000000000000002E-6</v>
@@ -23126,7 +23126,7 @@
         <v>73</v>
       </c>
       <c r="B19" s="1">
-        <v>1E-4</v>
+        <v>1.0000000000000001E-5</v>
       </c>
       <c r="C19">
         <v>9.0000000000000002E-6</v>
@@ -23152,7 +23152,7 @@
         <v>74</v>
       </c>
       <c r="B20" s="1">
-        <v>1E-4</v>
+        <v>1.0000000000000001E-5</v>
       </c>
       <c r="C20">
         <v>9.0000000000000002E-6</v>
@@ -23178,7 +23178,7 @@
         <v>75</v>
       </c>
       <c r="B21" s="1">
-        <v>1E-4</v>
+        <v>1.0000000000000001E-5</v>
       </c>
       <c r="C21">
         <v>9.0000000000000002E-6</v>
@@ -28066,7 +28066,7 @@
       <c r="E2">
         <v>400</v>
       </c>
-      <c r="F2">
+      <c r="F2" s="4">
         <v>0</v>
       </c>
     </row>
@@ -28087,7 +28087,7 @@
         <v>400</v>
       </c>
       <c r="F3" s="4">
-        <v>0</v>
+        <v>-0.02</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.45">
@@ -28107,7 +28107,7 @@
         <v>400</v>
       </c>
       <c r="F4" s="4">
-        <v>0</v>
+        <v>-0.02</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.45">
@@ -28147,7 +28147,7 @@
         <v>399</v>
       </c>
       <c r="F6" s="4">
-        <v>0</v>
+        <v>-0.02</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.45">
@@ -28167,7 +28167,7 @@
         <v>399</v>
       </c>
       <c r="F7" s="4">
-        <v>0</v>
+        <v>-0.02</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.45">
@@ -28207,7 +28207,7 @@
         <v>401</v>
       </c>
       <c r="F9" s="4">
-        <v>0</v>
+        <v>-0.02</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.45">
@@ -28227,7 +28227,7 @@
         <v>401</v>
       </c>
       <c r="F10" s="4">
-        <v>0</v>
+        <v>-0.02</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.45">
@@ -28267,7 +28267,7 @@
         <v>402</v>
       </c>
       <c r="F12" s="4">
-        <v>0</v>
+        <v>-0.02</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.45">
@@ -28287,7 +28287,7 @@
         <v>402</v>
       </c>
       <c r="F13" s="4">
-        <v>0</v>
+        <v>-0.02</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.45">
@@ -28327,7 +28327,7 @@
         <v>398</v>
       </c>
       <c r="F15" s="4">
-        <v>0</v>
+        <v>-0.02</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.45">
@@ -28347,7 +28347,7 @@
         <v>398</v>
       </c>
       <c r="F16" s="4">
-        <v>0</v>
+        <v>-0.02</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Control run for case kv 1E-13 and kh 1e-3 m/day
</commit_message>
<xml_diff>
--- a/setup.xlsx
+++ b/setup.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cmarinriver\Projects\ConfinedLab\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{566D8907-7F27-48FB-83A0-CB2391BF6ED7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C894EEF-4FCA-4C26-ACA8-FCE6993622AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14168" yWindow="2107" windowWidth="21599" windowHeight="11423" firstSheet="9" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15796" firstSheet="3" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="grid" sheetId="1" r:id="rId1"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2459" uniqueCount="1191">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2443" uniqueCount="1192">
   <si>
     <t>nlay</t>
   </si>
@@ -3570,9 +3570,6 @@
     <t>Run01</t>
   </si>
   <si>
-    <t>Run02</t>
-  </si>
-  <si>
     <t>kv_1E-12_kh_1E-07</t>
   </si>
   <si>
@@ -3619,6 +3616,12 @@
   </si>
   <si>
     <t>Run03</t>
+  </si>
+  <si>
+    <t>Run02.1</t>
+  </si>
+  <si>
+    <t>Run02.2</t>
   </si>
 </sst>
 </file>
@@ -3675,18 +3678,12 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="3">
@@ -3732,7 +3729,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -3759,9 +3756,6 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="11" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="11" fontId="6" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="11" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
@@ -5229,65 +5223,27 @@
         <v>43</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>1180</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>1181</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>1182</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>1183</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>1184</v>
-      </c>
-      <c r="G1" s="19" t="s">
-        <v>1163</v>
-      </c>
-      <c r="H1" s="19" t="s">
-        <v>1164</v>
-      </c>
-      <c r="I1" s="19" t="s">
-        <v>1165</v>
-      </c>
-      <c r="J1" s="19" t="s">
-        <v>1166</v>
-      </c>
-      <c r="K1" s="19" t="s">
-        <v>1167</v>
-      </c>
-      <c r="L1" s="4" t="s">
-        <v>1185</v>
-      </c>
-      <c r="M1" s="4" t="s">
-        <v>1186</v>
-      </c>
-      <c r="N1" s="4" t="s">
-        <v>1187</v>
-      </c>
-      <c r="O1" s="4" t="s">
-        <v>1188</v>
-      </c>
-      <c r="P1" s="4" t="s">
-        <v>1189</v>
-      </c>
-      <c r="Q1" s="19" t="s">
-        <v>1168</v>
-      </c>
-      <c r="R1" s="19" t="s">
-        <v>1169</v>
-      </c>
-      <c r="S1" s="19" t="s">
-        <v>1170</v>
-      </c>
-      <c r="T1" s="19" t="s">
-        <v>1171</v>
-      </c>
-      <c r="U1" s="19" t="s">
-        <v>1172</v>
-      </c>
+        <v>1157</v>
+      </c>
+      <c r="C1" s="4"/>
+      <c r="D1" s="4"/>
+      <c r="E1" s="4"/>
+      <c r="F1" s="4"/>
+      <c r="G1" s="16"/>
+      <c r="H1" s="16"/>
+      <c r="I1" s="16"/>
+      <c r="J1" s="16"/>
+      <c r="K1" s="16"/>
+      <c r="L1" s="4"/>
+      <c r="M1" s="4"/>
+      <c r="N1" s="4"/>
+      <c r="O1" s="4"/>
+      <c r="P1" s="4"/>
+      <c r="Q1" s="16"/>
+      <c r="R1" s="16"/>
+      <c r="S1" s="16"/>
+      <c r="T1" s="16"/>
+      <c r="U1" s="16"/>
       <c r="V1" s="4"/>
       <c r="W1" s="4"/>
       <c r="X1" s="4"/>
@@ -5314,65 +5270,27 @@
         <v>50</v>
       </c>
       <c r="B2" s="1">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="C2" s="1">
-        <v>8.6400000000000005E-2</v>
-      </c>
-      <c r="D2" s="1">
-        <v>0.86399999999999999</v>
-      </c>
-      <c r="E2" s="1">
-        <v>8.64</v>
-      </c>
-      <c r="F2" s="1">
         <v>86.4</v>
       </c>
-      <c r="G2" s="20">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="H2" s="20">
-        <v>8.6400000000000005E-2</v>
-      </c>
-      <c r="I2" s="20">
-        <v>0.86399999999999999</v>
-      </c>
-      <c r="J2" s="20">
-        <v>8.64</v>
-      </c>
-      <c r="K2" s="20">
-        <v>86.4</v>
-      </c>
-      <c r="L2" s="1">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="M2" s="1">
-        <v>8.6400000000000005E-2</v>
-      </c>
-      <c r="N2" s="1">
-        <v>0.86399999999999999</v>
-      </c>
-      <c r="O2" s="1">
-        <v>8.64</v>
-      </c>
-      <c r="P2" s="1">
-        <v>86.4</v>
-      </c>
-      <c r="Q2" s="20">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="R2" s="20">
-        <v>8.6400000000000005E-2</v>
-      </c>
-      <c r="S2" s="20">
-        <v>0.86399999999999999</v>
-      </c>
-      <c r="T2" s="20">
-        <v>8.64</v>
-      </c>
-      <c r="U2" s="20">
-        <v>86.4</v>
-      </c>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+      <c r="G2" s="17"/>
+      <c r="H2" s="17"/>
+      <c r="I2" s="17"/>
+      <c r="J2" s="17"/>
+      <c r="K2" s="17"/>
+      <c r="L2" s="1"/>
+      <c r="M2" s="1"/>
+      <c r="N2" s="1"/>
+      <c r="O2" s="1"/>
+      <c r="P2" s="1"/>
+      <c r="Q2" s="17"/>
+      <c r="R2" s="17"/>
+      <c r="S2" s="17"/>
+      <c r="T2" s="17"/>
+      <c r="U2" s="17"/>
       <c r="V2" s="1"/>
       <c r="W2" s="1"/>
       <c r="X2" s="1"/>
@@ -5399,65 +5317,27 @@
         <v>54</v>
       </c>
       <c r="B3" s="13">
-        <v>8.6400000000000003E-6</v>
-      </c>
-      <c r="C3" s="13">
-        <v>8.6400000000000003E-6</v>
-      </c>
-      <c r="D3" s="13">
-        <v>8.6400000000000003E-6</v>
-      </c>
-      <c r="E3" s="13">
-        <v>8.6400000000000003E-6</v>
-      </c>
-      <c r="F3" s="13">
-        <v>8.6400000000000003E-6</v>
-      </c>
-      <c r="G3" s="21">
-        <v>8.6399999999999999E-5</v>
-      </c>
-      <c r="H3" s="21">
-        <v>8.6399999999999999E-5</v>
-      </c>
-      <c r="I3" s="21">
-        <v>8.6399999999999999E-5</v>
-      </c>
-      <c r="J3" s="21">
-        <v>8.6399999999999999E-5</v>
-      </c>
-      <c r="K3" s="21">
-        <v>8.6399999999999999E-5</v>
-      </c>
-      <c r="L3" s="13">
-        <v>8.6399999999999997E-4</v>
-      </c>
-      <c r="M3" s="13">
-        <v>8.6399999999999997E-4</v>
-      </c>
-      <c r="N3" s="13">
-        <v>8.6399999999999997E-4</v>
-      </c>
-      <c r="O3" s="13">
-        <v>8.6399999999999997E-4</v>
-      </c>
-      <c r="P3" s="13">
-        <v>8.6399999999999997E-4</v>
-      </c>
-      <c r="Q3" s="21">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="R3" s="21">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="S3" s="21">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="T3" s="21">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="U3" s="21">
-        <v>8.6400000000000001E-3</v>
-      </c>
+        <v>8.6399999999999999E-9</v>
+      </c>
+      <c r="C3" s="15"/>
+      <c r="D3" s="13"/>
+      <c r="E3" s="13"/>
+      <c r="F3" s="13"/>
+      <c r="G3" s="18"/>
+      <c r="H3" s="18"/>
+      <c r="I3" s="18"/>
+      <c r="J3" s="18"/>
+      <c r="K3" s="18"/>
+      <c r="L3" s="13"/>
+      <c r="M3" s="13"/>
+      <c r="N3" s="13"/>
+      <c r="O3" s="13"/>
+      <c r="P3" s="13"/>
+      <c r="Q3" s="18"/>
+      <c r="R3" s="18"/>
+      <c r="S3" s="18"/>
+      <c r="T3" s="18"/>
+      <c r="U3" s="18"/>
       <c r="V3" s="13"/>
       <c r="W3" s="13"/>
       <c r="X3" s="13"/>
@@ -5484,65 +5364,27 @@
         <v>56</v>
       </c>
       <c r="B4" s="1">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="C4" s="1">
-        <v>8.6400000000000005E-2</v>
-      </c>
-      <c r="D4" s="1">
-        <v>0.86399999999999999</v>
-      </c>
-      <c r="E4" s="1">
-        <v>8.64</v>
-      </c>
-      <c r="F4" s="1">
         <v>86.4</v>
       </c>
-      <c r="G4" s="20">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="H4" s="20">
-        <v>8.6400000000000005E-2</v>
-      </c>
-      <c r="I4" s="20">
-        <v>0.86399999999999999</v>
-      </c>
-      <c r="J4" s="20">
-        <v>8.64</v>
-      </c>
-      <c r="K4" s="20">
-        <v>86.4</v>
-      </c>
-      <c r="L4" s="1">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="M4" s="1">
-        <v>8.6400000000000005E-2</v>
-      </c>
-      <c r="N4" s="1">
-        <v>0.86399999999999999</v>
-      </c>
-      <c r="O4" s="1">
-        <v>8.64</v>
-      </c>
-      <c r="P4" s="1">
-        <v>86.4</v>
-      </c>
-      <c r="Q4" s="20">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="R4" s="20">
-        <v>8.6400000000000005E-2</v>
-      </c>
-      <c r="S4" s="20">
-        <v>0.86399999999999999</v>
-      </c>
-      <c r="T4" s="20">
-        <v>8.64</v>
-      </c>
-      <c r="U4" s="20">
-        <v>86.4</v>
-      </c>
+      <c r="C4" s="1"/>
+      <c r="D4" s="1"/>
+      <c r="E4" s="1"/>
+      <c r="F4" s="1"/>
+      <c r="G4" s="17"/>
+      <c r="H4" s="17"/>
+      <c r="I4" s="17"/>
+      <c r="J4" s="17"/>
+      <c r="K4" s="17"/>
+      <c r="L4" s="1"/>
+      <c r="M4" s="1"/>
+      <c r="N4" s="1"/>
+      <c r="O4" s="1"/>
+      <c r="P4" s="1"/>
+      <c r="Q4" s="17"/>
+      <c r="R4" s="17"/>
+      <c r="S4" s="17"/>
+      <c r="T4" s="17"/>
+      <c r="U4" s="17"/>
       <c r="V4" s="1"/>
       <c r="W4" s="1"/>
       <c r="X4" s="1"/>
@@ -5569,65 +5411,27 @@
         <v>58</v>
       </c>
       <c r="B5" s="13">
-        <v>8.6400000000000003E-6</v>
-      </c>
-      <c r="C5" s="13">
-        <v>8.6400000000000003E-6</v>
-      </c>
-      <c r="D5" s="13">
-        <v>8.6400000000000003E-6</v>
-      </c>
-      <c r="E5" s="13">
-        <v>8.6400000000000003E-6</v>
-      </c>
-      <c r="F5" s="13">
-        <v>8.6400000000000003E-6</v>
-      </c>
-      <c r="G5" s="21">
-        <v>8.6399999999999999E-5</v>
-      </c>
-      <c r="H5" s="21">
-        <v>8.6399999999999999E-5</v>
-      </c>
-      <c r="I5" s="21">
-        <v>8.6399999999999999E-5</v>
-      </c>
-      <c r="J5" s="21">
-        <v>8.6399999999999999E-5</v>
-      </c>
-      <c r="K5" s="21">
-        <v>8.6399999999999999E-5</v>
-      </c>
-      <c r="L5" s="13">
-        <v>8.6399999999999997E-4</v>
-      </c>
-      <c r="M5" s="13">
-        <v>8.6399999999999997E-4</v>
-      </c>
-      <c r="N5" s="13">
-        <v>8.6399999999999997E-4</v>
-      </c>
-      <c r="O5" s="13">
-        <v>8.6399999999999997E-4</v>
-      </c>
-      <c r="P5" s="13">
-        <v>8.6399999999999997E-4</v>
-      </c>
-      <c r="Q5" s="21">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="R5" s="21">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="S5" s="21">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="T5" s="21">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="U5" s="21">
-        <v>8.6400000000000001E-3</v>
-      </c>
+        <v>8.6399999999999999E-9</v>
+      </c>
+      <c r="C5" s="15"/>
+      <c r="D5" s="13"/>
+      <c r="E5" s="13"/>
+      <c r="F5" s="13"/>
+      <c r="G5" s="18"/>
+      <c r="H5" s="18"/>
+      <c r="I5" s="18"/>
+      <c r="J5" s="18"/>
+      <c r="K5" s="18"/>
+      <c r="L5" s="13"/>
+      <c r="M5" s="13"/>
+      <c r="N5" s="13"/>
+      <c r="O5" s="13"/>
+      <c r="P5" s="13"/>
+      <c r="Q5" s="18"/>
+      <c r="R5" s="18"/>
+      <c r="S5" s="18"/>
+      <c r="T5" s="18"/>
+      <c r="U5" s="18"/>
       <c r="V5" s="13"/>
       <c r="W5" s="13"/>
       <c r="X5" s="13"/>
@@ -5654,65 +5458,27 @@
         <v>60</v>
       </c>
       <c r="B6" s="1">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="C6" s="1">
-        <v>8.6400000000000005E-2</v>
-      </c>
-      <c r="D6" s="1">
-        <v>0.86399999999999999</v>
-      </c>
-      <c r="E6" s="1">
-        <v>8.64</v>
-      </c>
-      <c r="F6" s="1">
         <v>86.4</v>
       </c>
-      <c r="G6" s="20">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="H6" s="20">
-        <v>8.6400000000000005E-2</v>
-      </c>
-      <c r="I6" s="20">
-        <v>0.86399999999999999</v>
-      </c>
-      <c r="J6" s="20">
-        <v>8.64</v>
-      </c>
-      <c r="K6" s="20">
-        <v>86.4</v>
-      </c>
-      <c r="L6" s="1">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="M6" s="1">
-        <v>8.6400000000000005E-2</v>
-      </c>
-      <c r="N6" s="1">
-        <v>0.86399999999999999</v>
-      </c>
-      <c r="O6" s="1">
-        <v>8.64</v>
-      </c>
-      <c r="P6" s="1">
-        <v>86.4</v>
-      </c>
-      <c r="Q6" s="20">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="R6" s="20">
-        <v>8.6400000000000005E-2</v>
-      </c>
-      <c r="S6" s="20">
-        <v>0.86399999999999999</v>
-      </c>
-      <c r="T6" s="20">
-        <v>8.64</v>
-      </c>
-      <c r="U6" s="20">
-        <v>86.4</v>
-      </c>
+      <c r="C6" s="1"/>
+      <c r="D6" s="1"/>
+      <c r="E6" s="1"/>
+      <c r="F6" s="1"/>
+      <c r="G6" s="17"/>
+      <c r="H6" s="17"/>
+      <c r="I6" s="17"/>
+      <c r="J6" s="17"/>
+      <c r="K6" s="17"/>
+      <c r="L6" s="1"/>
+      <c r="M6" s="1"/>
+      <c r="N6" s="1"/>
+      <c r="O6" s="1"/>
+      <c r="P6" s="1"/>
+      <c r="Q6" s="17"/>
+      <c r="R6" s="17"/>
+      <c r="S6" s="17"/>
+      <c r="T6" s="17"/>
+      <c r="U6" s="17"/>
       <c r="V6" s="1"/>
       <c r="W6" s="1"/>
       <c r="X6" s="1"/>
@@ -5739,65 +5505,27 @@
         <v>62</v>
       </c>
       <c r="B7" s="1">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="C7" s="1">
-        <v>8.6400000000000005E-2</v>
-      </c>
-      <c r="D7" s="1">
-        <v>0.86399999999999999</v>
-      </c>
-      <c r="E7" s="1">
-        <v>8.64</v>
-      </c>
-      <c r="F7" s="1">
         <v>86.4</v>
       </c>
-      <c r="G7" s="20">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="H7" s="20">
-        <v>8.6400000000000005E-2</v>
-      </c>
-      <c r="I7" s="20">
-        <v>0.86399999999999999</v>
-      </c>
-      <c r="J7" s="20">
-        <v>8.64</v>
-      </c>
-      <c r="K7" s="20">
-        <v>86.4</v>
-      </c>
-      <c r="L7" s="1">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="M7" s="1">
-        <v>8.6400000000000005E-2</v>
-      </c>
-      <c r="N7" s="1">
-        <v>0.86399999999999999</v>
-      </c>
-      <c r="O7" s="1">
-        <v>8.64</v>
-      </c>
-      <c r="P7" s="1">
-        <v>86.4</v>
-      </c>
-      <c r="Q7" s="20">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="R7" s="20">
-        <v>8.6400000000000005E-2</v>
-      </c>
-      <c r="S7" s="20">
-        <v>0.86399999999999999</v>
-      </c>
-      <c r="T7" s="20">
-        <v>8.64</v>
-      </c>
-      <c r="U7" s="20">
-        <v>86.4</v>
-      </c>
+      <c r="C7" s="1"/>
+      <c r="D7" s="1"/>
+      <c r="E7" s="1"/>
+      <c r="F7" s="1"/>
+      <c r="G7" s="17"/>
+      <c r="H7" s="17"/>
+      <c r="I7" s="17"/>
+      <c r="J7" s="17"/>
+      <c r="K7" s="17"/>
+      <c r="L7" s="1"/>
+      <c r="M7" s="1"/>
+      <c r="N7" s="1"/>
+      <c r="O7" s="1"/>
+      <c r="P7" s="1"/>
+      <c r="Q7" s="17"/>
+      <c r="R7" s="17"/>
+      <c r="S7" s="17"/>
+      <c r="T7" s="17"/>
+      <c r="U7" s="17"/>
       <c r="V7" s="1"/>
       <c r="W7" s="1"/>
       <c r="X7" s="1"/>
@@ -5824,65 +5552,27 @@
         <v>63</v>
       </c>
       <c r="B8" s="13">
-        <v>8.6400000000000003E-6</v>
-      </c>
-      <c r="C8" s="13">
-        <v>8.6400000000000003E-6</v>
-      </c>
-      <c r="D8" s="13">
-        <v>8.6400000000000003E-6</v>
-      </c>
-      <c r="E8" s="13">
-        <v>8.6400000000000003E-6</v>
-      </c>
-      <c r="F8" s="13">
-        <v>8.6400000000000003E-6</v>
-      </c>
-      <c r="G8" s="21">
-        <v>8.6399999999999999E-5</v>
-      </c>
-      <c r="H8" s="21">
-        <v>8.6399999999999999E-5</v>
-      </c>
-      <c r="I8" s="21">
-        <v>8.6399999999999999E-5</v>
-      </c>
-      <c r="J8" s="21">
-        <v>8.6399999999999999E-5</v>
-      </c>
-      <c r="K8" s="21">
-        <v>8.6399999999999999E-5</v>
-      </c>
-      <c r="L8" s="13">
-        <v>8.6399999999999997E-4</v>
-      </c>
-      <c r="M8" s="13">
-        <v>8.6399999999999997E-4</v>
-      </c>
-      <c r="N8" s="13">
-        <v>8.6399999999999997E-4</v>
-      </c>
-      <c r="O8" s="13">
-        <v>8.6399999999999997E-4</v>
-      </c>
-      <c r="P8" s="13">
-        <v>8.6399999999999997E-4</v>
-      </c>
-      <c r="Q8" s="21">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="R8" s="21">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="S8" s="21">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="T8" s="21">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="U8" s="21">
-        <v>8.6400000000000001E-3</v>
-      </c>
+        <v>8.6399999999999999E-9</v>
+      </c>
+      <c r="C8" s="15"/>
+      <c r="D8" s="13"/>
+      <c r="E8" s="13"/>
+      <c r="F8" s="13"/>
+      <c r="G8" s="18"/>
+      <c r="H8" s="18"/>
+      <c r="I8" s="18"/>
+      <c r="J8" s="18"/>
+      <c r="K8" s="18"/>
+      <c r="L8" s="13"/>
+      <c r="M8" s="13"/>
+      <c r="N8" s="13"/>
+      <c r="O8" s="13"/>
+      <c r="P8" s="13"/>
+      <c r="Q8" s="18"/>
+      <c r="R8" s="18"/>
+      <c r="S8" s="18"/>
+      <c r="T8" s="18"/>
+      <c r="U8" s="18"/>
       <c r="V8" s="13"/>
       <c r="W8" s="13"/>
       <c r="X8" s="13"/>
@@ -5909,65 +5599,27 @@
         <v>64</v>
       </c>
       <c r="B9" s="1">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="C9" s="1">
-        <v>8.6400000000000005E-2</v>
-      </c>
-      <c r="D9" s="1">
-        <v>0.86399999999999999</v>
-      </c>
-      <c r="E9" s="1">
-        <v>8.64</v>
-      </c>
-      <c r="F9" s="1">
         <v>86.4</v>
       </c>
-      <c r="G9" s="20">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="H9" s="20">
-        <v>8.6400000000000005E-2</v>
-      </c>
-      <c r="I9" s="20">
-        <v>0.86399999999999999</v>
-      </c>
-      <c r="J9" s="20">
-        <v>8.64</v>
-      </c>
-      <c r="K9" s="20">
-        <v>86.4</v>
-      </c>
-      <c r="L9" s="1">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="M9" s="1">
-        <v>8.6400000000000005E-2</v>
-      </c>
-      <c r="N9" s="1">
-        <v>0.86399999999999999</v>
-      </c>
-      <c r="O9" s="1">
-        <v>8.64</v>
-      </c>
-      <c r="P9" s="1">
-        <v>86.4</v>
-      </c>
-      <c r="Q9" s="20">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="R9" s="20">
-        <v>8.6400000000000005E-2</v>
-      </c>
-      <c r="S9" s="20">
-        <v>0.86399999999999999</v>
-      </c>
-      <c r="T9" s="20">
-        <v>8.64</v>
-      </c>
-      <c r="U9" s="20">
-        <v>86.4</v>
-      </c>
+      <c r="C9" s="1"/>
+      <c r="D9" s="1"/>
+      <c r="E9" s="1"/>
+      <c r="F9" s="1"/>
+      <c r="G9" s="17"/>
+      <c r="H9" s="17"/>
+      <c r="I9" s="17"/>
+      <c r="J9" s="17"/>
+      <c r="K9" s="17"/>
+      <c r="L9" s="1"/>
+      <c r="M9" s="1"/>
+      <c r="N9" s="1"/>
+      <c r="O9" s="1"/>
+      <c r="P9" s="1"/>
+      <c r="Q9" s="17"/>
+      <c r="R9" s="17"/>
+      <c r="S9" s="17"/>
+      <c r="T9" s="17"/>
+      <c r="U9" s="17"/>
       <c r="V9" s="1"/>
       <c r="W9" s="1"/>
       <c r="X9" s="1"/>
@@ -5994,65 +5646,27 @@
         <v>65</v>
       </c>
       <c r="B10" s="13">
-        <v>8.6400000000000003E-6</v>
-      </c>
-      <c r="C10" s="13">
-        <v>8.6400000000000003E-6</v>
-      </c>
-      <c r="D10" s="13">
-        <v>8.6400000000000003E-6</v>
-      </c>
-      <c r="E10" s="13">
-        <v>8.6400000000000003E-6</v>
-      </c>
-      <c r="F10" s="13">
-        <v>8.6400000000000003E-6</v>
-      </c>
-      <c r="G10" s="21">
-        <v>8.6399999999999999E-5</v>
-      </c>
-      <c r="H10" s="21">
-        <v>8.6399999999999999E-5</v>
-      </c>
-      <c r="I10" s="21">
-        <v>8.6399999999999999E-5</v>
-      </c>
-      <c r="J10" s="21">
-        <v>8.6399999999999999E-5</v>
-      </c>
-      <c r="K10" s="21">
-        <v>8.6399999999999999E-5</v>
-      </c>
-      <c r="L10" s="13">
-        <v>8.6399999999999997E-4</v>
-      </c>
-      <c r="M10" s="13">
-        <v>8.6399999999999997E-4</v>
-      </c>
-      <c r="N10" s="13">
-        <v>8.6399999999999997E-4</v>
-      </c>
-      <c r="O10" s="13">
-        <v>8.6399999999999997E-4</v>
-      </c>
-      <c r="P10" s="13">
-        <v>8.6399999999999997E-4</v>
-      </c>
-      <c r="Q10" s="21">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="R10" s="21">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="S10" s="21">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="T10" s="21">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="U10" s="21">
-        <v>8.6400000000000001E-3</v>
-      </c>
+        <v>8.6399999999999999E-9</v>
+      </c>
+      <c r="C10" s="15"/>
+      <c r="D10" s="13"/>
+      <c r="E10" s="13"/>
+      <c r="F10" s="13"/>
+      <c r="G10" s="18"/>
+      <c r="H10" s="18"/>
+      <c r="I10" s="18"/>
+      <c r="J10" s="18"/>
+      <c r="K10" s="18"/>
+      <c r="L10" s="13"/>
+      <c r="M10" s="13"/>
+      <c r="N10" s="13"/>
+      <c r="O10" s="13"/>
+      <c r="P10" s="13"/>
+      <c r="Q10" s="18"/>
+      <c r="R10" s="18"/>
+      <c r="S10" s="18"/>
+      <c r="T10" s="18"/>
+      <c r="U10" s="18"/>
       <c r="V10" s="13"/>
       <c r="W10" s="13"/>
       <c r="X10" s="13"/>
@@ -6079,65 +5693,27 @@
         <v>66</v>
       </c>
       <c r="B11" s="1">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="C11" s="1">
-        <v>8.6400000000000005E-2</v>
-      </c>
-      <c r="D11" s="1">
-        <v>0.86399999999999999</v>
-      </c>
-      <c r="E11" s="1">
-        <v>8.64</v>
-      </c>
-      <c r="F11" s="1">
         <v>86.4</v>
       </c>
-      <c r="G11" s="20">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="H11" s="20">
-        <v>8.6400000000000005E-2</v>
-      </c>
-      <c r="I11" s="20">
-        <v>0.86399999999999999</v>
-      </c>
-      <c r="J11" s="20">
-        <v>8.64</v>
-      </c>
-      <c r="K11" s="20">
-        <v>86.4</v>
-      </c>
-      <c r="L11" s="1">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="M11" s="1">
-        <v>8.6400000000000005E-2</v>
-      </c>
-      <c r="N11" s="1">
-        <v>0.86399999999999999</v>
-      </c>
-      <c r="O11" s="1">
-        <v>8.64</v>
-      </c>
-      <c r="P11" s="1">
-        <v>86.4</v>
-      </c>
-      <c r="Q11" s="20">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="R11" s="20">
-        <v>8.6400000000000005E-2</v>
-      </c>
-      <c r="S11" s="20">
-        <v>0.86399999999999999</v>
-      </c>
-      <c r="T11" s="20">
-        <v>8.64</v>
-      </c>
-      <c r="U11" s="20">
-        <v>86.4</v>
-      </c>
+      <c r="C11" s="1"/>
+      <c r="D11" s="1"/>
+      <c r="E11" s="1"/>
+      <c r="F11" s="1"/>
+      <c r="G11" s="17"/>
+      <c r="H11" s="17"/>
+      <c r="I11" s="17"/>
+      <c r="J11" s="17"/>
+      <c r="K11" s="17"/>
+      <c r="L11" s="1"/>
+      <c r="M11" s="1"/>
+      <c r="N11" s="1"/>
+      <c r="O11" s="1"/>
+      <c r="P11" s="1"/>
+      <c r="Q11" s="17"/>
+      <c r="R11" s="17"/>
+      <c r="S11" s="17"/>
+      <c r="T11" s="17"/>
+      <c r="U11" s="17"/>
       <c r="V11" s="1"/>
       <c r="W11" s="1"/>
       <c r="X11" s="1"/>
@@ -6648,6 +6224,7 @@
   <cols>
     <col min="1" max="1" width="15.46484375" style="4" bestFit="1" customWidth="1"/>
     <col min="32" max="32" width="18.59765625" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="27.19921875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:37" x14ac:dyDescent="0.45">
@@ -13454,63 +13031,33 @@
         <v>43</v>
       </c>
       <c r="AF91" s="16" t="s">
-        <v>1153</v>
+        <v>1163</v>
       </c>
       <c r="AG91" s="16" t="s">
-        <v>1154</v>
+        <v>1164</v>
       </c>
       <c r="AH91" s="16" t="s">
-        <v>1155</v>
+        <v>1165</v>
       </c>
       <c r="AI91" s="16" t="s">
-        <v>1156</v>
+        <v>1166</v>
       </c>
       <c r="AJ91" s="16" t="s">
-        <v>1157</v>
+        <v>1167</v>
       </c>
       <c r="AK91" s="16" t="s">
-        <v>1158</v>
+        <v>1168</v>
       </c>
       <c r="AL91" s="16" t="s">
-        <v>1159</v>
+        <v>1169</v>
       </c>
       <c r="AM91" s="16" t="s">
-        <v>1160</v>
+        <v>1170</v>
       </c>
       <c r="AN91" s="16" t="s">
-        <v>1161</v>
+        <v>1171</v>
       </c>
       <c r="AO91" s="16" t="s">
-        <v>1162</v>
-      </c>
-      <c r="AP91" s="19" t="s">
-        <v>1163</v>
-      </c>
-      <c r="AQ91" s="19" t="s">
-        <v>1164</v>
-      </c>
-      <c r="AR91" s="19" t="s">
-        <v>1165</v>
-      </c>
-      <c r="AS91" s="19" t="s">
-        <v>1166</v>
-      </c>
-      <c r="AT91" s="19" t="s">
-        <v>1167</v>
-      </c>
-      <c r="AU91" s="19" t="s">
-        <v>1168</v>
-      </c>
-      <c r="AV91" s="19" t="s">
-        <v>1169</v>
-      </c>
-      <c r="AW91" s="19" t="s">
-        <v>1170</v>
-      </c>
-      <c r="AX91" s="19" t="s">
-        <v>1171</v>
-      </c>
-      <c r="AY91" s="19" t="s">
         <v>1172</v>
       </c>
       <c r="BN91" s="4" t="s">
@@ -13639,36 +13186,6 @@
       <c r="AO92" s="17">
         <v>86.4</v>
       </c>
-      <c r="AP92" s="20">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="AQ92" s="20">
-        <v>8.6400000000000005E-2</v>
-      </c>
-      <c r="AR92" s="20">
-        <v>0.86399999999999999</v>
-      </c>
-      <c r="AS92" s="20">
-        <v>8.64</v>
-      </c>
-      <c r="AT92" s="20">
-        <v>86.4</v>
-      </c>
-      <c r="AU92" s="20">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="AV92" s="20">
-        <v>8.6400000000000005E-2</v>
-      </c>
-      <c r="AW92" s="20">
-        <v>0.86399999999999999</v>
-      </c>
-      <c r="AX92" s="20">
-        <v>8.64</v>
-      </c>
-      <c r="AY92" s="20">
-        <v>86.4</v>
-      </c>
       <c r="BN92" s="4" t="s">
         <v>93</v>
       </c>
@@ -13766,63 +13283,33 @@
         <v>54</v>
       </c>
       <c r="AF93" s="18">
-        <v>8.6399999999999999E-9</v>
+        <v>8.6399999999999999E-5</v>
       </c>
       <c r="AG93" s="18">
-        <v>8.6399999999999999E-9</v>
+        <v>8.6399999999999999E-5</v>
       </c>
       <c r="AH93" s="18">
-        <v>8.6399999999999999E-9</v>
+        <v>8.6399999999999999E-5</v>
       </c>
       <c r="AI93" s="18">
-        <v>8.6399999999999999E-9</v>
+        <v>8.6399999999999999E-5</v>
       </c>
       <c r="AJ93" s="18">
-        <v>8.6399999999999999E-9</v>
+        <v>8.6399999999999999E-5</v>
       </c>
       <c r="AK93" s="18">
-        <v>8.6400000000000001E-7</v>
+        <v>8.6400000000000001E-3</v>
       </c>
       <c r="AL93" s="18">
-        <v>8.6400000000000001E-7</v>
+        <v>8.6400000000000001E-3</v>
       </c>
       <c r="AM93" s="18">
-        <v>8.6400000000000001E-7</v>
+        <v>8.6400000000000001E-3</v>
       </c>
       <c r="AN93" s="18">
-        <v>8.6400000000000001E-7</v>
+        <v>8.6400000000000001E-3</v>
       </c>
       <c r="AO93" s="18">
-        <v>8.6400000000000001E-7</v>
-      </c>
-      <c r="AP93" s="21">
-        <v>8.6399999999999999E-5</v>
-      </c>
-      <c r="AQ93" s="21">
-        <v>8.6399999999999999E-5</v>
-      </c>
-      <c r="AR93" s="21">
-        <v>8.6399999999999999E-5</v>
-      </c>
-      <c r="AS93" s="21">
-        <v>8.6399999999999999E-5</v>
-      </c>
-      <c r="AT93" s="21">
-        <v>8.6399999999999999E-5</v>
-      </c>
-      <c r="AU93" s="21">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="AV93" s="21">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="AW93" s="21">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="AX93" s="21">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="AY93" s="21">
         <v>8.6400000000000001E-3</v>
       </c>
       <c r="BN93" s="4" t="s">
@@ -13951,36 +13438,6 @@
       <c r="AO94" s="17">
         <v>86.4</v>
       </c>
-      <c r="AP94" s="20">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="AQ94" s="20">
-        <v>8.6400000000000005E-2</v>
-      </c>
-      <c r="AR94" s="20">
-        <v>0.86399999999999999</v>
-      </c>
-      <c r="AS94" s="20">
-        <v>8.64</v>
-      </c>
-      <c r="AT94" s="20">
-        <v>86.4</v>
-      </c>
-      <c r="AU94" s="20">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="AV94" s="20">
-        <v>8.6400000000000005E-2</v>
-      </c>
-      <c r="AW94" s="20">
-        <v>0.86399999999999999</v>
-      </c>
-      <c r="AX94" s="20">
-        <v>8.64</v>
-      </c>
-      <c r="AY94" s="20">
-        <v>86.4</v>
-      </c>
       <c r="BN94" s="4" t="s">
         <v>94</v>
       </c>
@@ -14078,63 +13535,33 @@
         <v>58</v>
       </c>
       <c r="AF95" s="18">
-        <v>8.6399999999999999E-9</v>
+        <v>8.6399999999999999E-5</v>
       </c>
       <c r="AG95" s="18">
-        <v>8.6399999999999999E-9</v>
+        <v>8.6399999999999999E-5</v>
       </c>
       <c r="AH95" s="18">
-        <v>8.6399999999999999E-9</v>
+        <v>8.6399999999999999E-5</v>
       </c>
       <c r="AI95" s="18">
-        <v>8.6399999999999999E-9</v>
+        <v>8.6399999999999999E-5</v>
       </c>
       <c r="AJ95" s="18">
-        <v>8.6399999999999999E-9</v>
+        <v>8.6399999999999999E-5</v>
       </c>
       <c r="AK95" s="18">
-        <v>8.6400000000000001E-7</v>
+        <v>8.6400000000000001E-3</v>
       </c>
       <c r="AL95" s="18">
-        <v>8.6400000000000001E-7</v>
+        <v>8.6400000000000001E-3</v>
       </c>
       <c r="AM95" s="18">
-        <v>8.6400000000000001E-7</v>
+        <v>8.6400000000000001E-3</v>
       </c>
       <c r="AN95" s="18">
-        <v>8.6400000000000001E-7</v>
+        <v>8.6400000000000001E-3</v>
       </c>
       <c r="AO95" s="18">
-        <v>8.6400000000000001E-7</v>
-      </c>
-      <c r="AP95" s="21">
-        <v>8.6399999999999999E-5</v>
-      </c>
-      <c r="AQ95" s="21">
-        <v>8.6399999999999999E-5</v>
-      </c>
-      <c r="AR95" s="21">
-        <v>8.6399999999999999E-5</v>
-      </c>
-      <c r="AS95" s="21">
-        <v>8.6399999999999999E-5</v>
-      </c>
-      <c r="AT95" s="21">
-        <v>8.6399999999999999E-5</v>
-      </c>
-      <c r="AU95" s="21">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="AV95" s="21">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="AW95" s="21">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="AX95" s="21">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="AY95" s="21">
         <v>8.6400000000000001E-3</v>
       </c>
       <c r="BN95" s="4" t="s">
@@ -14263,36 +13690,6 @@
       <c r="AO96" s="17">
         <v>86.4</v>
       </c>
-      <c r="AP96" s="20">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="AQ96" s="20">
-        <v>8.6400000000000005E-2</v>
-      </c>
-      <c r="AR96" s="20">
-        <v>0.86399999999999999</v>
-      </c>
-      <c r="AS96" s="20">
-        <v>8.64</v>
-      </c>
-      <c r="AT96" s="20">
-        <v>86.4</v>
-      </c>
-      <c r="AU96" s="20">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="AV96" s="20">
-        <v>8.6400000000000005E-2</v>
-      </c>
-      <c r="AW96" s="20">
-        <v>0.86399999999999999</v>
-      </c>
-      <c r="AX96" s="20">
-        <v>8.64</v>
-      </c>
-      <c r="AY96" s="20">
-        <v>86.4</v>
-      </c>
       <c r="BN96" s="4" t="s">
         <v>94</v>
       </c>
@@ -14419,36 +13816,6 @@
       <c r="AO97" s="17">
         <v>86.4</v>
       </c>
-      <c r="AP97" s="20">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="AQ97" s="20">
-        <v>8.6400000000000005E-2</v>
-      </c>
-      <c r="AR97" s="20">
-        <v>0.86399999999999999</v>
-      </c>
-      <c r="AS97" s="20">
-        <v>8.64</v>
-      </c>
-      <c r="AT97" s="20">
-        <v>86.4</v>
-      </c>
-      <c r="AU97" s="20">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="AV97" s="20">
-        <v>8.6400000000000005E-2</v>
-      </c>
-      <c r="AW97" s="20">
-        <v>0.86399999999999999</v>
-      </c>
-      <c r="AX97" s="20">
-        <v>8.64</v>
-      </c>
-      <c r="AY97" s="20">
-        <v>86.4</v>
-      </c>
       <c r="BN97" s="4" t="s">
         <v>95</v>
       </c>
@@ -14546,63 +13913,33 @@
         <v>63</v>
       </c>
       <c r="AF98" s="18">
-        <v>8.6399999999999999E-9</v>
+        <v>8.6399999999999999E-5</v>
       </c>
       <c r="AG98" s="18">
-        <v>8.6399999999999999E-9</v>
+        <v>8.6399999999999999E-5</v>
       </c>
       <c r="AH98" s="18">
-        <v>8.6399999999999999E-9</v>
+        <v>8.6399999999999999E-5</v>
       </c>
       <c r="AI98" s="18">
-        <v>8.6399999999999999E-9</v>
+        <v>8.6399999999999999E-5</v>
       </c>
       <c r="AJ98" s="18">
-        <v>8.6399999999999999E-9</v>
+        <v>8.6399999999999999E-5</v>
       </c>
       <c r="AK98" s="18">
-        <v>8.6400000000000001E-7</v>
+        <v>8.6400000000000001E-3</v>
       </c>
       <c r="AL98" s="18">
-        <v>8.6400000000000001E-7</v>
+        <v>8.6400000000000001E-3</v>
       </c>
       <c r="AM98" s="18">
-        <v>8.6400000000000001E-7</v>
+        <v>8.6400000000000001E-3</v>
       </c>
       <c r="AN98" s="18">
-        <v>8.6400000000000001E-7</v>
+        <v>8.6400000000000001E-3</v>
       </c>
       <c r="AO98" s="18">
-        <v>8.6400000000000001E-7</v>
-      </c>
-      <c r="AP98" s="21">
-        <v>8.6399999999999999E-5</v>
-      </c>
-      <c r="AQ98" s="21">
-        <v>8.6399999999999999E-5</v>
-      </c>
-      <c r="AR98" s="21">
-        <v>8.6399999999999999E-5</v>
-      </c>
-      <c r="AS98" s="21">
-        <v>8.6399999999999999E-5</v>
-      </c>
-      <c r="AT98" s="21">
-        <v>8.6399999999999999E-5</v>
-      </c>
-      <c r="AU98" s="21">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="AV98" s="21">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="AW98" s="21">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="AX98" s="21">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="AY98" s="21">
         <v>8.6400000000000001E-3</v>
       </c>
       <c r="BN98" s="4" t="s">
@@ -14731,36 +14068,6 @@
       <c r="AO99" s="17">
         <v>86.4</v>
       </c>
-      <c r="AP99" s="20">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="AQ99" s="20">
-        <v>8.6400000000000005E-2</v>
-      </c>
-      <c r="AR99" s="20">
-        <v>0.86399999999999999</v>
-      </c>
-      <c r="AS99" s="20">
-        <v>8.64</v>
-      </c>
-      <c r="AT99" s="20">
-        <v>86.4</v>
-      </c>
-      <c r="AU99" s="20">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="AV99" s="20">
-        <v>8.6400000000000005E-2</v>
-      </c>
-      <c r="AW99" s="20">
-        <v>0.86399999999999999</v>
-      </c>
-      <c r="AX99" s="20">
-        <v>8.64</v>
-      </c>
-      <c r="AY99" s="20">
-        <v>86.4</v>
-      </c>
       <c r="BN99" s="4" t="s">
         <v>95</v>
       </c>
@@ -14858,63 +14165,33 @@
         <v>65</v>
       </c>
       <c r="AF100" s="18">
-        <v>8.6399999999999999E-9</v>
+        <v>8.6399999999999999E-5</v>
       </c>
       <c r="AG100" s="18">
-        <v>8.6399999999999999E-9</v>
+        <v>8.6399999999999999E-5</v>
       </c>
       <c r="AH100" s="18">
-        <v>8.6399999999999999E-9</v>
+        <v>8.6399999999999999E-5</v>
       </c>
       <c r="AI100" s="18">
-        <v>8.6399999999999999E-9</v>
+        <v>8.6399999999999999E-5</v>
       </c>
       <c r="AJ100" s="18">
-        <v>8.6399999999999999E-9</v>
+        <v>8.6399999999999999E-5</v>
       </c>
       <c r="AK100" s="18">
-        <v>8.6400000000000001E-7</v>
+        <v>8.6400000000000001E-3</v>
       </c>
       <c r="AL100" s="18">
-        <v>8.6400000000000001E-7</v>
+        <v>8.6400000000000001E-3</v>
       </c>
       <c r="AM100" s="18">
-        <v>8.6400000000000001E-7</v>
+        <v>8.6400000000000001E-3</v>
       </c>
       <c r="AN100" s="18">
-        <v>8.6400000000000001E-7</v>
+        <v>8.6400000000000001E-3</v>
       </c>
       <c r="AO100" s="18">
-        <v>8.6400000000000001E-7</v>
-      </c>
-      <c r="AP100" s="21">
-        <v>8.6399999999999999E-5</v>
-      </c>
-      <c r="AQ100" s="21">
-        <v>8.6399999999999999E-5</v>
-      </c>
-      <c r="AR100" s="21">
-        <v>8.6399999999999999E-5</v>
-      </c>
-      <c r="AS100" s="21">
-        <v>8.6399999999999999E-5</v>
-      </c>
-      <c r="AT100" s="21">
-        <v>8.6399999999999999E-5</v>
-      </c>
-      <c r="AU100" s="21">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="AV100" s="21">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="AW100" s="21">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="AX100" s="21">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="AY100" s="21">
         <v>8.6400000000000001E-3</v>
       </c>
       <c r="BN100" s="4" t="s">
@@ -15043,36 +14320,6 @@
       <c r="AO101" s="17">
         <v>86.4</v>
       </c>
-      <c r="AP101" s="20">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="AQ101" s="20">
-        <v>8.6400000000000005E-2</v>
-      </c>
-      <c r="AR101" s="20">
-        <v>0.86399999999999999</v>
-      </c>
-      <c r="AS101" s="20">
-        <v>8.64</v>
-      </c>
-      <c r="AT101" s="20">
-        <v>86.4</v>
-      </c>
-      <c r="AU101" s="20">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="AV101" s="20">
-        <v>8.6400000000000005E-2</v>
-      </c>
-      <c r="AW101" s="20">
-        <v>0.86399999999999999</v>
-      </c>
-      <c r="AX101" s="20">
-        <v>8.64</v>
-      </c>
-      <c r="AY101" s="20">
-        <v>86.4</v>
-      </c>
       <c r="BN101" s="4" t="s">
         <v>96</v>
       </c>
@@ -15260,7 +14507,7 @@
         <v>6.1373542849109256E-4</v>
       </c>
       <c r="AE103" s="14" t="s">
-        <v>1174</v>
+        <v>1190</v>
       </c>
       <c r="BN103" s="4" t="s">
         <v>97</v>
@@ -15374,19 +14621,19 @@
         <v>1157</v>
       </c>
       <c r="AK104" s="4" t="s">
+        <v>1174</v>
+      </c>
+      <c r="AL104" s="4" t="s">
         <v>1175</v>
       </c>
-      <c r="AL104" s="4" t="s">
+      <c r="AM104" s="4" t="s">
         <v>1176</v>
       </c>
-      <c r="AM104" s="4" t="s">
+      <c r="AN104" s="4" t="s">
         <v>1177</v>
       </c>
-      <c r="AN104" s="4" t="s">
+      <c r="AO104" s="4" t="s">
         <v>1178</v>
-      </c>
-      <c r="AO104" s="4" t="s">
-        <v>1179</v>
       </c>
       <c r="AP104" s="4" t="s">
         <v>1158</v>
@@ -15890,7 +15137,7 @@
         <v>8.6400000000000001E-7</v>
       </c>
       <c r="BN108" t="s">
-        <v>1174</v>
+        <v>1190</v>
       </c>
     </row>
     <row r="109" spans="1:78" x14ac:dyDescent="0.45">
@@ -16886,7 +16133,7 @@
         <v>9.0184342071178349E-4</v>
       </c>
       <c r="AE116" s="14" t="s">
-        <v>1190</v>
+        <v>1191</v>
       </c>
       <c r="AF116" s="4"/>
       <c r="AG116" s="4"/>
@@ -16990,63 +16237,63 @@
         <v>43</v>
       </c>
       <c r="AF117" s="4" t="s">
+        <v>1179</v>
+      </c>
+      <c r="AG117" s="4" t="s">
         <v>1180</v>
       </c>
-      <c r="AG117" s="4" t="s">
+      <c r="AH117" s="4" t="s">
         <v>1181</v>
       </c>
-      <c r="AH117" s="4" t="s">
+      <c r="AI117" s="4" t="s">
         <v>1182</v>
       </c>
-      <c r="AI117" s="4" t="s">
+      <c r="AJ117" s="4" t="s">
         <v>1183</v>
       </c>
-      <c r="AJ117" s="4" t="s">
+      <c r="AK117" s="16" t="s">
+        <v>1163</v>
+      </c>
+      <c r="AL117" s="16" t="s">
+        <v>1164</v>
+      </c>
+      <c r="AM117" s="16" t="s">
+        <v>1165</v>
+      </c>
+      <c r="AN117" s="16" t="s">
+        <v>1166</v>
+      </c>
+      <c r="AO117" s="16" t="s">
+        <v>1167</v>
+      </c>
+      <c r="AP117" s="4" t="s">
         <v>1184</v>
       </c>
-      <c r="AK117" s="19" t="s">
-        <v>1163</v>
-      </c>
-      <c r="AL117" s="19" t="s">
-        <v>1164</v>
-      </c>
-      <c r="AM117" s="19" t="s">
-        <v>1165</v>
-      </c>
-      <c r="AN117" s="19" t="s">
-        <v>1166</v>
-      </c>
-      <c r="AO117" s="19" t="s">
-        <v>1167</v>
-      </c>
-      <c r="AP117" s="4" t="s">
+      <c r="AQ117" s="4" t="s">
         <v>1185</v>
       </c>
-      <c r="AQ117" s="4" t="s">
+      <c r="AR117" s="4" t="s">
         <v>1186</v>
       </c>
-      <c r="AR117" s="4" t="s">
+      <c r="AS117" s="4" t="s">
         <v>1187</v>
       </c>
-      <c r="AS117" s="4" t="s">
+      <c r="AT117" s="4" t="s">
         <v>1188</v>
       </c>
-      <c r="AT117" s="4" t="s">
-        <v>1189</v>
-      </c>
-      <c r="AU117" s="19" t="s">
+      <c r="AU117" s="16" t="s">
         <v>1168</v>
       </c>
-      <c r="AV117" s="19" t="s">
+      <c r="AV117" s="16" t="s">
         <v>1169</v>
       </c>
-      <c r="AW117" s="19" t="s">
+      <c r="AW117" s="16" t="s">
         <v>1170</v>
       </c>
-      <c r="AX117" s="19" t="s">
+      <c r="AX117" s="16" t="s">
         <v>1171</v>
       </c>
-      <c r="AY117" s="19" t="s">
+      <c r="AY117" s="16" t="s">
         <v>1172</v>
       </c>
       <c r="AZ117" s="4"/>
@@ -17165,19 +16412,19 @@
       <c r="AJ118" s="1">
         <v>86.4</v>
       </c>
-      <c r="AK118" s="20">
+      <c r="AK118" s="17">
         <v>8.6400000000000001E-3</v>
       </c>
-      <c r="AL118" s="20">
+      <c r="AL118" s="17">
         <v>8.6400000000000005E-2</v>
       </c>
-      <c r="AM118" s="20">
+      <c r="AM118" s="17">
         <v>0.86399999999999999</v>
       </c>
-      <c r="AN118" s="20">
+      <c r="AN118" s="17">
         <v>8.64</v>
       </c>
-      <c r="AO118" s="20">
+      <c r="AO118" s="17">
         <v>86.4</v>
       </c>
       <c r="AP118" s="1">
@@ -17195,19 +16442,19 @@
       <c r="AT118" s="1">
         <v>86.4</v>
       </c>
-      <c r="AU118" s="20">
+      <c r="AU118" s="17">
         <v>8.6400000000000001E-3</v>
       </c>
-      <c r="AV118" s="20">
+      <c r="AV118" s="17">
         <v>8.6400000000000005E-2</v>
       </c>
-      <c r="AW118" s="20">
+      <c r="AW118" s="17">
         <v>0.86399999999999999</v>
       </c>
-      <c r="AX118" s="20">
+      <c r="AX118" s="17">
         <v>8.64</v>
       </c>
-      <c r="AY118" s="20">
+      <c r="AY118" s="17">
         <v>86.4</v>
       </c>
       <c r="AZ118" s="1"/>
@@ -17326,19 +16573,19 @@
       <c r="AJ119" s="13">
         <v>8.6400000000000003E-6</v>
       </c>
-      <c r="AK119" s="21">
+      <c r="AK119" s="18">
         <v>8.6399999999999999E-5</v>
       </c>
-      <c r="AL119" s="21">
+      <c r="AL119" s="18">
         <v>8.6399999999999999E-5</v>
       </c>
-      <c r="AM119" s="21">
+      <c r="AM119" s="18">
         <v>8.6399999999999999E-5</v>
       </c>
-      <c r="AN119" s="21">
+      <c r="AN119" s="18">
         <v>8.6399999999999999E-5</v>
       </c>
-      <c r="AO119" s="21">
+      <c r="AO119" s="18">
         <v>8.6399999999999999E-5</v>
       </c>
       <c r="AP119" s="13">
@@ -17356,19 +16603,19 @@
       <c r="AT119" s="13">
         <v>8.6399999999999997E-4</v>
       </c>
-      <c r="AU119" s="21">
+      <c r="AU119" s="18">
         <v>8.6400000000000001E-3</v>
       </c>
-      <c r="AV119" s="21">
+      <c r="AV119" s="18">
         <v>8.6400000000000001E-3</v>
       </c>
-      <c r="AW119" s="21">
+      <c r="AW119" s="18">
         <v>8.6400000000000001E-3</v>
       </c>
-      <c r="AX119" s="21">
+      <c r="AX119" s="18">
         <v>8.6400000000000001E-3</v>
       </c>
-      <c r="AY119" s="21">
+      <c r="AY119" s="18">
         <v>8.6400000000000001E-3</v>
       </c>
       <c r="AZ119" s="13"/>
@@ -17487,19 +16734,19 @@
       <c r="AJ120" s="1">
         <v>86.4</v>
       </c>
-      <c r="AK120" s="20">
+      <c r="AK120" s="17">
         <v>8.6400000000000001E-3</v>
       </c>
-      <c r="AL120" s="20">
+      <c r="AL120" s="17">
         <v>8.6400000000000005E-2</v>
       </c>
-      <c r="AM120" s="20">
+      <c r="AM120" s="17">
         <v>0.86399999999999999</v>
       </c>
-      <c r="AN120" s="20">
+      <c r="AN120" s="17">
         <v>8.64</v>
       </c>
-      <c r="AO120" s="20">
+      <c r="AO120" s="17">
         <v>86.4</v>
       </c>
       <c r="AP120" s="1">
@@ -17517,19 +16764,19 @@
       <c r="AT120" s="1">
         <v>86.4</v>
       </c>
-      <c r="AU120" s="20">
+      <c r="AU120" s="17">
         <v>8.6400000000000001E-3</v>
       </c>
-      <c r="AV120" s="20">
+      <c r="AV120" s="17">
         <v>8.6400000000000005E-2</v>
       </c>
-      <c r="AW120" s="20">
+      <c r="AW120" s="17">
         <v>0.86399999999999999</v>
       </c>
-      <c r="AX120" s="20">
+      <c r="AX120" s="17">
         <v>8.64</v>
       </c>
-      <c r="AY120" s="20">
+      <c r="AY120" s="17">
         <v>86.4</v>
       </c>
       <c r="AZ120" s="1"/>
@@ -17648,19 +16895,19 @@
       <c r="AJ121" s="13">
         <v>8.6400000000000003E-6</v>
       </c>
-      <c r="AK121" s="21">
+      <c r="AK121" s="18">
         <v>8.6399999999999999E-5</v>
       </c>
-      <c r="AL121" s="21">
+      <c r="AL121" s="18">
         <v>8.6399999999999999E-5</v>
       </c>
-      <c r="AM121" s="21">
+      <c r="AM121" s="18">
         <v>8.6399999999999999E-5</v>
       </c>
-      <c r="AN121" s="21">
+      <c r="AN121" s="18">
         <v>8.6399999999999999E-5</v>
       </c>
-      <c r="AO121" s="21">
+      <c r="AO121" s="18">
         <v>8.6399999999999999E-5</v>
       </c>
       <c r="AP121" s="13">
@@ -17678,19 +16925,19 @@
       <c r="AT121" s="13">
         <v>8.6399999999999997E-4</v>
       </c>
-      <c r="AU121" s="21">
+      <c r="AU121" s="18">
         <v>8.6400000000000001E-3</v>
       </c>
-      <c r="AV121" s="21">
+      <c r="AV121" s="18">
         <v>8.6400000000000001E-3</v>
       </c>
-      <c r="AW121" s="21">
+      <c r="AW121" s="18">
         <v>8.6400000000000001E-3</v>
       </c>
-      <c r="AX121" s="21">
+      <c r="AX121" s="18">
         <v>8.6400000000000001E-3</v>
       </c>
-      <c r="AY121" s="21">
+      <c r="AY121" s="18">
         <v>8.6400000000000001E-3</v>
       </c>
       <c r="AZ121" s="13"/>
@@ -17809,19 +17056,19 @@
       <c r="AJ122" s="1">
         <v>86.4</v>
       </c>
-      <c r="AK122" s="20">
+      <c r="AK122" s="17">
         <v>8.6400000000000001E-3</v>
       </c>
-      <c r="AL122" s="20">
+      <c r="AL122" s="17">
         <v>8.6400000000000005E-2</v>
       </c>
-      <c r="AM122" s="20">
+      <c r="AM122" s="17">
         <v>0.86399999999999999</v>
       </c>
-      <c r="AN122" s="20">
+      <c r="AN122" s="17">
         <v>8.64</v>
       </c>
-      <c r="AO122" s="20">
+      <c r="AO122" s="17">
         <v>86.4</v>
       </c>
       <c r="AP122" s="1">
@@ -17839,19 +17086,19 @@
       <c r="AT122" s="1">
         <v>86.4</v>
       </c>
-      <c r="AU122" s="20">
+      <c r="AU122" s="17">
         <v>8.6400000000000001E-3</v>
       </c>
-      <c r="AV122" s="20">
+      <c r="AV122" s="17">
         <v>8.6400000000000005E-2</v>
       </c>
-      <c r="AW122" s="20">
+      <c r="AW122" s="17">
         <v>0.86399999999999999</v>
       </c>
-      <c r="AX122" s="20">
+      <c r="AX122" s="17">
         <v>8.64</v>
       </c>
-      <c r="AY122" s="20">
+      <c r="AY122" s="17">
         <v>86.4</v>
       </c>
       <c r="AZ122" s="1"/>
@@ -17970,19 +17217,19 @@
       <c r="AJ123" s="1">
         <v>86.4</v>
       </c>
-      <c r="AK123" s="20">
+      <c r="AK123" s="17">
         <v>8.6400000000000001E-3</v>
       </c>
-      <c r="AL123" s="20">
+      <c r="AL123" s="17">
         <v>8.6400000000000005E-2</v>
       </c>
-      <c r="AM123" s="20">
+      <c r="AM123" s="17">
         <v>0.86399999999999999</v>
       </c>
-      <c r="AN123" s="20">
+      <c r="AN123" s="17">
         <v>8.64</v>
       </c>
-      <c r="AO123" s="20">
+      <c r="AO123" s="17">
         <v>86.4</v>
       </c>
       <c r="AP123" s="1">
@@ -18000,19 +17247,19 @@
       <c r="AT123" s="1">
         <v>86.4</v>
       </c>
-      <c r="AU123" s="20">
+      <c r="AU123" s="17">
         <v>8.6400000000000001E-3</v>
       </c>
-      <c r="AV123" s="20">
+      <c r="AV123" s="17">
         <v>8.6400000000000005E-2</v>
       </c>
-      <c r="AW123" s="20">
+      <c r="AW123" s="17">
         <v>0.86399999999999999</v>
       </c>
-      <c r="AX123" s="20">
+      <c r="AX123" s="17">
         <v>8.64</v>
       </c>
-      <c r="AY123" s="20">
+      <c r="AY123" s="17">
         <v>86.4</v>
       </c>
       <c r="AZ123" s="1"/>
@@ -18131,19 +17378,19 @@
       <c r="AJ124" s="13">
         <v>8.6400000000000003E-6</v>
       </c>
-      <c r="AK124" s="21">
+      <c r="AK124" s="18">
         <v>8.6399999999999999E-5</v>
       </c>
-      <c r="AL124" s="21">
+      <c r="AL124" s="18">
         <v>8.6399999999999999E-5</v>
       </c>
-      <c r="AM124" s="21">
+      <c r="AM124" s="18">
         <v>8.6399999999999999E-5</v>
       </c>
-      <c r="AN124" s="21">
+      <c r="AN124" s="18">
         <v>8.6399999999999999E-5</v>
       </c>
-      <c r="AO124" s="21">
+      <c r="AO124" s="18">
         <v>8.6399999999999999E-5</v>
       </c>
       <c r="AP124" s="13">
@@ -18161,19 +17408,19 @@
       <c r="AT124" s="13">
         <v>8.6399999999999997E-4</v>
       </c>
-      <c r="AU124" s="21">
+      <c r="AU124" s="18">
         <v>8.6400000000000001E-3</v>
       </c>
-      <c r="AV124" s="21">
+      <c r="AV124" s="18">
         <v>8.6400000000000001E-3</v>
       </c>
-      <c r="AW124" s="21">
+      <c r="AW124" s="18">
         <v>8.6400000000000001E-3</v>
       </c>
-      <c r="AX124" s="21">
+      <c r="AX124" s="18">
         <v>8.6400000000000001E-3</v>
       </c>
-      <c r="AY124" s="21">
+      <c r="AY124" s="18">
         <v>8.6400000000000001E-3</v>
       </c>
       <c r="AZ124" s="13"/>
@@ -18292,19 +17539,19 @@
       <c r="AJ125" s="1">
         <v>86.4</v>
       </c>
-      <c r="AK125" s="20">
+      <c r="AK125" s="17">
         <v>8.6400000000000001E-3</v>
       </c>
-      <c r="AL125" s="20">
+      <c r="AL125" s="17">
         <v>8.6400000000000005E-2</v>
       </c>
-      <c r="AM125" s="20">
+      <c r="AM125" s="17">
         <v>0.86399999999999999</v>
       </c>
-      <c r="AN125" s="20">
+      <c r="AN125" s="17">
         <v>8.64</v>
       </c>
-      <c r="AO125" s="20">
+      <c r="AO125" s="17">
         <v>86.4</v>
       </c>
       <c r="AP125" s="1">
@@ -18322,19 +17569,19 @@
       <c r="AT125" s="1">
         <v>86.4</v>
       </c>
-      <c r="AU125" s="20">
+      <c r="AU125" s="17">
         <v>8.6400000000000001E-3</v>
       </c>
-      <c r="AV125" s="20">
+      <c r="AV125" s="17">
         <v>8.6400000000000005E-2</v>
       </c>
-      <c r="AW125" s="20">
+      <c r="AW125" s="17">
         <v>0.86399999999999999</v>
       </c>
-      <c r="AX125" s="20">
+      <c r="AX125" s="17">
         <v>8.64</v>
       </c>
-      <c r="AY125" s="20">
+      <c r="AY125" s="17">
         <v>86.4</v>
       </c>
       <c r="AZ125" s="1"/>
@@ -18414,19 +17661,19 @@
       <c r="AJ126" s="13">
         <v>8.6400000000000003E-6</v>
       </c>
-      <c r="AK126" s="21">
+      <c r="AK126" s="18">
         <v>8.6399999999999999E-5</v>
       </c>
-      <c r="AL126" s="21">
+      <c r="AL126" s="18">
         <v>8.6399999999999999E-5</v>
       </c>
-      <c r="AM126" s="21">
+      <c r="AM126" s="18">
         <v>8.6399999999999999E-5</v>
       </c>
-      <c r="AN126" s="21">
+      <c r="AN126" s="18">
         <v>8.6399999999999999E-5</v>
       </c>
-      <c r="AO126" s="21">
+      <c r="AO126" s="18">
         <v>8.6399999999999999E-5</v>
       </c>
       <c r="AP126" s="13">
@@ -18444,19 +17691,19 @@
       <c r="AT126" s="13">
         <v>8.6399999999999997E-4</v>
       </c>
-      <c r="AU126" s="21">
+      <c r="AU126" s="18">
         <v>8.6400000000000001E-3</v>
       </c>
-      <c r="AV126" s="21">
+      <c r="AV126" s="18">
         <v>8.6400000000000001E-3</v>
       </c>
-      <c r="AW126" s="21">
+      <c r="AW126" s="18">
         <v>8.6400000000000001E-3</v>
       </c>
-      <c r="AX126" s="21">
+      <c r="AX126" s="18">
         <v>8.6400000000000001E-3</v>
       </c>
-      <c r="AY126" s="21">
+      <c r="AY126" s="18">
         <v>8.6400000000000001E-3</v>
       </c>
       <c r="AZ126" s="13"/>
@@ -18536,19 +17783,19 @@
       <c r="AJ127" s="1">
         <v>86.4</v>
       </c>
-      <c r="AK127" s="20">
+      <c r="AK127" s="17">
         <v>8.6400000000000001E-3</v>
       </c>
-      <c r="AL127" s="20">
+      <c r="AL127" s="17">
         <v>8.6400000000000005E-2</v>
       </c>
-      <c r="AM127" s="20">
+      <c r="AM127" s="17">
         <v>0.86399999999999999</v>
       </c>
-      <c r="AN127" s="20">
+      <c r="AN127" s="17">
         <v>8.64</v>
       </c>
-      <c r="AO127" s="20">
+      <c r="AO127" s="17">
         <v>86.4</v>
       </c>
       <c r="AP127" s="1">
@@ -18566,19 +17813,19 @@
       <c r="AT127" s="1">
         <v>86.4</v>
       </c>
-      <c r="AU127" s="20">
+      <c r="AU127" s="17">
         <v>8.6400000000000001E-3</v>
       </c>
-      <c r="AV127" s="20">
+      <c r="AV127" s="17">
         <v>8.6400000000000005E-2</v>
       </c>
-      <c r="AW127" s="20">
+      <c r="AW127" s="17">
         <v>0.86399999999999999</v>
       </c>
-      <c r="AX127" s="20">
+      <c r="AX127" s="17">
         <v>8.64</v>
       </c>
-      <c r="AY127" s="20">
+      <c r="AY127" s="17">
         <v>86.4</v>
       </c>
       <c r="AZ127" s="1"/>
@@ -18587,7 +17834,7 @@
       <c r="BC127" s="1"/>
       <c r="BD127" s="1"/>
       <c r="BN127" t="s">
-        <v>1190</v>
+        <v>1191</v>
       </c>
     </row>
     <row r="128" spans="1:78" x14ac:dyDescent="0.45">
@@ -18731,6 +17978,9 @@
       <c r="AA129" s="1">
         <f t="shared" si="15"/>
         <v>6.7192904177343729E-4</v>
+      </c>
+      <c r="AE129" s="14" t="s">
+        <v>1189</v>
       </c>
       <c r="AF129" s="1"/>
       <c r="AG129" s="1"/>
@@ -18834,8 +18084,13 @@
         <f t="shared" ref="AA130:AA154" si="19">+W130</f>
         <v>6.8402164621609858E-4</v>
       </c>
-      <c r="AF130" s="1"/>
-      <c r="AG130" s="1"/>
+      <c r="AE130" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="AF130" s="4" t="s">
+        <v>1157</v>
+      </c>
+      <c r="AG130" s="4"/>
       <c r="AH130" s="1"/>
       <c r="AI130" s="1"/>
       <c r="AJ130" s="1"/>
@@ -18936,7 +18191,12 @@
         <f t="shared" si="19"/>
         <v>7.3510433221211555E-4</v>
       </c>
-      <c r="AF131" s="1"/>
+      <c r="AE131" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="AF131" s="1">
+        <v>86.4</v>
+      </c>
       <c r="AG131" s="1"/>
       <c r="AH131" s="1"/>
       <c r="AI131" s="1"/>
@@ -19038,6 +18298,13 @@
         <f t="shared" si="19"/>
         <v>6.8958168854050443E-4</v>
       </c>
+      <c r="AE132" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="AF132" s="13">
+        <v>8.6399999999999999E-9</v>
+      </c>
+      <c r="AG132" s="15"/>
       <c r="BN132" s="4" t="s">
         <v>94</v>
       </c>
@@ -19125,6 +18392,13 @@
         <f t="shared" si="19"/>
         <v>7.0175093423377206E-4</v>
       </c>
+      <c r="AE133" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="AF133" s="1">
+        <v>86.4</v>
+      </c>
+      <c r="AG133" s="1"/>
       <c r="BN133" s="4" t="s">
         <v>94</v>
       </c>
@@ -19212,6 +18486,13 @@
         <f t="shared" si="19"/>
         <v>9.24392529713391E-4</v>
       </c>
+      <c r="AE134" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="AF134" s="13">
+        <v>8.6399999999999999E-9</v>
+      </c>
+      <c r="AG134" s="15"/>
       <c r="BN134" s="4" t="s">
         <v>94</v>
       </c>
@@ -19299,6 +18580,13 @@
         <f t="shared" si="19"/>
         <v>4.2679489394130968E-4</v>
       </c>
+      <c r="AE135" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="AF135" s="1">
+        <v>86.4</v>
+      </c>
+      <c r="AG135" s="1"/>
       <c r="BN135" s="4" t="s">
         <v>95</v>
       </c>
@@ -19386,6 +18674,13 @@
         <f t="shared" si="19"/>
         <v>7.0492044974188462E-4</v>
       </c>
+      <c r="AE136" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="AF136" s="1">
+        <v>86.4</v>
+      </c>
+      <c r="AG136" s="1"/>
       <c r="BN136" s="4" t="s">
         <v>95</v>
       </c>
@@ -19473,6 +18768,13 @@
         <f t="shared" si="19"/>
         <v>6.0317831663807579E-4</v>
       </c>
+      <c r="AE137" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="AF137" s="13">
+        <v>8.6399999999999999E-9</v>
+      </c>
+      <c r="AG137" s="15"/>
       <c r="BN137" s="4" t="s">
         <v>95</v>
       </c>
@@ -19560,6 +18862,13 @@
         <f t="shared" si="19"/>
         <v>5.3431529879549361E-4</v>
       </c>
+      <c r="AE138" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="AF138" s="1">
+        <v>86.4</v>
+      </c>
+      <c r="AG138" s="1"/>
       <c r="BN138" s="4" t="s">
         <v>96</v>
       </c>
@@ -19647,6 +18956,13 @@
         <f t="shared" si="19"/>
         <v>9.2650687165257131E-4</v>
       </c>
+      <c r="AE139" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="AF139" s="13">
+        <v>8.6399999999999999E-9</v>
+      </c>
+      <c r="AG139" s="15"/>
       <c r="BN139" s="4" t="s">
         <v>96</v>
       </c>
@@ -19734,6 +19050,13 @@
         <f t="shared" si="19"/>
         <v>4.9093461376614072E-4</v>
       </c>
+      <c r="AE140" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="AF140" s="1">
+        <v>86.4</v>
+      </c>
+      <c r="AG140" s="1"/>
       <c r="BN140" s="4" t="s">
         <v>96</v>
       </c>

</xml_diff>

<commit_message>
Control run not converging. Doubled pumping rate
</commit_message>
<xml_diff>
--- a/setup.xlsx
+++ b/setup.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cmarinriver\Projects\ConfinedLab\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C894EEF-4FCA-4C26-ACA8-FCE6993622AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87682DB6-E830-4E8C-84C4-D2AEA9815CC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15796" firstSheet="3" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15796" firstSheet="3" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="grid" sheetId="1" r:id="rId1"/>
@@ -44650,7 +44650,7 @@
         <v>400</v>
       </c>
       <c r="F2" s="4">
-        <v>-50</v>
+        <v>-100</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.45">
@@ -44670,7 +44670,7 @@
         <v>399</v>
       </c>
       <c r="F3" s="4">
-        <v>-50</v>
+        <v>-100</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.45">
@@ -44690,7 +44690,7 @@
         <v>401</v>
       </c>
       <c r="F4" s="4">
-        <v>-50</v>
+        <v>-100</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.45">
@@ -44710,7 +44710,7 @@
         <v>402</v>
       </c>
       <c r="F5" s="4">
-        <v>-50</v>
+        <v>-100</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.45">
@@ -44730,7 +44730,7 @@
         <v>398</v>
       </c>
       <c r="F6" s="4">
-        <v>-50</v>
+        <v>-100</v>
       </c>
     </row>
   </sheetData>
@@ -44804,7 +44804,7 @@
         <v>400</v>
       </c>
       <c r="F3" s="4">
-        <v>-50</v>
+        <v>-100</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.45">
@@ -44824,7 +44824,7 @@
         <v>400</v>
       </c>
       <c r="F4" s="4">
-        <v>-50</v>
+        <v>-100</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.45">
@@ -44864,7 +44864,7 @@
         <v>399</v>
       </c>
       <c r="F6" s="4">
-        <v>-50</v>
+        <v>-100</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.45">
@@ -44884,7 +44884,7 @@
         <v>399</v>
       </c>
       <c r="F7" s="4">
-        <v>-50</v>
+        <v>-100</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.45">
@@ -44924,7 +44924,7 @@
         <v>401</v>
       </c>
       <c r="F9" s="4">
-        <v>-50</v>
+        <v>-100</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.45">
@@ -44944,7 +44944,7 @@
         <v>401</v>
       </c>
       <c r="F10" s="4">
-        <v>-50</v>
+        <v>-100</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.45">
@@ -44984,7 +44984,7 @@
         <v>402</v>
       </c>
       <c r="F12" s="4">
-        <v>-50</v>
+        <v>-100</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.45">
@@ -45004,7 +45004,7 @@
         <v>402</v>
       </c>
       <c r="F13" s="4">
-        <v>-50</v>
+        <v>-100</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.45">
@@ -45044,7 +45044,7 @@
         <v>398</v>
       </c>
       <c r="F15" s="4">
-        <v>-50</v>
+        <v>-100</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.45">
@@ -45064,7 +45064,7 @@
         <v>398</v>
       </c>
       <c r="F16" s="4">
-        <v>-50</v>
+        <v>-100</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Back to initial pumping rate. Decrease convergece criteria by one order of magnitude for control run
</commit_message>
<xml_diff>
--- a/setup.xlsx
+++ b/setup.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cmarinriver\Projects\ConfinedLab\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87682DB6-E830-4E8C-84C4-D2AEA9815CC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8506B43F-7934-46F8-A247-74182959C85A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15796" firstSheet="3" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15796" firstSheet="3" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="grid" sheetId="1" r:id="rId1"/>
@@ -44650,7 +44650,7 @@
         <v>400</v>
       </c>
       <c r="F2" s="4">
-        <v>-100</v>
+        <v>-50</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.45">
@@ -44670,7 +44670,7 @@
         <v>399</v>
       </c>
       <c r="F3" s="4">
-        <v>-100</v>
+        <v>-50</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.45">
@@ -44690,7 +44690,7 @@
         <v>401</v>
       </c>
       <c r="F4" s="4">
-        <v>-100</v>
+        <v>-50</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.45">
@@ -44710,7 +44710,7 @@
         <v>402</v>
       </c>
       <c r="F5" s="4">
-        <v>-100</v>
+        <v>-50</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.45">
@@ -44730,7 +44730,7 @@
         <v>398</v>
       </c>
       <c r="F6" s="4">
-        <v>-100</v>
+        <v>-50</v>
       </c>
     </row>
   </sheetData>
@@ -44741,13 +44741,13 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.06640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="12.265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A1" s="5" t="s">
         <v>91</v>
       </c>
@@ -44767,7 +44767,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>93</v>
       </c>
@@ -44786,8 +44786,9 @@
       <c r="F2" s="4">
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="G2" s="4"/>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>93</v>
       </c>
@@ -44804,10 +44805,11 @@
         <v>400</v>
       </c>
       <c r="F3" s="4">
-        <v>-100</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.45">
+        <v>-50</v>
+      </c>
+      <c r="G3" s="4"/>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>93</v>
       </c>
@@ -44824,10 +44826,11 @@
         <v>400</v>
       </c>
       <c r="F4" s="4">
-        <v>-100</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.45">
+        <v>-50</v>
+      </c>
+      <c r="G4" s="4"/>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>94</v>
       </c>
@@ -44846,8 +44849,9 @@
       <c r="F5" s="4">
         <v>0</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="G5" s="4"/>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>94</v>
       </c>
@@ -44864,10 +44868,11 @@
         <v>399</v>
       </c>
       <c r="F6" s="4">
-        <v>-100</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.45">
+        <v>-50</v>
+      </c>
+      <c r="G6" s="4"/>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>94</v>
       </c>
@@ -44884,10 +44889,11 @@
         <v>399</v>
       </c>
       <c r="F7" s="4">
-        <v>-100</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.45">
+        <v>-50</v>
+      </c>
+      <c r="G7" s="4"/>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>95</v>
       </c>
@@ -44906,8 +44912,9 @@
       <c r="F8" s="4">
         <v>0</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="G8" s="4"/>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>95</v>
       </c>
@@ -44924,10 +44931,11 @@
         <v>401</v>
       </c>
       <c r="F9" s="4">
-        <v>-100</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.45">
+        <v>-50</v>
+      </c>
+      <c r="G9" s="4"/>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
         <v>95</v>
       </c>
@@ -44944,10 +44952,11 @@
         <v>401</v>
       </c>
       <c r="F10" s="4">
-        <v>-100</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.45">
+        <v>-50</v>
+      </c>
+      <c r="G10" s="4"/>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
         <v>96</v>
       </c>
@@ -44966,8 +44975,9 @@
       <c r="F11" s="4">
         <v>0</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="G11" s="4"/>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
         <v>96</v>
       </c>
@@ -44984,10 +44994,11 @@
         <v>402</v>
       </c>
       <c r="F12" s="4">
-        <v>-100</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.45">
+        <v>-50</v>
+      </c>
+      <c r="G12" s="4"/>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
         <v>96</v>
       </c>
@@ -45004,10 +45015,11 @@
         <v>402</v>
       </c>
       <c r="F13" s="4">
-        <v>-100</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.45">
+        <v>-50</v>
+      </c>
+      <c r="G13" s="4"/>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
         <v>97</v>
       </c>
@@ -45026,8 +45038,9 @@
       <c r="F14" s="4">
         <v>0</v>
       </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="G14" s="4"/>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
         <v>97</v>
       </c>
@@ -45044,10 +45057,11 @@
         <v>398</v>
       </c>
       <c r="F15" s="4">
-        <v>-100</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.45">
+        <v>-50</v>
+      </c>
+      <c r="G15" s="4"/>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
         <v>97</v>
       </c>
@@ -45064,8 +45078,21 @@
         <v>398</v>
       </c>
       <c r="F16" s="4">
-        <v>-100</v>
-      </c>
+        <v>-50</v>
+      </c>
+      <c r="G16" s="4"/>
+    </row>
+    <row r="17" spans="7:7" x14ac:dyDescent="0.45">
+      <c r="G17" s="4"/>
+    </row>
+    <row r="18" spans="7:7" x14ac:dyDescent="0.45">
+      <c r="G18" s="4"/>
+    </row>
+    <row r="19" spans="7:7" x14ac:dyDescent="0.45">
+      <c r="G19" s="4"/>
+    </row>
+    <row r="20" spans="7:7" x14ac:dyDescent="0.45">
+      <c r="G20" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Change thin cells threshold for control run
</commit_message>
<xml_diff>
--- a/setup.xlsx
+++ b/setup.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cmarinriver\Projects\ConfinedLab\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8506B43F-7934-46F8-A247-74182959C85A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7D33F23-147F-4BEE-B880-E7460E9D6C69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15796" firstSheet="3" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5250" yWindow="2775" windowWidth="21600" windowHeight="11423" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="grid" sheetId="1" r:id="rId1"/>
@@ -26112,7 +26112,7 @@
         <v>70</v>
       </c>
       <c r="J2" s="4">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K2" s="4">
         <v>1</v>
@@ -26147,7 +26147,7 @@
         <v>70</v>
       </c>
       <c r="J3" s="4">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K3" s="4">
         <v>2</v>
@@ -26182,7 +26182,7 @@
         <v>70</v>
       </c>
       <c r="J4" s="4">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K4" s="4">
         <v>3</v>
@@ -26217,7 +26217,7 @@
         <v>70</v>
       </c>
       <c r="J5" s="4">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K5" s="4">
         <v>4</v>
@@ -26252,7 +26252,7 @@
         <v>70</v>
       </c>
       <c r="J6" s="4">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K6" s="4">
         <v>5</v>

</xml_diff>

<commit_message>
Set threshold for thin cells to Zero in control run
</commit_message>
<xml_diff>
--- a/setup.xlsx
+++ b/setup.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cmarinriver\Projects\ConfinedLab\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7D33F23-147F-4BEE-B880-E7460E9D6C69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{753F2932-83FD-44A0-88BD-B0C0188D58DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5250" yWindow="2775" windowWidth="21600" windowHeight="11423" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26112,7 +26112,7 @@
         <v>70</v>
       </c>
       <c r="J2" s="4">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K2" s="4">
         <v>1</v>
@@ -26147,7 +26147,7 @@
         <v>70</v>
       </c>
       <c r="J3" s="4">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K3" s="4">
         <v>2</v>
@@ -26182,7 +26182,7 @@
         <v>70</v>
       </c>
       <c r="J4" s="4">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K4" s="4">
         <v>3</v>
@@ -26217,7 +26217,7 @@
         <v>70</v>
       </c>
       <c r="J5" s="4">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K5" s="4">
         <v>4</v>
@@ -26252,7 +26252,7 @@
         <v>70</v>
       </c>
       <c r="J6" s="4">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K6" s="4">
         <v>5</v>

</xml_diff>

<commit_message>
Run 03 for kh 1e-3 and kv 1e-12/1e-13 m3/day
</commit_message>
<xml_diff>
--- a/setup.xlsx
+++ b/setup.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cmarinriver\Projects\ConfinedLab\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{753F2932-83FD-44A0-88BD-B0C0188D58DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC14C1F3-3894-466A-B410-8F6EE96B7693}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5250" yWindow="2775" windowWidth="21600" windowHeight="11423" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15796" firstSheet="6" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="grid" sheetId="1" r:id="rId1"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2443" uniqueCount="1192">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2445" uniqueCount="1192">
   <si>
     <t>nlay</t>
   </si>
@@ -5225,7 +5225,9 @@
       <c r="B1" s="4" t="s">
         <v>1157</v>
       </c>
-      <c r="C1" s="4"/>
+      <c r="C1" s="4" t="s">
+        <v>1178</v>
+      </c>
       <c r="D1" s="4"/>
       <c r="E1" s="4"/>
       <c r="F1" s="4"/>
@@ -5272,7 +5274,9 @@
       <c r="B2" s="1">
         <v>86.4</v>
       </c>
-      <c r="C2" s="1"/>
+      <c r="C2" s="1">
+        <v>86.4</v>
+      </c>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
@@ -5319,7 +5323,9 @@
       <c r="B3" s="13">
         <v>8.6399999999999999E-9</v>
       </c>
-      <c r="C3" s="15"/>
+      <c r="C3" s="15">
+        <v>8.6400000000000006E-8</v>
+      </c>
       <c r="D3" s="13"/>
       <c r="E3" s="13"/>
       <c r="F3" s="13"/>
@@ -5366,7 +5372,9 @@
       <c r="B4" s="1">
         <v>86.4</v>
       </c>
-      <c r="C4" s="1"/>
+      <c r="C4" s="1">
+        <v>86.4</v>
+      </c>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
       <c r="F4" s="1"/>
@@ -5413,7 +5421,9 @@
       <c r="B5" s="13">
         <v>8.6399999999999999E-9</v>
       </c>
-      <c r="C5" s="15"/>
+      <c r="C5" s="15">
+        <v>8.6400000000000006E-8</v>
+      </c>
       <c r="D5" s="13"/>
       <c r="E5" s="13"/>
       <c r="F5" s="13"/>
@@ -5460,7 +5470,9 @@
       <c r="B6" s="1">
         <v>86.4</v>
       </c>
-      <c r="C6" s="1"/>
+      <c r="C6" s="1">
+        <v>86.4</v>
+      </c>
       <c r="D6" s="1"/>
       <c r="E6" s="1"/>
       <c r="F6" s="1"/>
@@ -5507,7 +5519,9 @@
       <c r="B7" s="1">
         <v>86.4</v>
       </c>
-      <c r="C7" s="1"/>
+      <c r="C7" s="1">
+        <v>86.4</v>
+      </c>
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
       <c r="F7" s="1"/>
@@ -5554,7 +5568,9 @@
       <c r="B8" s="13">
         <v>8.6399999999999999E-9</v>
       </c>
-      <c r="C8" s="15"/>
+      <c r="C8" s="15">
+        <v>8.6400000000000006E-8</v>
+      </c>
       <c r="D8" s="13"/>
       <c r="E8" s="13"/>
       <c r="F8" s="13"/>
@@ -5601,7 +5617,9 @@
       <c r="B9" s="1">
         <v>86.4</v>
       </c>
-      <c r="C9" s="1"/>
+      <c r="C9" s="1">
+        <v>86.4</v>
+      </c>
       <c r="D9" s="1"/>
       <c r="E9" s="1"/>
       <c r="F9" s="1"/>
@@ -5648,7 +5666,9 @@
       <c r="B10" s="13">
         <v>8.6399999999999999E-9</v>
       </c>
-      <c r="C10" s="15"/>
+      <c r="C10" s="15">
+        <v>8.6400000000000006E-8</v>
+      </c>
       <c r="D10" s="13"/>
       <c r="E10" s="13"/>
       <c r="F10" s="13"/>
@@ -5695,7 +5715,9 @@
       <c r="B11" s="1">
         <v>86.4</v>
       </c>
-      <c r="C11" s="1"/>
+      <c r="C11" s="1">
+        <v>86.4</v>
+      </c>
       <c r="D11" s="1"/>
       <c r="E11" s="1"/>
       <c r="F11" s="1"/>
@@ -18090,7 +18112,9 @@
       <c r="AF130" s="4" t="s">
         <v>1157</v>
       </c>
-      <c r="AG130" s="4"/>
+      <c r="AG130" s="4" t="s">
+        <v>1178</v>
+      </c>
       <c r="AH130" s="1"/>
       <c r="AI130" s="1"/>
       <c r="AJ130" s="1"/>
@@ -18197,7 +18221,9 @@
       <c r="AF131" s="1">
         <v>86.4</v>
       </c>
-      <c r="AG131" s="1"/>
+      <c r="AG131" s="1">
+        <v>86.4</v>
+      </c>
       <c r="AH131" s="1"/>
       <c r="AI131" s="1"/>
       <c r="AJ131" s="1"/>
@@ -18304,7 +18330,9 @@
       <c r="AF132" s="13">
         <v>8.6399999999999999E-9</v>
       </c>
-      <c r="AG132" s="15"/>
+      <c r="AG132" s="15">
+        <v>8.6400000000000006E-8</v>
+      </c>
       <c r="BN132" s="4" t="s">
         <v>94</v>
       </c>
@@ -18398,7 +18426,9 @@
       <c r="AF133" s="1">
         <v>86.4</v>
       </c>
-      <c r="AG133" s="1"/>
+      <c r="AG133" s="1">
+        <v>86.4</v>
+      </c>
       <c r="BN133" s="4" t="s">
         <v>94</v>
       </c>
@@ -18492,7 +18522,9 @@
       <c r="AF134" s="13">
         <v>8.6399999999999999E-9</v>
       </c>
-      <c r="AG134" s="15"/>
+      <c r="AG134" s="15">
+        <v>8.6400000000000006E-8</v>
+      </c>
       <c r="BN134" s="4" t="s">
         <v>94</v>
       </c>
@@ -18586,7 +18618,9 @@
       <c r="AF135" s="1">
         <v>86.4</v>
       </c>
-      <c r="AG135" s="1"/>
+      <c r="AG135" s="1">
+        <v>86.4</v>
+      </c>
       <c r="BN135" s="4" t="s">
         <v>95</v>
       </c>
@@ -18680,7 +18714,9 @@
       <c r="AF136" s="1">
         <v>86.4</v>
       </c>
-      <c r="AG136" s="1"/>
+      <c r="AG136" s="1">
+        <v>86.4</v>
+      </c>
       <c r="BN136" s="4" t="s">
         <v>95</v>
       </c>
@@ -18774,7 +18810,9 @@
       <c r="AF137" s="13">
         <v>8.6399999999999999E-9</v>
       </c>
-      <c r="AG137" s="15"/>
+      <c r="AG137" s="15">
+        <v>8.6400000000000006E-8</v>
+      </c>
       <c r="BN137" s="4" t="s">
         <v>95</v>
       </c>
@@ -18868,7 +18906,9 @@
       <c r="AF138" s="1">
         <v>86.4</v>
       </c>
-      <c r="AG138" s="1"/>
+      <c r="AG138" s="1">
+        <v>86.4</v>
+      </c>
       <c r="BN138" s="4" t="s">
         <v>96</v>
       </c>
@@ -18962,7 +19002,9 @@
       <c r="AF139" s="13">
         <v>8.6399999999999999E-9</v>
       </c>
-      <c r="AG139" s="15"/>
+      <c r="AG139" s="15">
+        <v>8.6400000000000006E-8</v>
+      </c>
       <c r="BN139" s="4" t="s">
         <v>96</v>
       </c>
@@ -19056,7 +19098,9 @@
       <c r="AF140" s="1">
         <v>86.4</v>
       </c>
-      <c r="AG140" s="1"/>
+      <c r="AG140" s="1">
+        <v>86.4</v>
+      </c>
       <c r="BN140" s="4" t="s">
         <v>96</v>
       </c>

</xml_diff>

<commit_message>
Modify pumping rates for sustainable yield estimation in Run03
</commit_message>
<xml_diff>
--- a/setup.xlsx
+++ b/setup.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cmarinriver\Projects\ConfinedLab\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC14C1F3-3894-466A-B410-8F6EE96B7693}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0891ED1-E2E2-4720-96CA-E52F8C90FE0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15796" firstSheet="6" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15796" firstSheet="6" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="grid" sheetId="1" r:id="rId1"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2445" uniqueCount="1192">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2466" uniqueCount="1192">
   <si>
     <t>nlay</t>
   </si>
@@ -4402,15 +4402,8 @@
       <c r="H1" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="I1" s="4" t="s">
-        <v>104</v>
-      </c>
-      <c r="J1" s="4" t="s">
-        <v>105</v>
-      </c>
-      <c r="K1" s="4" t="s">
-        <v>106</v>
-      </c>
+      <c r="I1" s="4"/>
+      <c r="K1" s="4"/>
       <c r="L1" s="4"/>
       <c r="M1" s="4"/>
     </row>
@@ -4439,15 +4432,8 @@
       <c r="H2" s="4">
         <v>0</v>
       </c>
-      <c r="I2" s="4">
-        <v>0</v>
-      </c>
-      <c r="J2" s="4">
-        <v>0</v>
-      </c>
-      <c r="K2" s="4">
-        <v>0</v>
-      </c>
+      <c r="I2" s="4"/>
+      <c r="K2" s="4"/>
       <c r="L2" s="4"/>
       <c r="M2" s="4"/>
     </row>
@@ -4462,29 +4448,22 @@
         <v>0</v>
       </c>
       <c r="D3" s="4">
-        <v>-100</v>
+        <v>-1000</v>
       </c>
       <c r="E3" s="4">
-        <v>-200</v>
+        <v>-10000</v>
       </c>
       <c r="F3" s="4">
-        <v>-1000</v>
+        <v>-100000</v>
       </c>
       <c r="G3" s="4">
-        <v>-2000</v>
+        <v>-200000</v>
       </c>
       <c r="H3" s="4">
-        <v>-20000</v>
-      </c>
-      <c r="I3" s="4">
-        <v>-100000</v>
-      </c>
-      <c r="J3" s="4">
-        <v>-200000</v>
-      </c>
-      <c r="K3" s="4">
         <v>-600000</v>
       </c>
+      <c r="I3" s="4"/>
+      <c r="K3" s="4"/>
       <c r="L3" s="4"/>
       <c r="M3" s="4"/>
     </row>
@@ -4499,29 +4478,22 @@
         <v>0</v>
       </c>
       <c r="D4" s="4">
-        <v>-100</v>
+        <v>-1000</v>
       </c>
       <c r="E4" s="4">
-        <v>-200</v>
+        <v>-10000</v>
       </c>
       <c r="F4" s="4">
-        <v>-1000</v>
+        <v>-100000</v>
       </c>
       <c r="G4" s="4">
-        <v>-2000</v>
+        <v>-200000</v>
       </c>
       <c r="H4" s="4">
-        <v>-20000</v>
-      </c>
-      <c r="I4" s="4">
-        <v>-100000</v>
-      </c>
-      <c r="J4" s="4">
-        <v>-200000</v>
-      </c>
-      <c r="K4" s="4">
         <v>-600000</v>
       </c>
+      <c r="I4" s="4"/>
+      <c r="K4" s="4"/>
       <c r="L4" s="4"/>
       <c r="M4" s="4"/>
     </row>
@@ -4550,15 +4522,8 @@
       <c r="H5" s="4">
         <v>0</v>
       </c>
-      <c r="I5" s="4">
-        <v>0</v>
-      </c>
-      <c r="J5" s="4">
-        <v>0</v>
-      </c>
-      <c r="K5" s="4">
-        <v>0</v>
-      </c>
+      <c r="I5" s="4"/>
+      <c r="K5" s="4"/>
       <c r="L5" s="4"/>
       <c r="M5" s="4"/>
     </row>
@@ -4573,29 +4538,22 @@
         <v>0</v>
       </c>
       <c r="D6" s="4">
-        <v>-100</v>
+        <v>-1000</v>
       </c>
       <c r="E6" s="4">
-        <v>-200</v>
+        <v>-10000</v>
       </c>
       <c r="F6" s="4">
-        <v>-1000</v>
+        <v>-100000</v>
       </c>
       <c r="G6" s="4">
-        <v>-2000</v>
+        <v>-200000</v>
       </c>
       <c r="H6" s="4">
-        <v>-20000</v>
-      </c>
-      <c r="I6" s="4">
-        <v>-100000</v>
-      </c>
-      <c r="J6" s="4">
-        <v>-200000</v>
-      </c>
-      <c r="K6" s="4">
         <v>-600000</v>
       </c>
+      <c r="I6" s="4"/>
+      <c r="K6" s="4"/>
       <c r="L6" s="4"/>
       <c r="M6" s="4"/>
     </row>
@@ -4610,29 +4568,22 @@
         <v>0</v>
       </c>
       <c r="D7" s="4">
-        <v>-100</v>
+        <v>-1000</v>
       </c>
       <c r="E7" s="4">
-        <v>-200</v>
+        <v>-10000</v>
       </c>
       <c r="F7" s="4">
-        <v>-1000</v>
+        <v>-100000</v>
       </c>
       <c r="G7" s="4">
-        <v>-2000</v>
+        <v>-200000</v>
       </c>
       <c r="H7" s="4">
-        <v>-20000</v>
-      </c>
-      <c r="I7" s="4">
-        <v>-100000</v>
-      </c>
-      <c r="J7" s="4">
-        <v>-200000</v>
-      </c>
-      <c r="K7" s="4">
         <v>-600000</v>
       </c>
+      <c r="I7" s="4"/>
+      <c r="K7" s="4"/>
       <c r="L7" s="4"/>
       <c r="M7" s="4"/>
     </row>
@@ -4661,15 +4612,8 @@
       <c r="H8" s="4">
         <v>0</v>
       </c>
-      <c r="I8" s="4">
-        <v>0</v>
-      </c>
-      <c r="J8" s="4">
-        <v>0</v>
-      </c>
-      <c r="K8" s="4">
-        <v>0</v>
-      </c>
+      <c r="I8" s="4"/>
+      <c r="K8" s="4"/>
       <c r="L8" s="4"/>
       <c r="M8" s="4"/>
     </row>
@@ -4684,29 +4628,22 @@
         <v>0</v>
       </c>
       <c r="D9" s="4">
-        <v>-100</v>
+        <v>-1000</v>
       </c>
       <c r="E9" s="4">
-        <v>-200</v>
+        <v>-10000</v>
       </c>
       <c r="F9" s="4">
-        <v>-1000</v>
+        <v>-100000</v>
       </c>
       <c r="G9" s="4">
-        <v>-2000</v>
+        <v>-200000</v>
       </c>
       <c r="H9" s="4">
-        <v>-20000</v>
-      </c>
-      <c r="I9" s="4">
-        <v>-100000</v>
-      </c>
-      <c r="J9" s="4">
-        <v>-200000</v>
-      </c>
-      <c r="K9" s="4">
         <v>-600000</v>
       </c>
+      <c r="I9" s="4"/>
+      <c r="K9" s="4"/>
       <c r="L9" s="4"/>
       <c r="M9" s="4"/>
     </row>
@@ -4721,29 +4658,22 @@
         <v>0</v>
       </c>
       <c r="D10" s="4">
-        <v>-100</v>
+        <v>-1000</v>
       </c>
       <c r="E10" s="4">
-        <v>-200</v>
+        <v>-10000</v>
       </c>
       <c r="F10" s="4">
-        <v>-1000</v>
+        <v>-100000</v>
       </c>
       <c r="G10" s="4">
-        <v>-2000</v>
+        <v>-200000</v>
       </c>
       <c r="H10" s="4">
-        <v>-20000</v>
-      </c>
-      <c r="I10" s="4">
-        <v>-100000</v>
-      </c>
-      <c r="J10" s="4">
-        <v>-200000</v>
-      </c>
-      <c r="K10" s="4">
         <v>-600000</v>
       </c>
+      <c r="I10" s="4"/>
+      <c r="K10" s="4"/>
       <c r="L10" s="4"/>
       <c r="M10" s="4"/>
     </row>
@@ -4772,15 +4702,8 @@
       <c r="H11" s="4">
         <v>0</v>
       </c>
-      <c r="I11" s="4">
-        <v>0</v>
-      </c>
-      <c r="J11" s="4">
-        <v>0</v>
-      </c>
-      <c r="K11" s="4">
-        <v>0</v>
-      </c>
+      <c r="I11" s="4"/>
+      <c r="K11" s="4"/>
       <c r="L11" s="4"/>
       <c r="M11" s="4"/>
     </row>
@@ -4795,29 +4718,22 @@
         <v>0</v>
       </c>
       <c r="D12" s="4">
-        <v>-100</v>
+        <v>-1000</v>
       </c>
       <c r="E12" s="4">
-        <v>-200</v>
+        <v>-10000</v>
       </c>
       <c r="F12" s="4">
-        <v>-1000</v>
+        <v>-100000</v>
       </c>
       <c r="G12" s="4">
-        <v>-2000</v>
+        <v>-200000</v>
       </c>
       <c r="H12" s="4">
-        <v>-20000</v>
-      </c>
-      <c r="I12" s="4">
-        <v>-100000</v>
-      </c>
-      <c r="J12" s="4">
-        <v>-200000</v>
-      </c>
-      <c r="K12" s="4">
         <v>-600000</v>
       </c>
+      <c r="I12" s="4"/>
+      <c r="K12" s="4"/>
       <c r="L12" s="4"/>
       <c r="M12" s="4"/>
     </row>
@@ -4832,29 +4748,22 @@
         <v>0</v>
       </c>
       <c r="D13" s="4">
-        <v>-100</v>
+        <v>-1000</v>
       </c>
       <c r="E13" s="4">
-        <v>-200</v>
+        <v>-10000</v>
       </c>
       <c r="F13" s="4">
-        <v>-1000</v>
+        <v>-100000</v>
       </c>
       <c r="G13" s="4">
-        <v>-2000</v>
+        <v>-200000</v>
       </c>
       <c r="H13" s="4">
-        <v>-20000</v>
-      </c>
-      <c r="I13" s="4">
-        <v>-100000</v>
-      </c>
-      <c r="J13" s="4">
-        <v>-200000</v>
-      </c>
-      <c r="K13" s="4">
         <v>-600000</v>
       </c>
+      <c r="I13" s="4"/>
+      <c r="K13" s="4"/>
       <c r="L13" s="4"/>
       <c r="M13" s="4"/>
     </row>
@@ -4883,15 +4792,8 @@
       <c r="H14" s="4">
         <v>0</v>
       </c>
-      <c r="I14" s="4">
-        <v>0</v>
-      </c>
-      <c r="J14" s="4">
-        <v>0</v>
-      </c>
-      <c r="K14" s="4">
-        <v>0</v>
-      </c>
+      <c r="I14" s="4"/>
+      <c r="K14" s="4"/>
       <c r="L14" s="4"/>
       <c r="M14" s="4"/>
     </row>
@@ -4906,29 +4808,22 @@
         <v>0</v>
       </c>
       <c r="D15" s="4">
-        <v>-100</v>
+        <v>-1000</v>
       </c>
       <c r="E15" s="4">
-        <v>-200</v>
+        <v>-10000</v>
       </c>
       <c r="F15" s="4">
-        <v>-1000</v>
+        <v>-100000</v>
       </c>
       <c r="G15" s="4">
-        <v>-2000</v>
+        <v>-200000</v>
       </c>
       <c r="H15" s="4">
-        <v>-20000</v>
-      </c>
-      <c r="I15" s="4">
-        <v>-100000</v>
-      </c>
-      <c r="J15" s="4">
-        <v>-200000</v>
-      </c>
-      <c r="K15" s="4">
         <v>-600000</v>
       </c>
+      <c r="I15" s="4"/>
+      <c r="K15" s="4"/>
       <c r="L15" s="4"/>
       <c r="M15" s="4"/>
     </row>
@@ -4943,29 +4838,22 @@
         <v>0</v>
       </c>
       <c r="D16" s="4">
-        <v>-100</v>
+        <v>-1000</v>
       </c>
       <c r="E16" s="4">
-        <v>-200</v>
+        <v>-10000</v>
       </c>
       <c r="F16" s="4">
-        <v>-1000</v>
+        <v>-100000</v>
       </c>
       <c r="G16" s="4">
-        <v>-2000</v>
+        <v>-200000</v>
       </c>
       <c r="H16" s="4">
-        <v>-20000</v>
-      </c>
-      <c r="I16" s="4">
-        <v>-100000</v>
-      </c>
-      <c r="J16" s="4">
-        <v>-200000</v>
-      </c>
-      <c r="K16" s="4">
         <v>-600000</v>
       </c>
+      <c r="I16" s="4"/>
+      <c r="K16" s="4"/>
       <c r="L16" s="4"/>
       <c r="M16" s="4"/>
     </row>
@@ -19450,7 +19338,7 @@
         <v>6.785411243790979E-4</v>
       </c>
     </row>
-    <row r="145" spans="1:27" x14ac:dyDescent="0.45">
+    <row r="145" spans="1:76" x14ac:dyDescent="0.45">
       <c r="A145" t="s">
         <v>264</v>
       </c>
@@ -19504,7 +19392,7 @@
         <v>7.2348983877483703E-4</v>
       </c>
     </row>
-    <row r="146" spans="1:27" x14ac:dyDescent="0.45">
+    <row r="146" spans="1:76" x14ac:dyDescent="0.45">
       <c r="A146" t="s">
         <v>265</v>
       </c>
@@ -19557,8 +19445,11 @@
         <f t="shared" si="19"/>
         <v>6.5532909863160892E-4</v>
       </c>
-    </row>
-    <row r="147" spans="1:27" x14ac:dyDescent="0.45">
+      <c r="BN146" t="s">
+        <v>1189</v>
+      </c>
+    </row>
+    <row r="147" spans="1:76" x14ac:dyDescent="0.45">
       <c r="A147" t="s">
         <v>266</v>
       </c>
@@ -19611,8 +19502,35 @@
         <f t="shared" si="19"/>
         <v>7.5474341979737567E-4</v>
       </c>
-    </row>
-    <row r="148" spans="1:27" x14ac:dyDescent="0.45">
+      <c r="BN147" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="BO147" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="BP147" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="BQ147" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="BR147" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="BS147" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="BT147" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="BU147" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="BV147" s="4"/>
+      <c r="BW147" s="4"/>
+      <c r="BX147" s="4"/>
+    </row>
+    <row r="148" spans="1:76" x14ac:dyDescent="0.45">
       <c r="A148" t="s">
         <v>267</v>
       </c>
@@ -19665,8 +19583,32 @@
         <f t="shared" si="19"/>
         <v>5.7669688744116539E-4</v>
       </c>
-    </row>
-    <row r="149" spans="1:27" x14ac:dyDescent="0.45">
+      <c r="BN148" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="BO148" s="4">
+        <v>0</v>
+      </c>
+      <c r="BP148" s="4">
+        <v>0</v>
+      </c>
+      <c r="BQ148" s="4">
+        <v>0</v>
+      </c>
+      <c r="BR148" s="4">
+        <v>0</v>
+      </c>
+      <c r="BS148" s="4">
+        <v>0</v>
+      </c>
+      <c r="BT148" s="4">
+        <v>0</v>
+      </c>
+      <c r="BU148" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="149" spans="1:76" x14ac:dyDescent="0.45">
       <c r="A149" t="s">
         <v>268</v>
       </c>
@@ -19719,8 +19661,32 @@
         <f t="shared" si="19"/>
         <v>8.0697176066542612E-4</v>
       </c>
-    </row>
-    <row r="150" spans="1:27" x14ac:dyDescent="0.45">
+      <c r="BN149" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="BO149" s="3">
+        <v>3600000</v>
+      </c>
+      <c r="BP149" s="4">
+        <v>0</v>
+      </c>
+      <c r="BQ149" s="4">
+        <v>-1000</v>
+      </c>
+      <c r="BR149" s="4">
+        <v>-10000</v>
+      </c>
+      <c r="BS149" s="4">
+        <v>-100000</v>
+      </c>
+      <c r="BT149" s="4">
+        <v>-200000</v>
+      </c>
+      <c r="BU149" s="4">
+        <v>-600000</v>
+      </c>
+    </row>
+    <row r="150" spans="1:76" x14ac:dyDescent="0.45">
       <c r="A150" t="s">
         <v>269</v>
       </c>
@@ -19773,8 +19739,32 @@
         <f t="shared" si="19"/>
         <v>6.0999509381094925E-4</v>
       </c>
-    </row>
-    <row r="151" spans="1:27" x14ac:dyDescent="0.45">
+      <c r="BN150" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="BO150" s="3">
+        <v>800000000</v>
+      </c>
+      <c r="BP150" s="4">
+        <v>0</v>
+      </c>
+      <c r="BQ150" s="4">
+        <v>-1000</v>
+      </c>
+      <c r="BR150" s="4">
+        <v>-10000</v>
+      </c>
+      <c r="BS150" s="4">
+        <v>-100000</v>
+      </c>
+      <c r="BT150" s="4">
+        <v>-200000</v>
+      </c>
+      <c r="BU150" s="4">
+        <v>-600000</v>
+      </c>
+    </row>
+    <row r="151" spans="1:76" x14ac:dyDescent="0.45">
       <c r="A151" t="s">
         <v>270</v>
       </c>
@@ -19827,8 +19817,32 @@
         <f t="shared" si="19"/>
         <v>5.3117803129513444E-4</v>
       </c>
-    </row>
-    <row r="152" spans="1:27" x14ac:dyDescent="0.45">
+      <c r="BN151" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="BO151" s="4">
+        <v>0</v>
+      </c>
+      <c r="BP151" s="4">
+        <v>0</v>
+      </c>
+      <c r="BQ151" s="4">
+        <v>0</v>
+      </c>
+      <c r="BR151" s="4">
+        <v>0</v>
+      </c>
+      <c r="BS151" s="4">
+        <v>0</v>
+      </c>
+      <c r="BT151" s="4">
+        <v>0</v>
+      </c>
+      <c r="BU151" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="152" spans="1:76" x14ac:dyDescent="0.45">
       <c r="A152" t="s">
         <v>271</v>
       </c>
@@ -19881,8 +19895,32 @@
         <f t="shared" si="19"/>
         <v>6.8402085428227407E-4</v>
       </c>
-    </row>
-    <row r="153" spans="1:27" x14ac:dyDescent="0.45">
+      <c r="BN152" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="BO152" s="3">
+        <v>3600000</v>
+      </c>
+      <c r="BP152" s="4">
+        <v>0</v>
+      </c>
+      <c r="BQ152" s="4">
+        <v>-1000</v>
+      </c>
+      <c r="BR152" s="4">
+        <v>-10000</v>
+      </c>
+      <c r="BS152" s="4">
+        <v>-100000</v>
+      </c>
+      <c r="BT152" s="4">
+        <v>-200000</v>
+      </c>
+      <c r="BU152" s="4">
+        <v>-600000</v>
+      </c>
+    </row>
+    <row r="153" spans="1:76" x14ac:dyDescent="0.45">
       <c r="A153" t="s">
         <v>272</v>
       </c>
@@ -19935,8 +19973,32 @@
         <f t="shared" si="19"/>
         <v>5.6115552392589597E-4</v>
       </c>
-    </row>
-    <row r="154" spans="1:27" x14ac:dyDescent="0.45">
+      <c r="BN153" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="BO153" s="3">
+        <v>800000000</v>
+      </c>
+      <c r="BP153" s="4">
+        <v>0</v>
+      </c>
+      <c r="BQ153" s="4">
+        <v>-1000</v>
+      </c>
+      <c r="BR153" s="4">
+        <v>-10000</v>
+      </c>
+      <c r="BS153" s="4">
+        <v>-100000</v>
+      </c>
+      <c r="BT153" s="4">
+        <v>-200000</v>
+      </c>
+      <c r="BU153" s="4">
+        <v>-600000</v>
+      </c>
+    </row>
+    <row r="154" spans="1:76" x14ac:dyDescent="0.45">
       <c r="A154" t="s">
         <v>273</v>
       </c>
@@ -19989,8 +20051,32 @@
         <f t="shared" si="19"/>
         <v>5.6175108458420442E-4</v>
       </c>
-    </row>
-    <row r="155" spans="1:27" x14ac:dyDescent="0.45">
+      <c r="BN154" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="BO154" s="4">
+        <v>0</v>
+      </c>
+      <c r="BP154" s="4">
+        <v>0</v>
+      </c>
+      <c r="BQ154" s="4">
+        <v>0</v>
+      </c>
+      <c r="BR154" s="4">
+        <v>0</v>
+      </c>
+      <c r="BS154" s="4">
+        <v>0</v>
+      </c>
+      <c r="BT154" s="4">
+        <v>0</v>
+      </c>
+      <c r="BU154" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="155" spans="1:76" x14ac:dyDescent="0.45">
       <c r="A155" t="s">
         <v>274</v>
       </c>
@@ -20018,8 +20104,32 @@
       <c r="I155">
         <v>36000</v>
       </c>
-    </row>
-    <row r="156" spans="1:27" x14ac:dyDescent="0.45">
+      <c r="BN155" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="BO155" s="3">
+        <v>3600000</v>
+      </c>
+      <c r="BP155" s="4">
+        <v>0</v>
+      </c>
+      <c r="BQ155" s="4">
+        <v>-1000</v>
+      </c>
+      <c r="BR155" s="4">
+        <v>-10000</v>
+      </c>
+      <c r="BS155" s="4">
+        <v>-100000</v>
+      </c>
+      <c r="BT155" s="4">
+        <v>-200000</v>
+      </c>
+      <c r="BU155" s="4">
+        <v>-600000</v>
+      </c>
+    </row>
+    <row r="156" spans="1:76" x14ac:dyDescent="0.45">
       <c r="A156" t="s">
         <v>275</v>
       </c>
@@ -20047,8 +20157,32 @@
       <c r="I156">
         <v>36000</v>
       </c>
-    </row>
-    <row r="157" spans="1:27" x14ac:dyDescent="0.45">
+      <c r="BN156" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="BO156" s="3">
+        <v>800000000</v>
+      </c>
+      <c r="BP156" s="4">
+        <v>0</v>
+      </c>
+      <c r="BQ156" s="4">
+        <v>-1000</v>
+      </c>
+      <c r="BR156" s="4">
+        <v>-10000</v>
+      </c>
+      <c r="BS156" s="4">
+        <v>-100000</v>
+      </c>
+      <c r="BT156" s="4">
+        <v>-200000</v>
+      </c>
+      <c r="BU156" s="4">
+        <v>-600000</v>
+      </c>
+    </row>
+    <row r="157" spans="1:76" x14ac:dyDescent="0.45">
       <c r="A157" t="s">
         <v>276</v>
       </c>
@@ -20076,8 +20210,32 @@
       <c r="I157">
         <v>36000</v>
       </c>
-    </row>
-    <row r="158" spans="1:27" x14ac:dyDescent="0.45">
+      <c r="BN157" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="BO157" s="4">
+        <v>0</v>
+      </c>
+      <c r="BP157" s="4">
+        <v>0</v>
+      </c>
+      <c r="BQ157" s="4">
+        <v>0</v>
+      </c>
+      <c r="BR157" s="4">
+        <v>0</v>
+      </c>
+      <c r="BS157" s="4">
+        <v>0</v>
+      </c>
+      <c r="BT157" s="4">
+        <v>0</v>
+      </c>
+      <c r="BU157" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="158" spans="1:76" x14ac:dyDescent="0.45">
       <c r="A158" t="s">
         <v>277</v>
       </c>
@@ -20105,8 +20263,32 @@
       <c r="I158">
         <v>36000</v>
       </c>
-    </row>
-    <row r="159" spans="1:27" x14ac:dyDescent="0.45">
+      <c r="BN158" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="BO158" s="3">
+        <v>3600000</v>
+      </c>
+      <c r="BP158" s="4">
+        <v>0</v>
+      </c>
+      <c r="BQ158" s="4">
+        <v>-1000</v>
+      </c>
+      <c r="BR158" s="4">
+        <v>-10000</v>
+      </c>
+      <c r="BS158" s="4">
+        <v>-100000</v>
+      </c>
+      <c r="BT158" s="4">
+        <v>-200000</v>
+      </c>
+      <c r="BU158" s="4">
+        <v>-600000</v>
+      </c>
+    </row>
+    <row r="159" spans="1:76" x14ac:dyDescent="0.45">
       <c r="A159" t="s">
         <v>278</v>
       </c>
@@ -20134,8 +20316,32 @@
       <c r="I159">
         <v>36000</v>
       </c>
-    </row>
-    <row r="160" spans="1:27" x14ac:dyDescent="0.45">
+      <c r="BN159" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="BO159" s="3">
+        <v>800000000</v>
+      </c>
+      <c r="BP159" s="4">
+        <v>0</v>
+      </c>
+      <c r="BQ159" s="4">
+        <v>-1000</v>
+      </c>
+      <c r="BR159" s="4">
+        <v>-10000</v>
+      </c>
+      <c r="BS159" s="4">
+        <v>-100000</v>
+      </c>
+      <c r="BT159" s="4">
+        <v>-200000</v>
+      </c>
+      <c r="BU159" s="4">
+        <v>-600000</v>
+      </c>
+    </row>
+    <row r="160" spans="1:76" x14ac:dyDescent="0.45">
       <c r="A160" t="s">
         <v>279</v>
       </c>
@@ -20163,8 +20369,32 @@
       <c r="I160">
         <v>36000</v>
       </c>
-    </row>
-    <row r="161" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="BN160" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="BO160" s="4">
+        <v>0</v>
+      </c>
+      <c r="BP160" s="4">
+        <v>0</v>
+      </c>
+      <c r="BQ160" s="4">
+        <v>0</v>
+      </c>
+      <c r="BR160" s="4">
+        <v>0</v>
+      </c>
+      <c r="BS160" s="4">
+        <v>0</v>
+      </c>
+      <c r="BT160" s="4">
+        <v>0</v>
+      </c>
+      <c r="BU160" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="161" spans="1:73" x14ac:dyDescent="0.45">
       <c r="A161" t="s">
         <v>280</v>
       </c>
@@ -20192,8 +20422,32 @@
       <c r="I161">
         <v>36000</v>
       </c>
-    </row>
-    <row r="162" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="BN161" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="BO161" s="3">
+        <v>3600000</v>
+      </c>
+      <c r="BP161" s="4">
+        <v>0</v>
+      </c>
+      <c r="BQ161" s="4">
+        <v>-1000</v>
+      </c>
+      <c r="BR161" s="4">
+        <v>-10000</v>
+      </c>
+      <c r="BS161" s="4">
+        <v>-100000</v>
+      </c>
+      <c r="BT161" s="4">
+        <v>-200000</v>
+      </c>
+      <c r="BU161" s="4">
+        <v>-600000</v>
+      </c>
+    </row>
+    <row r="162" spans="1:73" x14ac:dyDescent="0.45">
       <c r="A162" t="s">
         <v>281</v>
       </c>
@@ -20221,8 +20475,32 @@
       <c r="I162">
         <v>36000</v>
       </c>
-    </row>
-    <row r="163" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="BN162" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="BO162" s="3">
+        <v>800000000</v>
+      </c>
+      <c r="BP162" s="4">
+        <v>0</v>
+      </c>
+      <c r="BQ162" s="4">
+        <v>-1000</v>
+      </c>
+      <c r="BR162" s="4">
+        <v>-10000</v>
+      </c>
+      <c r="BS162" s="4">
+        <v>-100000</v>
+      </c>
+      <c r="BT162" s="4">
+        <v>-200000</v>
+      </c>
+      <c r="BU162" s="4">
+        <v>-600000</v>
+      </c>
+    </row>
+    <row r="163" spans="1:73" x14ac:dyDescent="0.45">
       <c r="A163" t="s">
         <v>282</v>
       </c>
@@ -20251,7 +20529,7 @@
         <v>36000</v>
       </c>
     </row>
-    <row r="164" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="164" spans="1:73" x14ac:dyDescent="0.45">
       <c r="A164" t="s">
         <v>283</v>
       </c>
@@ -20280,7 +20558,7 @@
         <v>36000</v>
       </c>
     </row>
-    <row r="165" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="165" spans="1:73" x14ac:dyDescent="0.45">
       <c r="A165" t="s">
         <v>284</v>
       </c>
@@ -20309,7 +20587,7 @@
         <v>36000</v>
       </c>
     </row>
-    <row r="166" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="166" spans="1:73" x14ac:dyDescent="0.45">
       <c r="A166" t="s">
         <v>285</v>
       </c>
@@ -20338,7 +20616,7 @@
         <v>36000</v>
       </c>
     </row>
-    <row r="167" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="167" spans="1:73" x14ac:dyDescent="0.45">
       <c r="A167" t="s">
         <v>286</v>
       </c>
@@ -20367,7 +20645,7 @@
         <v>36000</v>
       </c>
     </row>
-    <row r="168" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="168" spans="1:73" x14ac:dyDescent="0.45">
       <c r="A168" t="s">
         <v>287</v>
       </c>
@@ -20396,7 +20674,7 @@
         <v>36000</v>
       </c>
     </row>
-    <row r="169" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="169" spans="1:73" x14ac:dyDescent="0.45">
       <c r="A169" t="s">
         <v>288</v>
       </c>
@@ -20425,7 +20703,7 @@
         <v>36000</v>
       </c>
     </row>
-    <row r="170" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="170" spans="1:73" x14ac:dyDescent="0.45">
       <c r="A170" t="s">
         <v>289</v>
       </c>
@@ -20454,7 +20732,7 @@
         <v>36000</v>
       </c>
     </row>
-    <row r="171" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="171" spans="1:73" x14ac:dyDescent="0.45">
       <c r="A171" t="s">
         <v>290</v>
       </c>
@@ -20483,7 +20761,7 @@
         <v>36000</v>
       </c>
     </row>
-    <row r="172" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="172" spans="1:73" x14ac:dyDescent="0.45">
       <c r="A172" t="s">
         <v>291</v>
       </c>
@@ -20512,7 +20790,7 @@
         <v>36000</v>
       </c>
     </row>
-    <row r="173" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="173" spans="1:73" x14ac:dyDescent="0.45">
       <c r="A173" t="s">
         <v>292</v>
       </c>
@@ -20541,7 +20819,7 @@
         <v>36000</v>
       </c>
     </row>
-    <row r="174" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="174" spans="1:73" x14ac:dyDescent="0.45">
       <c r="A174" t="s">
         <v>293</v>
       </c>
@@ -20570,7 +20848,7 @@
         <v>36000</v>
       </c>
     </row>
-    <row r="175" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="175" spans="1:73" x14ac:dyDescent="0.45">
       <c r="A175" t="s">
         <v>294</v>
       </c>
@@ -20599,7 +20877,7 @@
         <v>36000</v>
       </c>
     </row>
-    <row r="176" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="176" spans="1:73" x14ac:dyDescent="0.45">
       <c r="A176" t="s">
         <v>295</v>
       </c>

</xml_diff>

<commit_message>
Modify convergence criterion of flows for Run 03
</commit_message>
<xml_diff>
--- a/setup.xlsx
+++ b/setup.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cmarinriver\Projects\ConfinedLab\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0891ED1-E2E2-4720-96CA-E52F8C90FE0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63DAAEDE-2FDB-45F4-B662-2017CFDA3D29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15796" firstSheet="6" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15796" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="grid" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Decrease convergence criterion for flows. Set thin threshold to 1 meter
</commit_message>
<xml_diff>
--- a/setup.xlsx
+++ b/setup.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cmarinriver\Projects\ConfinedLab\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63DAAEDE-2FDB-45F4-B662-2017CFDA3D29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{793FF981-8BC5-430B-B2D2-CF80F3D2C8E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15796" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26434,7 +26434,7 @@
         <v>70</v>
       </c>
       <c r="J2" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K2" s="4">
         <v>1</v>
@@ -26469,7 +26469,7 @@
         <v>70</v>
       </c>
       <c r="J3" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K3" s="4">
         <v>2</v>
@@ -26504,7 +26504,7 @@
         <v>70</v>
       </c>
       <c r="J4" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K4" s="4">
         <v>3</v>
@@ -26539,7 +26539,7 @@
         <v>70</v>
       </c>
       <c r="J5" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K5" s="4">
         <v>4</v>
@@ -26574,7 +26574,7 @@
         <v>70</v>
       </c>
       <c r="J6" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K6" s="4">
         <v>5</v>

</xml_diff>

<commit_message>
Change thin cell threshold to 2 meters
</commit_message>
<xml_diff>
--- a/setup.xlsx
+++ b/setup.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cmarinriver\Projects\ConfinedLab\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{793FF981-8BC5-430B-B2D2-CF80F3D2C8E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF998F78-E574-4901-9F1E-19BF24234160}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15796" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26434,7 +26434,7 @@
         <v>70</v>
       </c>
       <c r="J2" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K2" s="4">
         <v>1</v>
@@ -26469,7 +26469,7 @@
         <v>70</v>
       </c>
       <c r="J3" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K3" s="4">
         <v>2</v>
@@ -26504,7 +26504,7 @@
         <v>70</v>
       </c>
       <c r="J4" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K4" s="4">
         <v>3</v>
@@ -26539,7 +26539,7 @@
         <v>70</v>
       </c>
       <c r="J5" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K5" s="4">
         <v>4</v>
@@ -26574,7 +26574,7 @@
         <v>70</v>
       </c>
       <c r="J6" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K6" s="4">
         <v>5</v>

</xml_diff>

<commit_message>
Change thin cell threshold to 3 meters
</commit_message>
<xml_diff>
--- a/setup.xlsx
+++ b/setup.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cmarinriver\Projects\ConfinedLab\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF998F78-E574-4901-9F1E-19BF24234160}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D86B026-43E4-4661-A6BF-40A1B2BF9C0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15796" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26434,7 +26434,7 @@
         <v>70</v>
       </c>
       <c r="J2" s="4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K2" s="4">
         <v>1</v>
@@ -26469,7 +26469,7 @@
         <v>70</v>
       </c>
       <c r="J3" s="4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K3" s="4">
         <v>2</v>
@@ -26504,7 +26504,7 @@
         <v>70</v>
       </c>
       <c r="J4" s="4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K4" s="4">
         <v>3</v>
@@ -26539,7 +26539,7 @@
         <v>70</v>
       </c>
       <c r="J5" s="4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K5" s="4">
         <v>4</v>
@@ -26574,7 +26574,7 @@
         <v>70</v>
       </c>
       <c r="J6" s="4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K6" s="4">
         <v>5</v>

</xml_diff>

<commit_message>
Fix small bugs on modtransient 6. Reduces number of decimals in recharge rate
</commit_message>
<xml_diff>
--- a/setup.xlsx
+++ b/setup.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cmarinriver\Projects\ConfinedLab\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D86B026-43E4-4661-A6BF-40A1B2BF9C0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CE76D5B-775C-4CA8-9DCA-352EC9C711FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15796" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28300,7 +28300,7 @@
         <v>38</v>
       </c>
       <c r="B22">
-        <v>5.5555555555555599E-4</v>
+        <v>5.5999999999999995E-4</v>
       </c>
       <c r="C22">
         <v>3.1154231364886891E-4</v>
@@ -28325,8 +28325,8 @@
       <c r="A23" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="B23">
-        <v>5.5555555555555599E-4</v>
+      <c r="B23" s="4">
+        <v>5.5999999999999995E-4</v>
       </c>
       <c r="C23">
         <v>3.1154231364886891E-5</v>
@@ -28351,8 +28351,8 @@
       <c r="A24" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="B24">
-        <v>5.5555555555555599E-4</v>
+      <c r="B24" s="4">
+        <v>5.5999999999999995E-4</v>
       </c>
       <c r="C24">
         <v>3.1154231364886891E-4</v>
@@ -28377,8 +28377,8 @@
       <c r="A25" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="B25">
-        <v>5.5555555555555599E-4</v>
+      <c r="B25" s="4">
+        <v>5.5999999999999995E-4</v>
       </c>
       <c r="C25">
         <v>3.1154231364886891E-5</v>
@@ -28403,8 +28403,8 @@
       <c r="A26" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="B26">
-        <v>5.5555555555555599E-4</v>
+      <c r="B26" s="4">
+        <v>5.5999999999999995E-4</v>
       </c>
       <c r="C26">
         <v>3.1154231364886891E-4</v>
@@ -28590,19 +28590,19 @@
         <v>0</v>
       </c>
       <c r="B2" s="1">
-        <v>5.5555555555555599E-4</v>
+        <v>5.5999999999999995E-4</v>
       </c>
       <c r="C2" s="1">
-        <v>5.5555555555555599E-4</v>
+        <v>5.5999999999999995E-4</v>
       </c>
       <c r="D2" s="1">
-        <v>5.5555555555555599E-4</v>
+        <v>5.5999999999999995E-4</v>
       </c>
       <c r="E2" s="1">
-        <v>5.5555555555555599E-4</v>
+        <v>5.5999999999999995E-4</v>
       </c>
       <c r="F2" s="1">
-        <v>5.5555555555555599E-4</v>
+        <v>5.5999999999999995E-4</v>
       </c>
       <c r="G2" s="1"/>
       <c r="I2" s="1"/>
@@ -28615,19 +28615,19 @@
         <v>3600000</v>
       </c>
       <c r="B3" s="1">
-        <v>5.5555555555555599E-4</v>
+        <v>5.5999999999999995E-4</v>
       </c>
       <c r="C3" s="1">
-        <v>5.5555555555555599E-4</v>
+        <v>5.5999999999999995E-4</v>
       </c>
       <c r="D3" s="1">
-        <v>5.5555555555555599E-4</v>
+        <v>5.5999999999999995E-4</v>
       </c>
       <c r="E3" s="1">
-        <v>5.5555555555555599E-4</v>
+        <v>5.5999999999999995E-4</v>
       </c>
       <c r="F3" s="1">
-        <v>5.5555555555555599E-4</v>
+        <v>5.5999999999999995E-4</v>
       </c>
       <c r="G3" s="1"/>
       <c r="I3" s="1"/>
@@ -28640,19 +28640,19 @@
         <v>800000000</v>
       </c>
       <c r="B4" s="1">
-        <v>5.5555555555555599E-4</v>
+        <v>5.5999999999999995E-4</v>
       </c>
       <c r="C4" s="1">
-        <v>5.5555555555555599E-4</v>
+        <v>5.5999999999999995E-4</v>
       </c>
       <c r="D4" s="1">
-        <v>5.5555555555555599E-4</v>
+        <v>5.5999999999999995E-4</v>
       </c>
       <c r="E4" s="1">
-        <v>5.5555555555555599E-4</v>
+        <v>5.5999999999999995E-4</v>
       </c>
       <c r="F4" s="1">
-        <v>5.5555555555555599E-4</v>
+        <v>5.5999999999999995E-4</v>
       </c>
       <c r="G4" s="1"/>
     </row>

</xml_diff>

<commit_message>
Increased number of iterations to 200
</commit_message>
<xml_diff>
--- a/setup.xlsx
+++ b/setup.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cmarinriver\Projects\ConfinedLab\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CE76D5B-775C-4CA8-9DCA-352EC9C711FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E8DDE15-48D3-4D88-AC03-9B771B36F203}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15796" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15796" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="grid" sheetId="1" r:id="rId1"/>
@@ -28299,8 +28299,8 @@
       <c r="A22" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="B22">
-        <v>5.5999999999999995E-4</v>
+      <c r="B22" s="1">
+        <v>5.5555555555555556E-4</v>
       </c>
       <c r="C22">
         <v>3.1154231364886891E-4</v>
@@ -28325,8 +28325,8 @@
       <c r="A23" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="B23" s="4">
-        <v>5.5999999999999995E-4</v>
+      <c r="B23" s="1">
+        <v>5.5555555555555556E-4</v>
       </c>
       <c r="C23">
         <v>3.1154231364886891E-5</v>
@@ -28351,8 +28351,8 @@
       <c r="A24" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="B24" s="4">
-        <v>5.5999999999999995E-4</v>
+      <c r="B24" s="1">
+        <v>5.5555555555555556E-4</v>
       </c>
       <c r="C24">
         <v>3.1154231364886891E-4</v>
@@ -28377,8 +28377,8 @@
       <c r="A25" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="B25" s="4">
-        <v>5.5999999999999995E-4</v>
+      <c r="B25" s="1">
+        <v>5.5555555555555556E-4</v>
       </c>
       <c r="C25">
         <v>3.1154231364886891E-5</v>
@@ -28403,8 +28403,8 @@
       <c r="A26" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="B26" s="4">
-        <v>5.5999999999999995E-4</v>
+      <c r="B26" s="1">
+        <v>5.5555555555555556E-4</v>
       </c>
       <c r="C26">
         <v>3.1154231364886891E-4</v>
@@ -28590,19 +28590,19 @@
         <v>0</v>
       </c>
       <c r="B2" s="1">
-        <v>5.5999999999999995E-4</v>
+        <v>5.5555555555555556E-4</v>
       </c>
       <c r="C2" s="1">
-        <v>5.5999999999999995E-4</v>
+        <v>5.5555555555555556E-4</v>
       </c>
       <c r="D2" s="1">
-        <v>5.5999999999999995E-4</v>
+        <v>5.5555555555555556E-4</v>
       </c>
       <c r="E2" s="1">
-        <v>5.5999999999999995E-4</v>
+        <v>5.5555555555555556E-4</v>
       </c>
       <c r="F2" s="1">
-        <v>5.5999999999999995E-4</v>
+        <v>5.5555555555555556E-4</v>
       </c>
       <c r="G2" s="1"/>
       <c r="I2" s="1"/>
@@ -28615,19 +28615,19 @@
         <v>3600000</v>
       </c>
       <c r="B3" s="1">
-        <v>5.5999999999999995E-4</v>
+        <v>5.5555555555555556E-4</v>
       </c>
       <c r="C3" s="1">
-        <v>5.5999999999999995E-4</v>
+        <v>5.5555555555555556E-4</v>
       </c>
       <c r="D3" s="1">
-        <v>5.5999999999999995E-4</v>
+        <v>5.5555555555555556E-4</v>
       </c>
       <c r="E3" s="1">
-        <v>5.5999999999999995E-4</v>
+        <v>5.5555555555555556E-4</v>
       </c>
       <c r="F3" s="1">
-        <v>5.5999999999999995E-4</v>
+        <v>5.5555555555555556E-4</v>
       </c>
       <c r="G3" s="1"/>
       <c r="I3" s="1"/>
@@ -28640,19 +28640,19 @@
         <v>800000000</v>
       </c>
       <c r="B4" s="1">
-        <v>5.5999999999999995E-4</v>
+        <v>5.5555555555555556E-4</v>
       </c>
       <c r="C4" s="1">
-        <v>5.5999999999999995E-4</v>
+        <v>5.5555555555555556E-4</v>
       </c>
       <c r="D4" s="1">
-        <v>5.5999999999999995E-4</v>
+        <v>5.5555555555555556E-4</v>
       </c>
       <c r="E4" s="1">
-        <v>5.5999999999999995E-4</v>
+        <v>5.5555555555555556E-4</v>
       </c>
       <c r="F4" s="1">
-        <v>5.5999999999999995E-4</v>
+        <v>5.5555555555555556E-4</v>
       </c>
       <c r="G4" s="1"/>
     </row>

</xml_diff>

<commit_message>
Modify model file to retry model run
</commit_message>
<xml_diff>
--- a/setup.xlsx
+++ b/setup.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cmarinriver\Projects\ConfinedLab\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1659BF11-04CB-4C73-B3BA-9602F578E27C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94F187C1-EA2D-43FA-82CF-CA59FEFE8AE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15796" firstSheet="3" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1440" yWindow="1440" windowWidth="21600" windowHeight="11423" firstSheet="6" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="grid" sheetId="1" r:id="rId1"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2509" uniqueCount="1194">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2510" uniqueCount="1194">
   <si>
     <t>nlay</t>
   </si>
@@ -5980,7 +5980,7 @@
   <dimension ref="A1:H20"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="3" width="17.06640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="4" width="17.06640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.45">
@@ -5993,6 +5993,9 @@
       <c r="C1" s="12" t="s">
         <v>920</v>
       </c>
+      <c r="D1" s="12" t="s">
+        <v>1066</v>
+      </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A2" s="16" t="s">
@@ -6004,7 +6007,9 @@
       <c r="C2" s="13">
         <v>86.4</v>
       </c>
-      <c r="D2" s="13"/>
+      <c r="D2" s="13">
+        <v>8.64</v>
+      </c>
       <c r="E2" s="13"/>
       <c r="F2" s="13"/>
       <c r="G2" s="13"/>
@@ -6020,7 +6025,9 @@
       <c r="C3" s="14">
         <v>8.6399999999999999E-9</v>
       </c>
-      <c r="D3" s="13"/>
+      <c r="D3" s="11">
+        <v>8.6400000000000006E-8</v>
+      </c>
       <c r="E3" s="13"/>
       <c r="F3" s="13"/>
       <c r="G3" s="13"/>
@@ -6036,7 +6043,9 @@
       <c r="C4" s="13">
         <v>86.4</v>
       </c>
-      <c r="D4" s="13"/>
+      <c r="D4" s="13">
+        <v>8.64</v>
+      </c>
       <c r="E4" s="13"/>
       <c r="F4" s="13"/>
       <c r="G4" s="13"/>
@@ -6052,7 +6061,9 @@
       <c r="C5" s="14">
         <v>8.6399999999999999E-9</v>
       </c>
-      <c r="D5" s="13"/>
+      <c r="D5" s="11">
+        <v>8.6400000000000006E-8</v>
+      </c>
       <c r="E5" s="13"/>
       <c r="F5" s="13"/>
       <c r="G5" s="13"/>
@@ -6068,7 +6079,9 @@
       <c r="C6" s="13">
         <v>86.4</v>
       </c>
-      <c r="D6" s="13"/>
+      <c r="D6" s="13">
+        <v>8.64</v>
+      </c>
       <c r="E6" s="13"/>
       <c r="F6" s="13"/>
       <c r="G6" s="13"/>
@@ -6084,7 +6097,9 @@
       <c r="C7" s="13">
         <v>86.4</v>
       </c>
-      <c r="D7" s="13"/>
+      <c r="D7" s="13">
+        <v>8.64</v>
+      </c>
       <c r="E7" s="13"/>
       <c r="F7" s="13"/>
       <c r="G7" s="13"/>
@@ -6100,7 +6115,9 @@
       <c r="C8" s="14">
         <v>8.6399999999999999E-9</v>
       </c>
-      <c r="D8" s="13"/>
+      <c r="D8" s="11">
+        <v>8.6400000000000006E-8</v>
+      </c>
       <c r="E8" s="13"/>
       <c r="F8" s="13"/>
       <c r="G8" s="13"/>
@@ -6116,7 +6133,9 @@
       <c r="C9" s="13">
         <v>86.4</v>
       </c>
-      <c r="D9" s="13"/>
+      <c r="D9" s="13">
+        <v>8.64</v>
+      </c>
       <c r="E9" s="13"/>
       <c r="F9" s="13"/>
       <c r="G9" s="13"/>
@@ -6132,7 +6151,9 @@
       <c r="C10" s="14">
         <v>8.6399999999999999E-9</v>
       </c>
-      <c r="D10" s="13"/>
+      <c r="D10" s="11">
+        <v>8.6400000000000006E-8</v>
+      </c>
       <c r="E10" s="13"/>
       <c r="F10" s="13"/>
       <c r="G10" s="13"/>
@@ -6148,7 +6169,9 @@
       <c r="C11" s="13">
         <v>86.4</v>
       </c>
-      <c r="D11" s="13"/>
+      <c r="D11" s="13">
+        <v>8.64</v>
+      </c>
       <c r="E11" s="13"/>
       <c r="F11" s="13"/>
       <c r="G11" s="13"/>

</xml_diff>

<commit_message>
Updated setup file for response time estimation to pumping
</commit_message>
<xml_diff>
--- a/setup.xlsx
+++ b/setup.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cmarinriver\Projects\ConfinedLab\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7969EB1-2877-467B-B226-29ECA8BC9604}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B641C5A-12B4-4CA8-9971-CE19F5130DC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15796" firstSheet="2" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15796" firstSheet="2" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="grid" sheetId="1" r:id="rId1"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2649" uniqueCount="1216">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2651" uniqueCount="1217">
   <si>
     <t>nlay</t>
   </si>
@@ -3695,6 +3695,9 @@
   </si>
   <si>
     <t>12_99_130</t>
+  </si>
+  <si>
+    <t>qv_11</t>
   </si>
 </sst>
 </file>
@@ -4221,7 +4224,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
-  <dimension ref="A1:L18"/>
+  <dimension ref="A1:M18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="8" width="10.73046875" bestFit="1" customWidth="1"/>
@@ -4229,7 +4232,7 @@
     <col min="12" max="12" width="11.796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>89</v>
       </c>
@@ -4239,35 +4242,38 @@
       <c r="C1" t="s">
         <v>114</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="11" t="s">
         <v>115</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="11" t="s">
         <v>116</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="11" t="s">
         <v>117</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="11" t="s">
         <v>118</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="11" t="s">
         <v>119</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="11" t="s">
         <v>120</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="11" t="s">
         <v>121</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="11" t="s">
         <v>122</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="11" t="s">
         <v>123</v>
       </c>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M1" s="11" t="s">
+        <v>1216</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>91</v>
       </c>
@@ -4290,22 +4296,25 @@
         <v>-10000</v>
       </c>
       <c r="H2" s="11">
+        <v>-30000</v>
+      </c>
+      <c r="I2" s="11">
         <v>-50000</v>
       </c>
-      <c r="I2" s="11">
+      <c r="J2" s="11">
         <v>-100000</v>
       </c>
-      <c r="J2" s="11">
+      <c r="K2" s="11">
         <v>-200000</v>
       </c>
-      <c r="K2" s="11">
+      <c r="L2" s="11">
         <v>-500000</v>
       </c>
-      <c r="L2" s="11">
+      <c r="M2" s="11">
         <v>-1000000</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>92</v>
       </c>
@@ -4328,22 +4337,25 @@
         <v>-10000</v>
       </c>
       <c r="H3" s="11">
+        <v>-30000</v>
+      </c>
+      <c r="I3" s="11">
         <v>-50000</v>
       </c>
-      <c r="I3" s="11">
+      <c r="J3" s="11">
         <v>-100000</v>
       </c>
-      <c r="J3" s="11">
+      <c r="K3" s="11">
         <v>-200000</v>
       </c>
-      <c r="K3" s="11">
+      <c r="L3" s="11">
         <v>-500000</v>
       </c>
-      <c r="L3" s="11">
+      <c r="M3" s="11">
         <v>-1000000</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>93</v>
       </c>
@@ -4366,22 +4378,25 @@
         <v>-10000</v>
       </c>
       <c r="H4" s="11">
+        <v>-30000</v>
+      </c>
+      <c r="I4" s="11">
         <v>-50000</v>
       </c>
-      <c r="I4" s="11">
+      <c r="J4" s="11">
         <v>-100000</v>
       </c>
-      <c r="J4" s="11">
+      <c r="K4" s="11">
         <v>-200000</v>
       </c>
-      <c r="K4" s="11">
+      <c r="L4" s="11">
         <v>-500000</v>
       </c>
-      <c r="L4" s="11">
+      <c r="M4" s="11">
         <v>-1000000</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>94</v>
       </c>
@@ -4404,22 +4419,25 @@
         <v>-10000</v>
       </c>
       <c r="H5" s="11">
+        <v>-30000</v>
+      </c>
+      <c r="I5" s="11">
         <v>-50000</v>
       </c>
-      <c r="I5" s="11">
+      <c r="J5" s="11">
         <v>-100000</v>
       </c>
-      <c r="J5" s="11">
+      <c r="K5" s="11">
         <v>-200000</v>
       </c>
-      <c r="K5" s="11">
+      <c r="L5" s="11">
         <v>-500000</v>
       </c>
-      <c r="L5" s="11">
+      <c r="M5" s="11">
         <v>-1000000</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>95</v>
       </c>
@@ -4442,22 +4460,25 @@
         <v>-10000</v>
       </c>
       <c r="H6" s="11">
+        <v>-30000</v>
+      </c>
+      <c r="I6" s="11">
         <v>-50000</v>
       </c>
-      <c r="I6" s="11">
+      <c r="J6" s="11">
         <v>-100000</v>
       </c>
-      <c r="J6" s="11">
+      <c r="K6" s="11">
         <v>-200000</v>
       </c>
-      <c r="K6" s="11">
+      <c r="L6" s="11">
         <v>-500000</v>
       </c>
-      <c r="L6" s="11">
+      <c r="M6" s="11">
         <v>-1000000</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A7" s="11" t="s">
         <v>147</v>
       </c>
@@ -4480,22 +4501,25 @@
         <v>-10000</v>
       </c>
       <c r="H7" s="11">
+        <v>-30000</v>
+      </c>
+      <c r="I7" s="11">
         <v>-50000</v>
       </c>
-      <c r="I7" s="11">
+      <c r="J7" s="11">
         <v>-100000</v>
       </c>
-      <c r="J7" s="11">
+      <c r="K7" s="11">
         <v>-200000</v>
       </c>
-      <c r="K7" s="11">
+      <c r="L7" s="11">
         <v>-500000</v>
       </c>
-      <c r="L7" s="11">
+      <c r="M7" s="11">
         <v>-1000000</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A8" s="11" t="s">
         <v>398</v>
       </c>
@@ -4518,22 +4542,25 @@
         <v>-10000</v>
       </c>
       <c r="H8" s="11">
+        <v>-30000</v>
+      </c>
+      <c r="I8" s="11">
         <v>-50000</v>
       </c>
-      <c r="I8" s="11">
+      <c r="J8" s="11">
         <v>-100000</v>
       </c>
-      <c r="J8" s="11">
+      <c r="K8" s="11">
         <v>-200000</v>
       </c>
-      <c r="K8" s="11">
+      <c r="L8" s="11">
         <v>-500000</v>
       </c>
-      <c r="L8" s="11">
+      <c r="M8" s="11">
         <v>-1000000</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A9" s="11" t="s">
         <v>399</v>
       </c>
@@ -4556,22 +4583,25 @@
         <v>-10000</v>
       </c>
       <c r="H9" s="11">
+        <v>-30000</v>
+      </c>
+      <c r="I9" s="11">
         <v>-50000</v>
       </c>
-      <c r="I9" s="11">
+      <c r="J9" s="11">
         <v>-100000</v>
       </c>
-      <c r="J9" s="11">
+      <c r="K9" s="11">
         <v>-200000</v>
       </c>
-      <c r="K9" s="11">
+      <c r="L9" s="11">
         <v>-500000</v>
       </c>
-      <c r="L9" s="11">
+      <c r="M9" s="11">
         <v>-1000000</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A10" s="11" t="s">
         <v>400</v>
       </c>
@@ -4594,22 +4624,25 @@
         <v>-10000</v>
       </c>
       <c r="H10" s="11">
+        <v>-30000</v>
+      </c>
+      <c r="I10" s="11">
         <v>-50000</v>
       </c>
-      <c r="I10" s="11">
+      <c r="J10" s="11">
         <v>-100000</v>
       </c>
-      <c r="J10" s="11">
+      <c r="K10" s="11">
         <v>-200000</v>
       </c>
-      <c r="K10" s="11">
+      <c r="L10" s="11">
         <v>-500000</v>
       </c>
-      <c r="L10" s="11">
+      <c r="M10" s="11">
         <v>-1000000</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A11" s="11" t="s">
         <v>401</v>
       </c>
@@ -4632,22 +4665,25 @@
         <v>-10000</v>
       </c>
       <c r="H11" s="11">
+        <v>-30000</v>
+      </c>
+      <c r="I11" s="11">
         <v>-50000</v>
       </c>
-      <c r="I11" s="11">
+      <c r="J11" s="11">
         <v>-100000</v>
       </c>
-      <c r="J11" s="11">
+      <c r="K11" s="11">
         <v>-200000</v>
       </c>
-      <c r="K11" s="11">
+      <c r="L11" s="11">
         <v>-500000</v>
       </c>
-      <c r="L11" s="11">
+      <c r="M11" s="11">
         <v>-1000000</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A12" s="11" t="s">
         <v>402</v>
       </c>
@@ -4670,22 +4706,25 @@
         <v>-10000</v>
       </c>
       <c r="H12" s="11">
+        <v>-30000</v>
+      </c>
+      <c r="I12" s="11">
         <v>-50000</v>
       </c>
-      <c r="I12" s="11">
+      <c r="J12" s="11">
         <v>-100000</v>
       </c>
-      <c r="J12" s="11">
+      <c r="K12" s="11">
         <v>-200000</v>
       </c>
-      <c r="K12" s="11">
+      <c r="L12" s="11">
         <v>-500000</v>
       </c>
-      <c r="L12" s="11">
+      <c r="M12" s="11">
         <v>-1000000</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A13" s="11" t="s">
         <v>403</v>
       </c>
@@ -4708,22 +4747,25 @@
         <v>-10000</v>
       </c>
       <c r="H13" s="11">
+        <v>-30000</v>
+      </c>
+      <c r="I13" s="11">
         <v>-50000</v>
       </c>
-      <c r="I13" s="11">
+      <c r="J13" s="11">
         <v>-100000</v>
       </c>
-      <c r="J13" s="11">
+      <c r="K13" s="11">
         <v>-200000</v>
       </c>
-      <c r="K13" s="11">
+      <c r="L13" s="11">
         <v>-500000</v>
       </c>
-      <c r="L13" s="11">
+      <c r="M13" s="11">
         <v>-1000000</v>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A14" s="11" t="s">
         <v>404</v>
       </c>
@@ -4746,22 +4788,25 @@
         <v>-10000</v>
       </c>
       <c r="H14" s="11">
+        <v>-30000</v>
+      </c>
+      <c r="I14" s="11">
         <v>-50000</v>
       </c>
-      <c r="I14" s="11">
+      <c r="J14" s="11">
         <v>-100000</v>
       </c>
-      <c r="J14" s="11">
+      <c r="K14" s="11">
         <v>-200000</v>
       </c>
-      <c r="K14" s="11">
+      <c r="L14" s="11">
         <v>-500000</v>
       </c>
-      <c r="L14" s="11">
+      <c r="M14" s="11">
         <v>-1000000</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A15" s="11" t="s">
         <v>405</v>
       </c>
@@ -4784,22 +4829,25 @@
         <v>-10000</v>
       </c>
       <c r="H15" s="11">
+        <v>-30000</v>
+      </c>
+      <c r="I15" s="11">
         <v>-50000</v>
       </c>
-      <c r="I15" s="11">
+      <c r="J15" s="11">
         <v>-100000</v>
       </c>
-      <c r="J15" s="11">
+      <c r="K15" s="11">
         <v>-200000</v>
       </c>
-      <c r="K15" s="11">
+      <c r="L15" s="11">
         <v>-500000</v>
       </c>
-      <c r="L15" s="11">
+      <c r="M15" s="11">
         <v>-1000000</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A16" s="11" t="s">
         <v>406</v>
       </c>
@@ -4822,18 +4870,21 @@
         <v>-10000</v>
       </c>
       <c r="H16" s="11">
+        <v>-30000</v>
+      </c>
+      <c r="I16" s="11">
         <v>-50000</v>
       </c>
-      <c r="I16" s="11">
+      <c r="J16" s="11">
         <v>-100000</v>
       </c>
-      <c r="J16" s="11">
+      <c r="K16" s="11">
         <v>-200000</v>
       </c>
-      <c r="K16" s="11">
+      <c r="L16" s="11">
         <v>-500000</v>
       </c>
-      <c r="L16" s="11">
+      <c r="M16" s="11">
         <v>-1000000</v>
       </c>
     </row>
@@ -4870,16 +4921,17 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
-  <dimension ref="A1:AC51"/>
+  <dimension ref="A1:AD51"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="12.265625" bestFit="1" customWidth="1"/>
     <col min="3" max="4" width="10.9296875" style="11" customWidth="1"/>
     <col min="6" max="6" width="10.59765625" style="11" customWidth="1"/>
-    <col min="10" max="10" width="10.9296875" style="11" customWidth="1"/>
+    <col min="9" max="9" width="10.6640625" style="11"/>
+    <col min="11" max="11" width="10.9296875" style="11" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:29" x14ac:dyDescent="0.45">
       <c r="A1" s="11" t="s">
         <v>89</v>
       </c>
@@ -4919,8 +4971,11 @@
       <c r="M1" s="11" t="s">
         <v>123</v>
       </c>
-    </row>
-    <row r="2" spans="1:28" x14ac:dyDescent="0.45">
+      <c r="N1" s="11" t="s">
+        <v>1216</v>
+      </c>
+    </row>
+    <row r="2" spans="1:29" x14ac:dyDescent="0.45">
       <c r="A2" s="11" t="s">
         <v>91</v>
       </c>
@@ -4960,7 +5015,9 @@
       <c r="M2" s="11">
         <v>0</v>
       </c>
-      <c r="P2" s="11"/>
+      <c r="N2" s="11">
+        <v>0</v>
+      </c>
       <c r="Q2" s="11"/>
       <c r="R2" s="11"/>
       <c r="S2" s="11"/>
@@ -4973,8 +5030,9 @@
       <c r="Z2" s="11"/>
       <c r="AA2" s="11"/>
       <c r="AB2" s="11"/>
-    </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.45">
+      <c r="AC2" s="11"/>
+    </row>
+    <row r="3" spans="1:29" x14ac:dyDescent="0.45">
       <c r="A3" s="11" t="s">
         <v>91</v>
       </c>
@@ -5000,21 +5058,23 @@
         <v>-10000</v>
       </c>
       <c r="I3" s="11">
+        <v>-30000</v>
+      </c>
+      <c r="J3" s="11">
         <v>-50000</v>
       </c>
-      <c r="J3" s="11">
+      <c r="K3" s="11">
         <v>-100000</v>
       </c>
-      <c r="K3" s="11">
+      <c r="L3" s="11">
         <v>-200000</v>
       </c>
-      <c r="L3" s="11">
+      <c r="M3" s="11">
         <v>-500000</v>
       </c>
-      <c r="M3" s="11">
+      <c r="N3" s="11">
         <v>-1000000</v>
       </c>
-      <c r="O3" s="11"/>
       <c r="P3" s="11"/>
       <c r="Q3" s="11"/>
       <c r="R3" s="11"/>
@@ -5028,8 +5088,9 @@
       <c r="Z3" s="11"/>
       <c r="AA3" s="11"/>
       <c r="AB3" s="11"/>
-    </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.45">
+      <c r="AC3" s="11"/>
+    </row>
+    <row r="4" spans="1:29" x14ac:dyDescent="0.45">
       <c r="A4" s="11" t="s">
         <v>91</v>
       </c>
@@ -5055,21 +5116,23 @@
         <v>-10000</v>
       </c>
       <c r="I4" s="11">
+        <v>-30000</v>
+      </c>
+      <c r="J4" s="11">
         <v>-50000</v>
       </c>
-      <c r="J4" s="11">
+      <c r="K4" s="11">
         <v>-100000</v>
       </c>
-      <c r="K4" s="11">
+      <c r="L4" s="11">
         <v>-200000</v>
       </c>
-      <c r="L4" s="11">
+      <c r="M4" s="11">
         <v>-500000</v>
       </c>
-      <c r="M4" s="11">
+      <c r="N4" s="11">
         <v>-1000000</v>
       </c>
-      <c r="O4" s="11"/>
       <c r="P4" s="11"/>
       <c r="Q4" s="11"/>
       <c r="R4" s="11"/>
@@ -5083,8 +5146,9 @@
       <c r="Z4" s="11"/>
       <c r="AA4" s="11"/>
       <c r="AB4" s="11"/>
-    </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.45">
+      <c r="AC4" s="11"/>
+    </row>
+    <row r="5" spans="1:29" x14ac:dyDescent="0.45">
       <c r="A5" s="11" t="s">
         <v>92</v>
       </c>
@@ -5124,7 +5188,9 @@
       <c r="M5" s="11">
         <v>0</v>
       </c>
-      <c r="O5" s="11"/>
+      <c r="N5" s="11">
+        <v>0</v>
+      </c>
       <c r="P5" s="11"/>
       <c r="Q5" s="11"/>
       <c r="R5" s="11"/>
@@ -5138,8 +5204,9 @@
       <c r="Z5" s="11"/>
       <c r="AA5" s="11"/>
       <c r="AB5" s="11"/>
-    </row>
-    <row r="6" spans="1:28" x14ac:dyDescent="0.45">
+      <c r="AC5" s="11"/>
+    </row>
+    <row r="6" spans="1:29" x14ac:dyDescent="0.45">
       <c r="A6" s="11" t="s">
         <v>92</v>
       </c>
@@ -5165,21 +5232,23 @@
         <v>-10000</v>
       </c>
       <c r="I6" s="11">
+        <v>-30000</v>
+      </c>
+      <c r="J6" s="11">
         <v>-50000</v>
       </c>
-      <c r="J6" s="11">
+      <c r="K6" s="11">
         <v>-100000</v>
       </c>
-      <c r="K6" s="11">
+      <c r="L6" s="11">
         <v>-200000</v>
       </c>
-      <c r="L6" s="11">
+      <c r="M6" s="11">
         <v>-500000</v>
       </c>
-      <c r="M6" s="11">
+      <c r="N6" s="11">
         <v>-1000000</v>
       </c>
-      <c r="O6" s="11"/>
       <c r="P6" s="11"/>
       <c r="Q6" s="11"/>
       <c r="R6" s="11"/>
@@ -5193,8 +5262,9 @@
       <c r="Z6" s="11"/>
       <c r="AA6" s="11"/>
       <c r="AB6" s="11"/>
-    </row>
-    <row r="7" spans="1:28" x14ac:dyDescent="0.45">
+      <c r="AC6" s="11"/>
+    </row>
+    <row r="7" spans="1:29" x14ac:dyDescent="0.45">
       <c r="A7" s="11" t="s">
         <v>92</v>
       </c>
@@ -5220,21 +5290,23 @@
         <v>-10000</v>
       </c>
       <c r="I7" s="11">
+        <v>-30000</v>
+      </c>
+      <c r="J7" s="11">
         <v>-50000</v>
       </c>
-      <c r="J7" s="11">
+      <c r="K7" s="11">
         <v>-100000</v>
       </c>
-      <c r="K7" s="11">
+      <c r="L7" s="11">
         <v>-200000</v>
       </c>
-      <c r="L7" s="11">
+      <c r="M7" s="11">
         <v>-500000</v>
       </c>
-      <c r="M7" s="11">
+      <c r="N7" s="11">
         <v>-1000000</v>
       </c>
-      <c r="O7" s="11"/>
       <c r="P7" s="11"/>
       <c r="Q7" s="11"/>
       <c r="R7" s="11"/>
@@ -5248,8 +5320,9 @@
       <c r="Z7" s="11"/>
       <c r="AA7" s="11"/>
       <c r="AB7" s="11"/>
-    </row>
-    <row r="8" spans="1:28" x14ac:dyDescent="0.45">
+      <c r="AC7" s="11"/>
+    </row>
+    <row r="8" spans="1:29" x14ac:dyDescent="0.45">
       <c r="A8" s="11" t="s">
         <v>93</v>
       </c>
@@ -5289,7 +5362,9 @@
       <c r="M8" s="11">
         <v>0</v>
       </c>
-      <c r="O8" s="11"/>
+      <c r="N8" s="11">
+        <v>0</v>
+      </c>
       <c r="P8" s="11"/>
       <c r="Q8" s="11"/>
       <c r="R8" s="11"/>
@@ -5303,8 +5378,9 @@
       <c r="Z8" s="11"/>
       <c r="AA8" s="11"/>
       <c r="AB8" s="11"/>
-    </row>
-    <row r="9" spans="1:28" x14ac:dyDescent="0.45">
+      <c r="AC8" s="11"/>
+    </row>
+    <row r="9" spans="1:29" x14ac:dyDescent="0.45">
       <c r="A9" s="11" t="s">
         <v>93</v>
       </c>
@@ -5330,21 +5406,23 @@
         <v>-10000</v>
       </c>
       <c r="I9" s="11">
+        <v>-30000</v>
+      </c>
+      <c r="J9" s="11">
         <v>-50000</v>
       </c>
-      <c r="J9" s="11">
+      <c r="K9" s="11">
         <v>-100000</v>
       </c>
-      <c r="K9" s="11">
+      <c r="L9" s="11">
         <v>-200000</v>
       </c>
-      <c r="L9" s="11">
+      <c r="M9" s="11">
         <v>-500000</v>
       </c>
-      <c r="M9" s="11">
+      <c r="N9" s="11">
         <v>-1000000</v>
       </c>
-      <c r="O9" s="11"/>
       <c r="P9" s="11"/>
       <c r="Q9" s="11"/>
       <c r="R9" s="11"/>
@@ -5358,8 +5436,9 @@
       <c r="Z9" s="11"/>
       <c r="AA9" s="11"/>
       <c r="AB9" s="11"/>
-    </row>
-    <row r="10" spans="1:28" x14ac:dyDescent="0.45">
+      <c r="AC9" s="11"/>
+    </row>
+    <row r="10" spans="1:29" x14ac:dyDescent="0.45">
       <c r="A10" s="11" t="s">
         <v>93</v>
       </c>
@@ -5385,21 +5464,23 @@
         <v>-10000</v>
       </c>
       <c r="I10" s="11">
+        <v>-30000</v>
+      </c>
+      <c r="J10" s="11">
         <v>-50000</v>
       </c>
-      <c r="J10" s="11">
+      <c r="K10" s="11">
         <v>-100000</v>
       </c>
-      <c r="K10" s="11">
+      <c r="L10" s="11">
         <v>-200000</v>
       </c>
-      <c r="L10" s="11">
+      <c r="M10" s="11">
         <v>-500000</v>
       </c>
-      <c r="M10" s="11">
+      <c r="N10" s="11">
         <v>-1000000</v>
       </c>
-      <c r="O10" s="11"/>
       <c r="P10" s="11"/>
       <c r="Q10" s="11"/>
       <c r="R10" s="11"/>
@@ -5413,8 +5494,9 @@
       <c r="Z10" s="11"/>
       <c r="AA10" s="11"/>
       <c r="AB10" s="11"/>
-    </row>
-    <row r="11" spans="1:28" x14ac:dyDescent="0.45">
+      <c r="AC10" s="11"/>
+    </row>
+    <row r="11" spans="1:29" x14ac:dyDescent="0.45">
       <c r="A11" s="11" t="s">
         <v>94</v>
       </c>
@@ -5454,7 +5536,9 @@
       <c r="M11" s="11">
         <v>0</v>
       </c>
-      <c r="O11" s="11"/>
+      <c r="N11" s="11">
+        <v>0</v>
+      </c>
       <c r="P11" s="11"/>
       <c r="Q11" s="11"/>
       <c r="R11" s="11"/>
@@ -5468,8 +5552,9 @@
       <c r="Z11" s="11"/>
       <c r="AA11" s="11"/>
       <c r="AB11" s="11"/>
-    </row>
-    <row r="12" spans="1:28" x14ac:dyDescent="0.45">
+      <c r="AC11" s="11"/>
+    </row>
+    <row r="12" spans="1:29" x14ac:dyDescent="0.45">
       <c r="A12" s="11" t="s">
         <v>94</v>
       </c>
@@ -5495,21 +5580,23 @@
         <v>-10000</v>
       </c>
       <c r="I12" s="11">
+        <v>-30000</v>
+      </c>
+      <c r="J12" s="11">
         <v>-50000</v>
       </c>
-      <c r="J12" s="11">
+      <c r="K12" s="11">
         <v>-100000</v>
       </c>
-      <c r="K12" s="11">
+      <c r="L12" s="11">
         <v>-200000</v>
       </c>
-      <c r="L12" s="11">
+      <c r="M12" s="11">
         <v>-500000</v>
       </c>
-      <c r="M12" s="11">
+      <c r="N12" s="11">
         <v>-1000000</v>
       </c>
-      <c r="O12" s="11"/>
       <c r="P12" s="11"/>
       <c r="Q12" s="11"/>
       <c r="R12" s="11"/>
@@ -5523,8 +5610,9 @@
       <c r="Z12" s="11"/>
       <c r="AA12" s="11"/>
       <c r="AB12" s="11"/>
-    </row>
-    <row r="13" spans="1:28" x14ac:dyDescent="0.45">
+      <c r="AC12" s="11"/>
+    </row>
+    <row r="13" spans="1:29" x14ac:dyDescent="0.45">
       <c r="A13" s="11" t="s">
         <v>94</v>
       </c>
@@ -5550,21 +5638,23 @@
         <v>-10000</v>
       </c>
       <c r="I13" s="11">
+        <v>-30000</v>
+      </c>
+      <c r="J13" s="11">
         <v>-50000</v>
       </c>
-      <c r="J13" s="11">
+      <c r="K13" s="11">
         <v>-100000</v>
       </c>
-      <c r="K13" s="11">
+      <c r="L13" s="11">
         <v>-200000</v>
       </c>
-      <c r="L13" s="11">
+      <c r="M13" s="11">
         <v>-500000</v>
       </c>
-      <c r="M13" s="11">
+      <c r="N13" s="11">
         <v>-1000000</v>
       </c>
-      <c r="O13" s="11"/>
       <c r="P13" s="11"/>
       <c r="Q13" s="11"/>
       <c r="R13" s="11"/>
@@ -5578,8 +5668,9 @@
       <c r="Z13" s="11"/>
       <c r="AA13" s="11"/>
       <c r="AB13" s="11"/>
-    </row>
-    <row r="14" spans="1:28" x14ac:dyDescent="0.45">
+      <c r="AC13" s="11"/>
+    </row>
+    <row r="14" spans="1:29" x14ac:dyDescent="0.45">
       <c r="A14" s="11" t="s">
         <v>95</v>
       </c>
@@ -5619,7 +5710,9 @@
       <c r="M14" s="11">
         <v>0</v>
       </c>
-      <c r="O14" s="11"/>
+      <c r="N14" s="11">
+        <v>0</v>
+      </c>
       <c r="P14" s="11"/>
       <c r="Q14" s="11"/>
       <c r="R14" s="11"/>
@@ -5633,8 +5726,9 @@
       <c r="Z14" s="11"/>
       <c r="AA14" s="11"/>
       <c r="AB14" s="11"/>
-    </row>
-    <row r="15" spans="1:28" x14ac:dyDescent="0.45">
+      <c r="AC14" s="11"/>
+    </row>
+    <row r="15" spans="1:29" x14ac:dyDescent="0.45">
       <c r="A15" s="11" t="s">
         <v>95</v>
       </c>
@@ -5660,21 +5754,23 @@
         <v>-10000</v>
       </c>
       <c r="I15" s="11">
+        <v>-30000</v>
+      </c>
+      <c r="J15" s="11">
         <v>-50000</v>
       </c>
-      <c r="J15" s="11">
+      <c r="K15" s="11">
         <v>-100000</v>
       </c>
-      <c r="K15" s="11">
+      <c r="L15" s="11">
         <v>-200000</v>
       </c>
-      <c r="L15" s="11">
+      <c r="M15" s="11">
         <v>-500000</v>
       </c>
-      <c r="M15" s="11">
+      <c r="N15" s="11">
         <v>-1000000</v>
       </c>
-      <c r="O15" s="11"/>
       <c r="P15" s="11"/>
       <c r="Q15" s="11"/>
       <c r="R15" s="11"/>
@@ -5688,8 +5784,9 @@
       <c r="Z15" s="11"/>
       <c r="AA15" s="11"/>
       <c r="AB15" s="11"/>
-    </row>
-    <row r="16" spans="1:28" x14ac:dyDescent="0.45">
+      <c r="AC15" s="11"/>
+    </row>
+    <row r="16" spans="1:29" x14ac:dyDescent="0.45">
       <c r="A16" s="11" t="s">
         <v>95</v>
       </c>
@@ -5715,21 +5812,23 @@
         <v>-10000</v>
       </c>
       <c r="I16" s="11">
+        <v>-30000</v>
+      </c>
+      <c r="J16" s="11">
         <v>-50000</v>
       </c>
-      <c r="J16" s="11">
+      <c r="K16" s="11">
         <v>-100000</v>
       </c>
-      <c r="K16" s="11">
+      <c r="L16" s="11">
         <v>-200000</v>
       </c>
-      <c r="L16" s="11">
+      <c r="M16" s="11">
         <v>-500000</v>
       </c>
-      <c r="M16" s="11">
+      <c r="N16" s="11">
         <v>-1000000</v>
       </c>
-      <c r="O16" s="11"/>
       <c r="P16" s="11"/>
       <c r="Q16" s="11"/>
       <c r="R16" s="11"/>
@@ -5743,8 +5842,9 @@
       <c r="Z16" s="11"/>
       <c r="AA16" s="11"/>
       <c r="AB16" s="11"/>
-    </row>
-    <row r="17" spans="1:28" x14ac:dyDescent="0.45">
+      <c r="AC16" s="11"/>
+    </row>
+    <row r="17" spans="1:29" x14ac:dyDescent="0.45">
       <c r="A17" s="11" t="s">
         <v>147</v>
       </c>
@@ -5784,7 +5884,9 @@
       <c r="M17" s="11">
         <v>0</v>
       </c>
-      <c r="O17" s="11"/>
+      <c r="N17" s="11">
+        <v>0</v>
+      </c>
       <c r="P17" s="11"/>
       <c r="Q17" s="11"/>
       <c r="R17" s="11"/>
@@ -5798,8 +5900,9 @@
       <c r="Z17" s="11"/>
       <c r="AA17" s="11"/>
       <c r="AB17" s="11"/>
-    </row>
-    <row r="18" spans="1:28" x14ac:dyDescent="0.45">
+      <c r="AC17" s="11"/>
+    </row>
+    <row r="18" spans="1:29" x14ac:dyDescent="0.45">
       <c r="A18" s="11" t="s">
         <v>147</v>
       </c>
@@ -5825,22 +5928,24 @@
         <v>-10000</v>
       </c>
       <c r="I18" s="11">
+        <v>-30000</v>
+      </c>
+      <c r="J18" s="11">
         <v>-50000</v>
       </c>
-      <c r="J18" s="11">
+      <c r="K18" s="11">
         <v>-100000</v>
       </c>
-      <c r="K18" s="11">
+      <c r="L18" s="11">
         <v>-200000</v>
       </c>
-      <c r="L18" s="11">
+      <c r="M18" s="11">
         <v>-500000</v>
       </c>
-      <c r="M18" s="11">
+      <c r="N18" s="11">
         <v>-1000000</v>
       </c>
-      <c r="N18" s="2"/>
-      <c r="O18" s="11"/>
+      <c r="O18" s="2"/>
       <c r="P18" s="11"/>
       <c r="Q18" s="11"/>
       <c r="R18" s="11"/>
@@ -5854,8 +5959,9 @@
       <c r="Z18" s="11"/>
       <c r="AA18" s="11"/>
       <c r="AB18" s="11"/>
-    </row>
-    <row r="19" spans="1:28" x14ac:dyDescent="0.45">
+      <c r="AC18" s="11"/>
+    </row>
+    <row r="19" spans="1:29" x14ac:dyDescent="0.45">
       <c r="A19" s="11" t="s">
         <v>147</v>
       </c>
@@ -5881,21 +5987,23 @@
         <v>-10000</v>
       </c>
       <c r="I19" s="11">
+        <v>-30000</v>
+      </c>
+      <c r="J19" s="11">
         <v>-50000</v>
       </c>
-      <c r="J19" s="11">
+      <c r="K19" s="11">
         <v>-100000</v>
       </c>
-      <c r="K19" s="11">
+      <c r="L19" s="11">
         <v>-200000</v>
       </c>
-      <c r="L19" s="11">
+      <c r="M19" s="11">
         <v>-500000</v>
       </c>
-      <c r="M19" s="11">
+      <c r="N19" s="11">
         <v>-1000000</v>
       </c>
-      <c r="O19" s="11"/>
       <c r="P19" s="11"/>
       <c r="Q19" s="11"/>
       <c r="R19" s="11"/>
@@ -5909,8 +6017,9 @@
       <c r="Z19" s="11"/>
       <c r="AA19" s="11"/>
       <c r="AB19" s="11"/>
-    </row>
-    <row r="20" spans="1:28" x14ac:dyDescent="0.45">
+      <c r="AC19" s="11"/>
+    </row>
+    <row r="20" spans="1:29" x14ac:dyDescent="0.45">
       <c r="A20" s="11" t="s">
         <v>398</v>
       </c>
@@ -5950,7 +6059,9 @@
       <c r="M20" s="11">
         <v>0</v>
       </c>
-      <c r="O20" s="11"/>
+      <c r="N20" s="11">
+        <v>0</v>
+      </c>
       <c r="P20" s="11"/>
       <c r="Q20" s="11"/>
       <c r="R20" s="11"/>
@@ -5964,8 +6075,9 @@
       <c r="Z20" s="11"/>
       <c r="AA20" s="11"/>
       <c r="AB20" s="11"/>
-    </row>
-    <row r="21" spans="1:28" x14ac:dyDescent="0.45">
+      <c r="AC20" s="11"/>
+    </row>
+    <row r="21" spans="1:29" x14ac:dyDescent="0.45">
       <c r="A21" s="11" t="s">
         <v>398</v>
       </c>
@@ -5991,21 +6103,23 @@
         <v>-10000</v>
       </c>
       <c r="I21" s="11">
+        <v>-30000</v>
+      </c>
+      <c r="J21" s="11">
         <v>-50000</v>
       </c>
-      <c r="J21" s="11">
+      <c r="K21" s="11">
         <v>-100000</v>
       </c>
-      <c r="K21" s="11">
+      <c r="L21" s="11">
         <v>-200000</v>
       </c>
-      <c r="L21" s="11">
+      <c r="M21" s="11">
         <v>-500000</v>
       </c>
-      <c r="M21" s="11">
+      <c r="N21" s="11">
         <v>-1000000</v>
       </c>
-      <c r="O21" s="11"/>
       <c r="P21" s="11"/>
       <c r="Q21" s="11"/>
       <c r="R21" s="11"/>
@@ -6019,8 +6133,9 @@
       <c r="Z21" s="11"/>
       <c r="AA21" s="11"/>
       <c r="AB21" s="11"/>
-    </row>
-    <row r="22" spans="1:28" x14ac:dyDescent="0.45">
+      <c r="AC21" s="11"/>
+    </row>
+    <row r="22" spans="1:29" x14ac:dyDescent="0.45">
       <c r="A22" s="11" t="s">
         <v>398</v>
       </c>
@@ -6046,21 +6161,23 @@
         <v>-10000</v>
       </c>
       <c r="I22" s="11">
+        <v>-30000</v>
+      </c>
+      <c r="J22" s="11">
         <v>-50000</v>
       </c>
-      <c r="J22" s="11">
+      <c r="K22" s="11">
         <v>-100000</v>
       </c>
-      <c r="K22" s="11">
+      <c r="L22" s="11">
         <v>-200000</v>
       </c>
-      <c r="L22" s="11">
+      <c r="M22" s="11">
         <v>-500000</v>
       </c>
-      <c r="M22" s="11">
+      <c r="N22" s="11">
         <v>-1000000</v>
       </c>
-      <c r="O22" s="11"/>
       <c r="P22" s="11"/>
       <c r="Q22" s="11"/>
       <c r="R22" s="11"/>
@@ -6074,8 +6191,9 @@
       <c r="Z22" s="11"/>
       <c r="AA22" s="11"/>
       <c r="AB22" s="11"/>
-    </row>
-    <row r="23" spans="1:28" x14ac:dyDescent="0.45">
+      <c r="AC22" s="11"/>
+    </row>
+    <row r="23" spans="1:29" x14ac:dyDescent="0.45">
       <c r="A23" s="11" t="s">
         <v>399</v>
       </c>
@@ -6115,7 +6233,9 @@
       <c r="M23" s="11">
         <v>0</v>
       </c>
-      <c r="O23" s="11"/>
+      <c r="N23" s="11">
+        <v>0</v>
+      </c>
       <c r="P23" s="11"/>
       <c r="Q23" s="11"/>
       <c r="R23" s="11"/>
@@ -6129,8 +6249,9 @@
       <c r="Z23" s="11"/>
       <c r="AA23" s="11"/>
       <c r="AB23" s="11"/>
-    </row>
-    <row r="24" spans="1:28" x14ac:dyDescent="0.45">
+      <c r="AC23" s="11"/>
+    </row>
+    <row r="24" spans="1:29" x14ac:dyDescent="0.45">
       <c r="A24" s="11" t="s">
         <v>399</v>
       </c>
@@ -6156,21 +6277,23 @@
         <v>-10000</v>
       </c>
       <c r="I24" s="11">
+        <v>-30000</v>
+      </c>
+      <c r="J24" s="11">
         <v>-50000</v>
       </c>
-      <c r="J24" s="11">
+      <c r="K24" s="11">
         <v>-100000</v>
       </c>
-      <c r="K24" s="11">
+      <c r="L24" s="11">
         <v>-200000</v>
       </c>
-      <c r="L24" s="11">
+      <c r="M24" s="11">
         <v>-500000</v>
       </c>
-      <c r="M24" s="11">
+      <c r="N24" s="11">
         <v>-1000000</v>
       </c>
-      <c r="O24" s="11"/>
       <c r="P24" s="11"/>
       <c r="Q24" s="11"/>
       <c r="R24" s="11"/>
@@ -6184,8 +6307,9 @@
       <c r="Z24" s="11"/>
       <c r="AA24" s="11"/>
       <c r="AB24" s="11"/>
-    </row>
-    <row r="25" spans="1:28" x14ac:dyDescent="0.45">
+      <c r="AC24" s="11"/>
+    </row>
+    <row r="25" spans="1:29" x14ac:dyDescent="0.45">
       <c r="A25" s="11" t="s">
         <v>399</v>
       </c>
@@ -6211,21 +6335,23 @@
         <v>-10000</v>
       </c>
       <c r="I25" s="11">
+        <v>-30000</v>
+      </c>
+      <c r="J25" s="11">
         <v>-50000</v>
       </c>
-      <c r="J25" s="11">
+      <c r="K25" s="11">
         <v>-100000</v>
       </c>
-      <c r="K25" s="11">
+      <c r="L25" s="11">
         <v>-200000</v>
       </c>
-      <c r="L25" s="11">
+      <c r="M25" s="11">
         <v>-500000</v>
       </c>
-      <c r="M25" s="11">
+      <c r="N25" s="11">
         <v>-1000000</v>
       </c>
-      <c r="O25" s="11"/>
       <c r="P25" s="11"/>
       <c r="Q25" s="11"/>
       <c r="R25" s="11"/>
@@ -6239,8 +6365,9 @@
       <c r="Z25" s="11"/>
       <c r="AA25" s="11"/>
       <c r="AB25" s="11"/>
-    </row>
-    <row r="26" spans="1:28" x14ac:dyDescent="0.45">
+      <c r="AC25" s="11"/>
+    </row>
+    <row r="26" spans="1:29" x14ac:dyDescent="0.45">
       <c r="A26" s="11" t="s">
         <v>400</v>
       </c>
@@ -6280,7 +6407,9 @@
       <c r="M26" s="11">
         <v>0</v>
       </c>
-      <c r="O26" s="11"/>
+      <c r="N26" s="11">
+        <v>0</v>
+      </c>
       <c r="P26" s="11"/>
       <c r="Q26" s="11"/>
       <c r="R26" s="11"/>
@@ -6294,8 +6423,9 @@
       <c r="Z26" s="11"/>
       <c r="AA26" s="11"/>
       <c r="AB26" s="11"/>
-    </row>
-    <row r="27" spans="1:28" x14ac:dyDescent="0.45">
+      <c r="AC26" s="11"/>
+    </row>
+    <row r="27" spans="1:29" x14ac:dyDescent="0.45">
       <c r="A27" s="11" t="s">
         <v>400</v>
       </c>
@@ -6321,21 +6451,23 @@
         <v>-10000</v>
       </c>
       <c r="I27" s="11">
+        <v>-30000</v>
+      </c>
+      <c r="J27" s="11">
         <v>-50000</v>
       </c>
-      <c r="J27" s="11">
+      <c r="K27" s="11">
         <v>-100000</v>
       </c>
-      <c r="K27" s="11">
+      <c r="L27" s="11">
         <v>-200000</v>
       </c>
-      <c r="L27" s="11">
+      <c r="M27" s="11">
         <v>-500000</v>
       </c>
-      <c r="M27" s="11">
+      <c r="N27" s="11">
         <v>-1000000</v>
       </c>
-      <c r="O27" s="11"/>
       <c r="P27" s="11"/>
       <c r="Q27" s="11"/>
       <c r="R27" s="11"/>
@@ -6349,8 +6481,9 @@
       <c r="Z27" s="11"/>
       <c r="AA27" s="11"/>
       <c r="AB27" s="11"/>
-    </row>
-    <row r="28" spans="1:28" x14ac:dyDescent="0.45">
+      <c r="AC27" s="11"/>
+    </row>
+    <row r="28" spans="1:29" x14ac:dyDescent="0.45">
       <c r="A28" s="11" t="s">
         <v>400</v>
       </c>
@@ -6376,21 +6509,23 @@
         <v>-10000</v>
       </c>
       <c r="I28" s="11">
+        <v>-30000</v>
+      </c>
+      <c r="J28" s="11">
         <v>-50000</v>
       </c>
-      <c r="J28" s="11">
+      <c r="K28" s="11">
         <v>-100000</v>
       </c>
-      <c r="K28" s="11">
+      <c r="L28" s="11">
         <v>-200000</v>
       </c>
-      <c r="L28" s="11">
+      <c r="M28" s="11">
         <v>-500000</v>
       </c>
-      <c r="M28" s="11">
+      <c r="N28" s="11">
         <v>-1000000</v>
       </c>
-      <c r="O28" s="11"/>
       <c r="P28" s="11"/>
       <c r="Q28" s="11"/>
       <c r="R28" s="11"/>
@@ -6404,8 +6539,9 @@
       <c r="Z28" s="11"/>
       <c r="AA28" s="11"/>
       <c r="AB28" s="11"/>
-    </row>
-    <row r="29" spans="1:28" x14ac:dyDescent="0.45">
+      <c r="AC28" s="11"/>
+    </row>
+    <row r="29" spans="1:29" x14ac:dyDescent="0.45">
       <c r="A29" s="11" t="s">
         <v>401</v>
       </c>
@@ -6445,7 +6581,9 @@
       <c r="M29" s="11">
         <v>0</v>
       </c>
-      <c r="O29" s="11"/>
+      <c r="N29" s="11">
+        <v>0</v>
+      </c>
       <c r="P29" s="11"/>
       <c r="Q29" s="11"/>
       <c r="R29" s="11"/>
@@ -6459,8 +6597,9 @@
       <c r="Z29" s="11"/>
       <c r="AA29" s="11"/>
       <c r="AB29" s="11"/>
-    </row>
-    <row r="30" spans="1:28" x14ac:dyDescent="0.45">
+      <c r="AC29" s="11"/>
+    </row>
+    <row r="30" spans="1:29" x14ac:dyDescent="0.45">
       <c r="A30" s="11" t="s">
         <v>401</v>
       </c>
@@ -6486,21 +6625,23 @@
         <v>-10000</v>
       </c>
       <c r="I30" s="11">
+        <v>-30000</v>
+      </c>
+      <c r="J30" s="11">
         <v>-50000</v>
       </c>
-      <c r="J30" s="11">
+      <c r="K30" s="11">
         <v>-100000</v>
       </c>
-      <c r="K30" s="11">
+      <c r="L30" s="11">
         <v>-200000</v>
       </c>
-      <c r="L30" s="11">
+      <c r="M30" s="11">
         <v>-500000</v>
       </c>
-      <c r="M30" s="11">
+      <c r="N30" s="11">
         <v>-1000000</v>
       </c>
-      <c r="O30" s="11"/>
       <c r="P30" s="11"/>
       <c r="Q30" s="11"/>
       <c r="R30" s="11"/>
@@ -6514,8 +6655,9 @@
       <c r="Z30" s="11"/>
       <c r="AA30" s="11"/>
       <c r="AB30" s="11"/>
-    </row>
-    <row r="31" spans="1:28" x14ac:dyDescent="0.45">
+      <c r="AC30" s="11"/>
+    </row>
+    <row r="31" spans="1:29" x14ac:dyDescent="0.45">
       <c r="A31" s="11" t="s">
         <v>401</v>
       </c>
@@ -6541,21 +6683,23 @@
         <v>-10000</v>
       </c>
       <c r="I31" s="11">
+        <v>-30000</v>
+      </c>
+      <c r="J31" s="11">
         <v>-50000</v>
       </c>
-      <c r="J31" s="11">
+      <c r="K31" s="11">
         <v>-100000</v>
       </c>
-      <c r="K31" s="11">
+      <c r="L31" s="11">
         <v>-200000</v>
       </c>
-      <c r="L31" s="11">
+      <c r="M31" s="11">
         <v>-500000</v>
       </c>
-      <c r="M31" s="11">
+      <c r="N31" s="11">
         <v>-1000000</v>
       </c>
-      <c r="O31" s="11"/>
       <c r="P31" s="11"/>
       <c r="Q31" s="11"/>
       <c r="R31" s="11"/>
@@ -6569,8 +6713,9 @@
       <c r="Z31" s="11"/>
       <c r="AA31" s="11"/>
       <c r="AB31" s="11"/>
-    </row>
-    <row r="32" spans="1:28" x14ac:dyDescent="0.45">
+      <c r="AC31" s="11"/>
+    </row>
+    <row r="32" spans="1:29" x14ac:dyDescent="0.45">
       <c r="A32" s="11" t="s">
         <v>402</v>
       </c>
@@ -6610,7 +6755,9 @@
       <c r="M32" s="11">
         <v>0</v>
       </c>
-      <c r="O32" s="11"/>
+      <c r="N32" s="11">
+        <v>0</v>
+      </c>
       <c r="P32" s="11"/>
       <c r="Q32" s="11"/>
       <c r="R32" s="11"/>
@@ -6624,8 +6771,9 @@
       <c r="Z32" s="11"/>
       <c r="AA32" s="11"/>
       <c r="AB32" s="11"/>
-    </row>
-    <row r="33" spans="1:29" x14ac:dyDescent="0.45">
+      <c r="AC32" s="11"/>
+    </row>
+    <row r="33" spans="1:30" x14ac:dyDescent="0.45">
       <c r="A33" s="11" t="s">
         <v>402</v>
       </c>
@@ -6651,21 +6799,23 @@
         <v>-10000</v>
       </c>
       <c r="I33" s="11">
+        <v>-30000</v>
+      </c>
+      <c r="J33" s="11">
         <v>-50000</v>
       </c>
-      <c r="J33" s="11">
+      <c r="K33" s="11">
         <v>-100000</v>
       </c>
-      <c r="K33" s="11">
+      <c r="L33" s="11">
         <v>-200000</v>
       </c>
-      <c r="L33" s="11">
+      <c r="M33" s="11">
         <v>-500000</v>
       </c>
-      <c r="M33" s="11">
+      <c r="N33" s="11">
         <v>-1000000</v>
       </c>
-      <c r="O33" s="11"/>
       <c r="P33" s="11"/>
       <c r="Q33" s="11"/>
       <c r="R33" s="11"/>
@@ -6679,8 +6829,9 @@
       <c r="Z33" s="11"/>
       <c r="AA33" s="11"/>
       <c r="AB33" s="11"/>
-    </row>
-    <row r="34" spans="1:29" x14ac:dyDescent="0.45">
+      <c r="AC33" s="11"/>
+    </row>
+    <row r="34" spans="1:30" x14ac:dyDescent="0.45">
       <c r="A34" s="11" t="s">
         <v>402</v>
       </c>
@@ -6706,21 +6857,23 @@
         <v>-10000</v>
       </c>
       <c r="I34" s="11">
+        <v>-30000</v>
+      </c>
+      <c r="J34" s="11">
         <v>-50000</v>
       </c>
-      <c r="J34" s="11">
+      <c r="K34" s="11">
         <v>-100000</v>
       </c>
-      <c r="K34" s="11">
+      <c r="L34" s="11">
         <v>-200000</v>
       </c>
-      <c r="L34" s="11">
+      <c r="M34" s="11">
         <v>-500000</v>
       </c>
-      <c r="M34" s="11">
+      <c r="N34" s="11">
         <v>-1000000</v>
       </c>
-      <c r="O34" s="11"/>
       <c r="P34" s="11"/>
       <c r="Q34" s="11"/>
       <c r="R34" s="11"/>
@@ -6734,8 +6887,9 @@
       <c r="Z34" s="11"/>
       <c r="AA34" s="11"/>
       <c r="AB34" s="11"/>
-    </row>
-    <row r="35" spans="1:29" x14ac:dyDescent="0.45">
+      <c r="AC34" s="11"/>
+    </row>
+    <row r="35" spans="1:30" x14ac:dyDescent="0.45">
       <c r="A35" s="11" t="s">
         <v>403</v>
       </c>
@@ -6775,7 +6929,9 @@
       <c r="M35" s="11">
         <v>0</v>
       </c>
-      <c r="O35" s="11"/>
+      <c r="N35" s="11">
+        <v>0</v>
+      </c>
       <c r="P35" s="11"/>
       <c r="Q35" s="11"/>
       <c r="R35" s="11"/>
@@ -6790,8 +6946,9 @@
       <c r="AA35" s="11"/>
       <c r="AB35" s="11"/>
       <c r="AC35" s="11"/>
-    </row>
-    <row r="36" spans="1:29" x14ac:dyDescent="0.45">
+      <c r="AD35" s="11"/>
+    </row>
+    <row r="36" spans="1:30" x14ac:dyDescent="0.45">
       <c r="A36" s="11" t="s">
         <v>403</v>
       </c>
@@ -6817,21 +6974,23 @@
         <v>-10000</v>
       </c>
       <c r="I36" s="11">
+        <v>-30000</v>
+      </c>
+      <c r="J36" s="11">
         <v>-50000</v>
       </c>
-      <c r="J36" s="11">
+      <c r="K36" s="11">
         <v>-100000</v>
       </c>
-      <c r="K36" s="11">
+      <c r="L36" s="11">
         <v>-200000</v>
       </c>
-      <c r="L36" s="11">
+      <c r="M36" s="11">
         <v>-500000</v>
       </c>
-      <c r="M36" s="11">
+      <c r="N36" s="11">
         <v>-1000000</v>
       </c>
-      <c r="O36" s="11"/>
       <c r="P36" s="11"/>
       <c r="Q36" s="11"/>
       <c r="R36" s="11"/>
@@ -6846,8 +7005,9 @@
       <c r="AA36" s="11"/>
       <c r="AB36" s="11"/>
       <c r="AC36" s="11"/>
-    </row>
-    <row r="37" spans="1:29" x14ac:dyDescent="0.45">
+      <c r="AD36" s="11"/>
+    </row>
+    <row r="37" spans="1:30" x14ac:dyDescent="0.45">
       <c r="A37" s="11" t="s">
         <v>403</v>
       </c>
@@ -6873,21 +7033,23 @@
         <v>-10000</v>
       </c>
       <c r="I37" s="11">
+        <v>-30000</v>
+      </c>
+      <c r="J37" s="11">
         <v>-50000</v>
       </c>
-      <c r="J37" s="11">
+      <c r="K37" s="11">
         <v>-100000</v>
       </c>
-      <c r="K37" s="11">
+      <c r="L37" s="11">
         <v>-200000</v>
       </c>
-      <c r="L37" s="11">
+      <c r="M37" s="11">
         <v>-500000</v>
       </c>
-      <c r="M37" s="11">
+      <c r="N37" s="11">
         <v>-1000000</v>
       </c>
-      <c r="O37" s="11"/>
       <c r="P37" s="11"/>
       <c r="Q37" s="11"/>
       <c r="R37" s="11"/>
@@ -6902,8 +7064,9 @@
       <c r="AA37" s="11"/>
       <c r="AB37" s="11"/>
       <c r="AC37" s="11"/>
-    </row>
-    <row r="38" spans="1:29" x14ac:dyDescent="0.45">
+      <c r="AD37" s="11"/>
+    </row>
+    <row r="38" spans="1:30" x14ac:dyDescent="0.45">
       <c r="A38" s="11" t="s">
         <v>404</v>
       </c>
@@ -6943,7 +7106,9 @@
       <c r="M38" s="11">
         <v>0</v>
       </c>
-      <c r="O38" s="11"/>
+      <c r="N38" s="11">
+        <v>0</v>
+      </c>
       <c r="P38" s="11"/>
       <c r="Q38" s="11"/>
       <c r="R38" s="11"/>
@@ -6957,8 +7122,9 @@
       <c r="Z38" s="11"/>
       <c r="AA38" s="11"/>
       <c r="AB38" s="11"/>
-    </row>
-    <row r="39" spans="1:29" x14ac:dyDescent="0.45">
+      <c r="AC38" s="11"/>
+    </row>
+    <row r="39" spans="1:30" x14ac:dyDescent="0.45">
       <c r="A39" s="11" t="s">
         <v>404</v>
       </c>
@@ -6984,21 +7150,23 @@
         <v>-10000</v>
       </c>
       <c r="I39" s="11">
+        <v>-30000</v>
+      </c>
+      <c r="J39" s="11">
         <v>-50000</v>
       </c>
-      <c r="J39" s="11">
+      <c r="K39" s="11">
         <v>-100000</v>
       </c>
-      <c r="K39" s="11">
+      <c r="L39" s="11">
         <v>-200000</v>
       </c>
-      <c r="L39" s="11">
+      <c r="M39" s="11">
         <v>-500000</v>
       </c>
-      <c r="M39" s="11">
+      <c r="N39" s="11">
         <v>-1000000</v>
       </c>
-      <c r="O39" s="11"/>
       <c r="P39" s="11"/>
       <c r="Q39" s="11"/>
       <c r="R39" s="11"/>
@@ -7012,8 +7180,9 @@
       <c r="Z39" s="11"/>
       <c r="AA39" s="11"/>
       <c r="AB39" s="11"/>
-    </row>
-    <row r="40" spans="1:29" x14ac:dyDescent="0.45">
+      <c r="AC39" s="11"/>
+    </row>
+    <row r="40" spans="1:30" x14ac:dyDescent="0.45">
       <c r="A40" s="11" t="s">
         <v>404</v>
       </c>
@@ -7039,21 +7208,23 @@
         <v>-10000</v>
       </c>
       <c r="I40" s="11">
+        <v>-30000</v>
+      </c>
+      <c r="J40" s="11">
         <v>-50000</v>
       </c>
-      <c r="J40" s="11">
+      <c r="K40" s="11">
         <v>-100000</v>
       </c>
-      <c r="K40" s="11">
+      <c r="L40" s="11">
         <v>-200000</v>
       </c>
-      <c r="L40" s="11">
+      <c r="M40" s="11">
         <v>-500000</v>
       </c>
-      <c r="M40" s="11">
+      <c r="N40" s="11">
         <v>-1000000</v>
       </c>
-      <c r="O40" s="11"/>
       <c r="P40" s="11"/>
       <c r="Q40" s="11"/>
       <c r="R40" s="11"/>
@@ -7067,8 +7238,9 @@
       <c r="Z40" s="11"/>
       <c r="AA40" s="11"/>
       <c r="AB40" s="11"/>
-    </row>
-    <row r="41" spans="1:29" x14ac:dyDescent="0.45">
+      <c r="AC40" s="11"/>
+    </row>
+    <row r="41" spans="1:30" x14ac:dyDescent="0.45">
       <c r="A41" s="11" t="s">
         <v>405</v>
       </c>
@@ -7108,7 +7280,9 @@
       <c r="M41" s="11">
         <v>0</v>
       </c>
-      <c r="O41" s="11"/>
+      <c r="N41" s="11">
+        <v>0</v>
+      </c>
       <c r="P41" s="11"/>
       <c r="Q41" s="11"/>
       <c r="R41" s="11"/>
@@ -7122,8 +7296,9 @@
       <c r="Z41" s="11"/>
       <c r="AA41" s="11"/>
       <c r="AB41" s="11"/>
-    </row>
-    <row r="42" spans="1:29" x14ac:dyDescent="0.45">
+      <c r="AC41" s="11"/>
+    </row>
+    <row r="42" spans="1:30" x14ac:dyDescent="0.45">
       <c r="A42" s="11" t="s">
         <v>405</v>
       </c>
@@ -7149,21 +7324,23 @@
         <v>-10000</v>
       </c>
       <c r="I42" s="11">
+        <v>-30000</v>
+      </c>
+      <c r="J42" s="11">
         <v>-50000</v>
       </c>
-      <c r="J42" s="11">
+      <c r="K42" s="11">
         <v>-100000</v>
       </c>
-      <c r="K42" s="11">
+      <c r="L42" s="11">
         <v>-200000</v>
       </c>
-      <c r="L42" s="11">
+      <c r="M42" s="11">
         <v>-500000</v>
       </c>
-      <c r="M42" s="11">
+      <c r="N42" s="11">
         <v>-1000000</v>
       </c>
-      <c r="O42" s="11"/>
       <c r="P42" s="11"/>
       <c r="Q42" s="11"/>
       <c r="R42" s="11"/>
@@ -7177,8 +7354,9 @@
       <c r="Z42" s="11"/>
       <c r="AA42" s="11"/>
       <c r="AB42" s="11"/>
-    </row>
-    <row r="43" spans="1:29" x14ac:dyDescent="0.45">
+      <c r="AC42" s="11"/>
+    </row>
+    <row r="43" spans="1:30" x14ac:dyDescent="0.45">
       <c r="A43" s="11" t="s">
         <v>405</v>
       </c>
@@ -7204,21 +7382,23 @@
         <v>-10000</v>
       </c>
       <c r="I43" s="11">
+        <v>-30000</v>
+      </c>
+      <c r="J43" s="11">
         <v>-50000</v>
       </c>
-      <c r="J43" s="11">
+      <c r="K43" s="11">
         <v>-100000</v>
       </c>
-      <c r="K43" s="11">
+      <c r="L43" s="11">
         <v>-200000</v>
       </c>
-      <c r="L43" s="11">
+      <c r="M43" s="11">
         <v>-500000</v>
       </c>
-      <c r="M43" s="11">
+      <c r="N43" s="11">
         <v>-1000000</v>
       </c>
-      <c r="O43" s="11"/>
       <c r="P43" s="11"/>
       <c r="Q43" s="11"/>
       <c r="R43" s="11"/>
@@ -7232,8 +7412,9 @@
       <c r="Z43" s="11"/>
       <c r="AA43" s="11"/>
       <c r="AB43" s="11"/>
-    </row>
-    <row r="44" spans="1:29" x14ac:dyDescent="0.45">
+      <c r="AC43" s="11"/>
+    </row>
+    <row r="44" spans="1:30" x14ac:dyDescent="0.45">
       <c r="A44" s="11" t="s">
         <v>406</v>
       </c>
@@ -7273,7 +7454,9 @@
       <c r="M44" s="11">
         <v>0</v>
       </c>
-      <c r="O44" s="11"/>
+      <c r="N44" s="11">
+        <v>0</v>
+      </c>
       <c r="P44" s="11"/>
       <c r="Q44" s="11"/>
       <c r="R44" s="11"/>
@@ -7287,8 +7470,9 @@
       <c r="Z44" s="11"/>
       <c r="AA44" s="11"/>
       <c r="AB44" s="11"/>
-    </row>
-    <row r="45" spans="1:29" x14ac:dyDescent="0.45">
+      <c r="AC44" s="11"/>
+    </row>
+    <row r="45" spans="1:30" x14ac:dyDescent="0.45">
       <c r="A45" s="11" t="s">
         <v>406</v>
       </c>
@@ -7314,21 +7498,23 @@
         <v>-10000</v>
       </c>
       <c r="I45" s="11">
+        <v>-30000</v>
+      </c>
+      <c r="J45" s="11">
         <v>-50000</v>
       </c>
-      <c r="J45" s="11">
+      <c r="K45" s="11">
         <v>-100000</v>
       </c>
-      <c r="K45" s="11">
+      <c r="L45" s="11">
         <v>-200000</v>
       </c>
-      <c r="L45" s="11">
+      <c r="M45" s="11">
         <v>-500000</v>
       </c>
-      <c r="M45" s="11">
+      <c r="N45" s="11">
         <v>-1000000</v>
       </c>
-      <c r="O45" s="11"/>
       <c r="P45" s="11"/>
       <c r="Q45" s="11"/>
       <c r="R45" s="11"/>
@@ -7342,8 +7528,9 @@
       <c r="Z45" s="11"/>
       <c r="AA45" s="11"/>
       <c r="AB45" s="11"/>
-    </row>
-    <row r="46" spans="1:29" x14ac:dyDescent="0.45">
+      <c r="AC45" s="11"/>
+    </row>
+    <row r="46" spans="1:30" x14ac:dyDescent="0.45">
       <c r="A46" s="11" t="s">
         <v>406</v>
       </c>
@@ -7369,21 +7556,23 @@
         <v>-10000</v>
       </c>
       <c r="I46" s="11">
+        <v>-30000</v>
+      </c>
+      <c r="J46" s="11">
         <v>-50000</v>
       </c>
-      <c r="J46" s="11">
+      <c r="K46" s="11">
         <v>-100000</v>
       </c>
-      <c r="K46" s="11">
+      <c r="L46" s="11">
         <v>-200000</v>
       </c>
-      <c r="L46" s="11">
+      <c r="M46" s="11">
         <v>-500000</v>
       </c>
-      <c r="M46" s="11">
+      <c r="N46" s="11">
         <v>-1000000</v>
       </c>
-      <c r="O46" s="11"/>
       <c r="P46" s="11"/>
       <c r="Q46" s="11"/>
       <c r="R46" s="11"/>
@@ -7397,42 +7586,43 @@
       <c r="Z46" s="11"/>
       <c r="AA46" s="11"/>
       <c r="AB46" s="11"/>
-    </row>
-    <row r="47" spans="1:29" x14ac:dyDescent="0.45">
+      <c r="AC46" s="11"/>
+    </row>
+    <row r="47" spans="1:30" x14ac:dyDescent="0.45">
       <c r="E47" s="11"/>
       <c r="G47" s="11"/>
       <c r="H47" s="11"/>
-      <c r="I47" s="11"/>
-      <c r="K47" s="11"/>
+      <c r="J47" s="11"/>
       <c r="L47" s="11"/>
       <c r="M47" s="11"/>
-    </row>
-    <row r="48" spans="1:29" x14ac:dyDescent="0.45">
+      <c r="N47" s="11"/>
+    </row>
+    <row r="48" spans="1:30" x14ac:dyDescent="0.45">
       <c r="E48" s="11"/>
       <c r="G48" s="11"/>
       <c r="H48" s="11"/>
-      <c r="I48" s="11"/>
-      <c r="K48" s="11"/>
+      <c r="J48" s="11"/>
       <c r="L48" s="11"/>
       <c r="M48" s="11"/>
-    </row>
-    <row r="49" spans="5:13" x14ac:dyDescent="0.45">
+      <c r="N48" s="11"/>
+    </row>
+    <row r="49" spans="5:14" x14ac:dyDescent="0.45">
       <c r="E49" s="11"/>
       <c r="G49" s="11"/>
       <c r="H49" s="11"/>
-      <c r="I49" s="11"/>
-      <c r="K49" s="11"/>
+      <c r="J49" s="11"/>
       <c r="L49" s="11"/>
       <c r="M49" s="11"/>
-    </row>
-    <row r="51" spans="5:13" x14ac:dyDescent="0.45">
+      <c r="N49" s="11"/>
+    </row>
+    <row r="51" spans="5:14" x14ac:dyDescent="0.45">
       <c r="E51" s="11"/>
       <c r="G51" s="11"/>
       <c r="H51" s="11"/>
-      <c r="I51" s="11"/>
-      <c r="K51" s="11"/>
+      <c r="J51" s="11"/>
       <c r="L51" s="11"/>
       <c r="M51" s="11"/>
+      <c r="N51" s="11"/>
     </row>
   </sheetData>
   <phoneticPr fontId="7" type="noConversion"/>
@@ -7462,7 +7652,7 @@
         <v>264</v>
       </c>
       <c r="B2" s="17">
-        <v>-5</v>
+        <v>-2.7777777777777781</v>
       </c>
       <c r="C2" s="17"/>
       <c r="D2" s="17"/>
@@ -7504,7 +7694,7 @@
         <v>265</v>
       </c>
       <c r="B3" s="17">
-        <v>-51</v>
+        <v>-28.333333333333332</v>
       </c>
       <c r="C3" s="17"/>
       <c r="D3" s="17"/>
@@ -7541,7 +7731,7 @@
         <v>266</v>
       </c>
       <c r="B4" s="17">
-        <v>-512</v>
+        <v>-284.44444444444446</v>
       </c>
       <c r="C4" s="17"/>
       <c r="D4" s="17"/>
@@ -7583,7 +7773,7 @@
         <v>267</v>
       </c>
       <c r="B5" s="17">
-        <v>-5114</v>
+        <v>-2841.1111111111113</v>
       </c>
       <c r="C5" s="17"/>
       <c r="D5" s="17"/>
@@ -7620,7 +7810,7 @@
         <v>125</v>
       </c>
       <c r="B6" s="17">
-        <v>-50376</v>
+        <v>-27986.666666666668</v>
       </c>
       <c r="C6" s="17"/>
       <c r="D6" s="17"/>
@@ -7662,7 +7852,7 @@
         <v>268</v>
       </c>
       <c r="B7" s="17">
-        <v>-6</v>
+        <v>-3.3333333333333335</v>
       </c>
       <c r="C7" s="17"/>
       <c r="D7" s="17"/>
@@ -7704,7 +7894,7 @@
         <v>269</v>
       </c>
       <c r="B8" s="17">
-        <v>-53</v>
+        <v>-29.444444444444443</v>
       </c>
       <c r="C8" s="17"/>
       <c r="D8" s="17"/>
@@ -7741,7 +7931,7 @@
         <v>270</v>
       </c>
       <c r="B9" s="17">
-        <v>-514</v>
+        <v>-285.55555555555554</v>
       </c>
       <c r="C9" s="17"/>
       <c r="D9" s="17"/>
@@ -7783,7 +7973,7 @@
         <v>271</v>
       </c>
       <c r="B10" s="17">
-        <v>-5116</v>
+        <v>-2842.2222222222217</v>
       </c>
       <c r="C10" s="17"/>
       <c r="D10" s="17"/>
@@ -7820,7 +8010,7 @@
         <v>126</v>
       </c>
       <c r="B11" s="17">
-        <v>-50367</v>
+        <v>-27981.666666666668</v>
       </c>
       <c r="C11" s="17"/>
       <c r="D11" s="17"/>
@@ -7862,7 +8052,7 @@
         <v>272</v>
       </c>
       <c r="B12" s="17">
-        <v>-9</v>
+        <v>-5</v>
       </c>
       <c r="C12" s="17"/>
       <c r="D12" s="17"/>
@@ -7876,7 +8066,7 @@
         <v>273</v>
       </c>
       <c r="B13" s="17">
-        <v>-62</v>
+        <v>-34.444444444444443</v>
       </c>
       <c r="C13" s="17"/>
       <c r="D13" s="17"/>
@@ -7890,7 +8080,7 @@
         <v>274</v>
       </c>
       <c r="B14" s="17">
-        <v>-529</v>
+        <v>-293.88888888888886</v>
       </c>
       <c r="C14" s="17"/>
       <c r="D14" s="17"/>
@@ -7904,7 +8094,7 @@
         <v>275</v>
       </c>
       <c r="B15" s="17">
-        <v>-5132</v>
+        <v>-2851.1111111111113</v>
       </c>
       <c r="C15" s="17"/>
       <c r="D15" s="17"/>
@@ -7918,7 +8108,7 @@
         <v>276</v>
       </c>
       <c r="B16" s="17">
-        <v>-50257</v>
+        <v>-27920.555555555558</v>
       </c>
       <c r="C16" s="17"/>
       <c r="D16" s="17"/>
@@ -7932,7 +8122,7 @@
         <v>291</v>
       </c>
       <c r="B17" s="17">
-        <v>-16</v>
+        <v>-8.8888888888888893</v>
       </c>
       <c r="C17" s="17"/>
       <c r="D17" s="17"/>
@@ -7946,7 +8136,7 @@
         <v>292</v>
       </c>
       <c r="B18" s="17">
-        <v>-88</v>
+        <v>-48.888888888888886</v>
       </c>
       <c r="C18" s="17"/>
       <c r="D18" s="17"/>
@@ -7960,7 +8150,7 @@
         <v>293</v>
       </c>
       <c r="B19" s="17">
-        <v>-616</v>
+        <v>-342.22222222222229</v>
       </c>
       <c r="C19" s="17"/>
       <c r="D19" s="17"/>
@@ -7974,7 +8164,7 @@
         <v>294</v>
       </c>
       <c r="B20" s="17">
-        <v>-5283</v>
+        <v>-2935</v>
       </c>
       <c r="C20" s="17"/>
       <c r="D20" s="17"/>
@@ -7988,7 +8178,7 @@
         <v>295</v>
       </c>
       <c r="B21" s="17">
-        <v>-46061</v>
+        <v>-25589.444444444442</v>
       </c>
       <c r="C21" s="17"/>
       <c r="D21" s="17"/>
@@ -8002,7 +8192,7 @@
         <v>240</v>
       </c>
       <c r="B22" s="17">
-        <v>-41</v>
+        <v>-22.777777777777775</v>
       </c>
       <c r="C22" s="17"/>
       <c r="D22" s="17"/>
@@ -8016,7 +8206,7 @@
         <v>241</v>
       </c>
       <c r="B23" s="17">
-        <v>-156</v>
+        <v>-86.666666666666671</v>
       </c>
       <c r="C23" s="17"/>
       <c r="D23" s="17"/>
@@ -8030,7 +8220,7 @@
         <v>242</v>
       </c>
       <c r="B24" s="17">
-        <v>-877</v>
+        <v>-487.22222222222229</v>
       </c>
       <c r="C24" s="17"/>
       <c r="D24" s="17"/>
@@ -8044,7 +8234,7 @@
         <v>243</v>
       </c>
       <c r="B25" s="17">
-        <v>-6156</v>
+        <v>-3420</v>
       </c>
       <c r="C25" s="17"/>
       <c r="D25" s="17"/>
@@ -8058,7 +8248,7 @@
         <v>244</v>
       </c>
       <c r="B26" s="17">
-        <v>-47658</v>
+        <v>-26476.666666666668</v>
       </c>
       <c r="C26" s="17"/>
       <c r="D26" s="17"/>
@@ -8072,7 +8262,7 @@
         <v>296</v>
       </c>
       <c r="B27" s="17">
-        <v>-179</v>
+        <v>-99.444444444444429</v>
       </c>
       <c r="C27" s="17"/>
       <c r="D27" s="17"/>
@@ -8086,7 +8276,7 @@
         <v>297</v>
       </c>
       <c r="B28" s="17">
-        <v>-413</v>
+        <v>-229.44444444444446</v>
       </c>
       <c r="C28" s="17"/>
       <c r="D28" s="17"/>
@@ -8100,7 +8290,7 @@
         <v>298</v>
       </c>
       <c r="B29" s="17">
-        <v>-1562</v>
+        <v>-867.77777777777783</v>
       </c>
       <c r="C29" s="17"/>
       <c r="D29" s="17"/>
@@ -8114,7 +8304,7 @@
         <v>299</v>
       </c>
       <c r="B30" s="17">
-        <v>-8763</v>
+        <v>-4868.333333333333</v>
       </c>
       <c r="C30" s="17"/>
       <c r="D30" s="17"/>
@@ -8128,7 +8318,7 @@
         <v>300</v>
       </c>
       <c r="B31" s="17">
-        <v>-60612</v>
+        <v>-33673.333333333336</v>
       </c>
       <c r="C31" s="17"/>
       <c r="D31" s="17"/>
@@ -8142,7 +8332,7 @@
         <v>245</v>
       </c>
       <c r="B32" s="17">
-        <v>-631</v>
+        <v>-350.5555555555556</v>
       </c>
       <c r="C32" s="17"/>
       <c r="D32" s="17"/>
@@ -8156,7 +8346,7 @@
         <v>246</v>
       </c>
       <c r="B33" s="17">
-        <v>-1733</v>
+        <v>-962.77777777777783</v>
       </c>
       <c r="C33" s="17"/>
       <c r="D33" s="17"/>
@@ -8170,7 +8360,7 @@
         <v>247</v>
       </c>
       <c r="B34" s="17">
-        <v>-4045</v>
+        <v>-2247.2222222222222</v>
       </c>
       <c r="C34" s="17"/>
       <c r="D34" s="17"/>
@@ -8184,7 +8374,7 @@
         <v>248</v>
       </c>
       <c r="B35" s="17">
-        <v>-15449</v>
+        <v>-8582.7777777777774</v>
       </c>
       <c r="C35" s="17"/>
       <c r="D35" s="17"/>
@@ -8198,7 +8388,7 @@
         <v>249</v>
       </c>
       <c r="B36" s="17">
-        <v>-86973</v>
+        <v>-48318.333333333336</v>
       </c>
       <c r="C36" s="17"/>
       <c r="D36" s="17"/>

</xml_diff>

<commit_message>
Modified setup file for response time pumping rates
</commit_message>
<xml_diff>
--- a/setup.xlsx
+++ b/setup.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cmarinriver\Projects\ConfinedLab\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B641C5A-12B4-4CA8-9971-CE19F5130DC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F928BB2A-1145-4D23-9B85-DDBC27CD0ABA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15796" firstSheet="2" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15796" firstSheet="2" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="grid" sheetId="1" r:id="rId1"/>
@@ -7652,7 +7652,7 @@
         <v>264</v>
       </c>
       <c r="B2" s="17">
-        <v>-2.7777777777777781</v>
+        <v>-3</v>
       </c>
       <c r="C2" s="17"/>
       <c r="D2" s="17"/>
@@ -7694,7 +7694,7 @@
         <v>265</v>
       </c>
       <c r="B3" s="17">
-        <v>-28.333333333333332</v>
+        <v>-28</v>
       </c>
       <c r="C3" s="17"/>
       <c r="D3" s="17"/>
@@ -7731,7 +7731,7 @@
         <v>266</v>
       </c>
       <c r="B4" s="17">
-        <v>-284.44444444444446</v>
+        <v>-284</v>
       </c>
       <c r="C4" s="17"/>
       <c r="D4" s="17"/>
@@ -7773,7 +7773,7 @@
         <v>267</v>
       </c>
       <c r="B5" s="17">
-        <v>-2841.1111111111113</v>
+        <v>-2841</v>
       </c>
       <c r="C5" s="17"/>
       <c r="D5" s="17"/>
@@ -7810,7 +7810,7 @@
         <v>125</v>
       </c>
       <c r="B6" s="17">
-        <v>-27986.666666666668</v>
+        <v>-27987</v>
       </c>
       <c r="C6" s="17"/>
       <c r="D6" s="17"/>
@@ -7852,7 +7852,7 @@
         <v>268</v>
       </c>
       <c r="B7" s="17">
-        <v>-3.3333333333333335</v>
+        <v>-3</v>
       </c>
       <c r="C7" s="17"/>
       <c r="D7" s="17"/>
@@ -7894,7 +7894,7 @@
         <v>269</v>
       </c>
       <c r="B8" s="17">
-        <v>-29.444444444444443</v>
+        <v>-29</v>
       </c>
       <c r="C8" s="17"/>
       <c r="D8" s="17"/>
@@ -7931,7 +7931,7 @@
         <v>270</v>
       </c>
       <c r="B9" s="17">
-        <v>-285.55555555555554</v>
+        <v>-286</v>
       </c>
       <c r="C9" s="17"/>
       <c r="D9" s="17"/>
@@ -7973,7 +7973,7 @@
         <v>271</v>
       </c>
       <c r="B10" s="17">
-        <v>-2842.2222222222217</v>
+        <v>-2842</v>
       </c>
       <c r="C10" s="17"/>
       <c r="D10" s="17"/>
@@ -8010,7 +8010,7 @@
         <v>126</v>
       </c>
       <c r="B11" s="17">
-        <v>-27981.666666666668</v>
+        <v>-27982</v>
       </c>
       <c r="C11" s="17"/>
       <c r="D11" s="17"/>
@@ -8066,7 +8066,7 @@
         <v>273</v>
       </c>
       <c r="B13" s="17">
-        <v>-34.444444444444443</v>
+        <v>-34</v>
       </c>
       <c r="C13" s="17"/>
       <c r="D13" s="17"/>
@@ -8080,7 +8080,7 @@
         <v>274</v>
       </c>
       <c r="B14" s="17">
-        <v>-293.88888888888886</v>
+        <v>-294</v>
       </c>
       <c r="C14" s="17"/>
       <c r="D14" s="17"/>
@@ -8094,7 +8094,7 @@
         <v>275</v>
       </c>
       <c r="B15" s="17">
-        <v>-2851.1111111111113</v>
+        <v>-2851</v>
       </c>
       <c r="C15" s="17"/>
       <c r="D15" s="17"/>
@@ -8108,7 +8108,7 @@
         <v>276</v>
       </c>
       <c r="B16" s="17">
-        <v>-27920.555555555558</v>
+        <v>-27921</v>
       </c>
       <c r="C16" s="17"/>
       <c r="D16" s="17"/>
@@ -8122,7 +8122,7 @@
         <v>291</v>
       </c>
       <c r="B17" s="17">
-        <v>-8.8888888888888893</v>
+        <v>-9</v>
       </c>
       <c r="C17" s="17"/>
       <c r="D17" s="17"/>
@@ -8136,7 +8136,7 @@
         <v>292</v>
       </c>
       <c r="B18" s="17">
-        <v>-48.888888888888886</v>
+        <v>-49</v>
       </c>
       <c r="C18" s="17"/>
       <c r="D18" s="17"/>
@@ -8150,7 +8150,7 @@
         <v>293</v>
       </c>
       <c r="B19" s="17">
-        <v>-342.22222222222229</v>
+        <v>-342</v>
       </c>
       <c r="C19" s="17"/>
       <c r="D19" s="17"/>
@@ -8178,7 +8178,7 @@
         <v>295</v>
       </c>
       <c r="B21" s="17">
-        <v>-25589.444444444442</v>
+        <v>-25589</v>
       </c>
       <c r="C21" s="17"/>
       <c r="D21" s="17"/>
@@ -8192,7 +8192,7 @@
         <v>240</v>
       </c>
       <c r="B22" s="17">
-        <v>-22.777777777777775</v>
+        <v>-23</v>
       </c>
       <c r="C22" s="17"/>
       <c r="D22" s="17"/>
@@ -8206,7 +8206,7 @@
         <v>241</v>
       </c>
       <c r="B23" s="17">
-        <v>-86.666666666666671</v>
+        <v>-87</v>
       </c>
       <c r="C23" s="17"/>
       <c r="D23" s="17"/>
@@ -8220,7 +8220,7 @@
         <v>242</v>
       </c>
       <c r="B24" s="17">
-        <v>-487.22222222222229</v>
+        <v>-487</v>
       </c>
       <c r="C24" s="17"/>
       <c r="D24" s="17"/>
@@ -8248,7 +8248,7 @@
         <v>244</v>
       </c>
       <c r="B26" s="17">
-        <v>-26476.666666666668</v>
+        <v>-26477</v>
       </c>
       <c r="C26" s="17"/>
       <c r="D26" s="17"/>
@@ -8262,7 +8262,7 @@
         <v>296</v>
       </c>
       <c r="B27" s="17">
-        <v>-99.444444444444429</v>
+        <v>-99</v>
       </c>
       <c r="C27" s="17"/>
       <c r="D27" s="17"/>
@@ -8276,7 +8276,7 @@
         <v>297</v>
       </c>
       <c r="B28" s="17">
-        <v>-229.44444444444446</v>
+        <v>-229</v>
       </c>
       <c r="C28" s="17"/>
       <c r="D28" s="17"/>
@@ -8290,7 +8290,7 @@
         <v>298</v>
       </c>
       <c r="B29" s="17">
-        <v>-867.77777777777783</v>
+        <v>-868</v>
       </c>
       <c r="C29" s="17"/>
       <c r="D29" s="17"/>
@@ -8304,7 +8304,7 @@
         <v>299</v>
       </c>
       <c r="B30" s="17">
-        <v>-4868.333333333333</v>
+        <v>-4868</v>
       </c>
       <c r="C30" s="17"/>
       <c r="D30" s="17"/>
@@ -8318,7 +8318,7 @@
         <v>300</v>
       </c>
       <c r="B31" s="17">
-        <v>-33673.333333333336</v>
+        <v>-33673</v>
       </c>
       <c r="C31" s="17"/>
       <c r="D31" s="17"/>
@@ -8332,7 +8332,7 @@
         <v>245</v>
       </c>
       <c r="B32" s="17">
-        <v>-350.5555555555556</v>
+        <v>-351</v>
       </c>
       <c r="C32" s="17"/>
       <c r="D32" s="17"/>
@@ -8346,7 +8346,7 @@
         <v>246</v>
       </c>
       <c r="B33" s="17">
-        <v>-962.77777777777783</v>
+        <v>-963</v>
       </c>
       <c r="C33" s="17"/>
       <c r="D33" s="17"/>
@@ -8360,7 +8360,7 @@
         <v>247</v>
       </c>
       <c r="B34" s="17">
-        <v>-2247.2222222222222</v>
+        <v>-2247</v>
       </c>
       <c r="C34" s="17"/>
       <c r="D34" s="17"/>
@@ -8374,7 +8374,7 @@
         <v>248</v>
       </c>
       <c r="B35" s="17">
-        <v>-8582.7777777777774</v>
+        <v>-8583</v>
       </c>
       <c r="C35" s="17"/>
       <c r="D35" s="17"/>
@@ -8388,7 +8388,7 @@
         <v>249</v>
       </c>
       <c r="B36" s="17">
-        <v>-48318.333333333336</v>
+        <v>-48318</v>
       </c>
       <c r="C36" s="17"/>
       <c r="D36" s="17"/>

</xml_diff>